<commit_message>
chore(editais): atualizacao automatica 2026-09-09 11:57
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N18"/>
+  <dimension ref="A1:N19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1013,51 +1013,130 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Extensão</t>
+          <t>Difusão do Conhecimento</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>EDITAL FAPES Nº 01/2026 – TCC EMPREENDEDOR INOVADOR</t>
+          <t>EDITAL FAPES Nº 28/2025 - PUBLICAÇÃO DE ARTIGOS TÉCNICO-CIENTÍFICOS</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Sem alteracoes</t>
+          <t>Removido (nao mais aberto)</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02 a 2026-10-27: Período de submissão das propostas (Segunda Chamada) (Até 17h59)</t>
+          <t>2026-09-06 a 2026-10-26: Submissão de propostas (4ª Chamada, até as 17h59)</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr"/>
       <c r="F9" s="2" t="inlineStr">
         <is>
+          <t>O objetivo geral deste edital é incentivar a publicação científica e tecnológica no Espírito Santo por meio da concessão de auxílio financeiro para publicação de artigos técnico-científicos que apresentem resultados de pesquisa desenvolvidas em Instituições de Ensino e/ou Pesquisa no estado. A chamada pública visa selecionar propostas para concessão de auxílio financeiro para tal finalidade, valorizando a produção técnico-científica e ampliando a visibilidade das atividades de pesquisa e inovação.</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisador ou aluno em atividade de pesquisa ou desenvolvimento inovador em Instituição de Ensino e/ou Pesquisa (IES/P) localizada no estado do Espírito Santo.</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>R$ 800.000,00</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>US$ 1.500,00</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>editais.duvidas@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-22 a 2026-02-25: Submissão de propostas (1ª Chamada, até as 17h59)
+2026-02-17: Prazo para impugnação do edital (Até 5 dias úteis antes do encerramento do prazo de submissão da primeira chamada)
+?: Interposição de recursos (1ª Chamada, 5 dias úteis após a publicação do resultado preliminar)
+2026-03-19 a 2026-05-25: Submissão de propostas (2ª Chamada, até as 17h59)
+?: Interposição de recursos (2ª Chamada, 5 dias úteis após a publicação do resultado preliminar)
+2026-06-19 a 2026-08-25: Submissão de propostas (3ª Chamada, até as 17h59)
+?: Interposição de recursos (3ª Chamada, 5 dias úteis após a publicação do resultado preliminar)
+2026-09-06 a 2026-10-26: Submissão de propostas (4ª Chamada, até as 17h59)
+?: Interposição de recursos (4ª Chamada, 5 dias úteis após a publicação do resultado preliminar)
+?: Contratação das propostas aprovadas (Até 30 dias após a publicação do resultado final homologado de cada chamada)
+?: Informar dados bancários (Até 30 dias após a assinatura e publicação do Termo de Outorga de cada projeto)
+?: Prestação de contas (Até 30 dias após o término de vigência do Termo de Outorga (prazo máximo de execução do projeto é de 12 meses))</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>O artigo deve ter sido aceito em periódico classificado entre A1 e A4 no Qualis-Capes (2021-2024) ou com percentil igual ou superior a 50% nas plataformas Scopus ou ISI Web of Science. O proponente poderá ser contratado para no máximo 2 propostas, desde que submetidas em chamadas distintas. Cada coordenador pode apresentar apenas uma proposta por chamada; caso envie mais de uma, apenas a última será considerada. O prazo máximo para execução de cada projeto é de 12 meses.</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_28_2025_Publicação_de_Artigos_Técnico-Científicos.pdf</t>
+        </is>
+      </c>
+      <c r="N9" s="2" t="inlineStr">
+        <is>
+          <t>difusao_do_conhecimento/EDITAL_FAPES_No_28_2025_-_PUBLICAÇÃO_DE_ARTIGOS_TÉCNICO-CIENTÍFICOS.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Extensão</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>EDITAL FAPES Nº 01/2026 – TCC EMPREENDEDOR INOVADOR</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02 a 2026-10-27: Período de submissão das propostas (Segunda Chamada) (Até 17h59)</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
           <t>Incentivar o desenvolvimento de Trabalhos de Conclusão de Curso (TCCs) com foco em inovação, empreendedorismo e aplicabilidade prática. O edital visa a concessão de Bolsas de Apoio a Trabalho de Conclusão de Curso (BTCC) para a execução de TCCs que apresentem soluções inovadoras e empreendedoras. As propostas devem ter fundamentação teórico-metodológica consistente, voltadas para aplicação prática e impacto econômico, social e/ou ambiental no Estado do Espírito Santo, alinhados aos ODS da ONU e ao Plano ES 500 Anos.</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>Professores orientadores com vínculo estatutário ou celetista por tempo indeterminado com Instituição de Ensino Superior (IES) reconhecida pelo Ministério da Educação (MEC), localizada no Espírito Santo, que submetam entre 3 (três) e 5 (cinco) propostas.</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>R$ 1.600.000,00</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>R$ 11.000,00</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr">
+      <c r="J10" s="2" t="inlineStr">
         <is>
           <t>editais.extensao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K9" s="2" t="inlineStr">
+      <c r="K10" s="2" t="inlineStr">
         <is>
           <t>?: Impugnação do Edital (Até 5 (cinco) dias úteis antes do encerramento do prazo de submissão das propostas de cada chamada.)
 2026-02-02 a 2026-03-30: Período de submissão das propostas (Primeira Chamada) (Até 17h59)
@@ -1074,66 +1153,66 @@
 ?: Prazo para solicitação de ofício para abertura de conta (Até 3 (três) dias úteis para o Outorgado.)</t>
         </is>
       </c>
-      <c r="L9" s="2" t="inlineStr">
+      <c r="L10" s="2" t="inlineStr">
         <is>
           <t>O prazo de execução dos projetos será de um semestre letivo, acrescido de até 3 (três) meses apenas para apresentação da Declaração ou Ata de Defesa do TCC. Cada projeto de TCC deve demonstrar potencial de geração de valor, criação de negócios ou produtos inovadores; estar alinhado aos ODS da ONU (especialmente ODS 4, 8, 9, 10 e 17) e ao Plano ES 500 Anos, e ser desenvolvido em consonância com os Projetos Pedagógicos dos respectivos cursos de graduação. As propostas concorrerão com as demais de suas respectivas microrregiões, sendo apoiados, na primeira chamada, no máximo 20 (vinte) projetos de TCC por microrregião e, na segunda e terceira chamadas, até 10 (dez) projetos de TCC por microrregião. Recursos remanescentes serão destinados a projetos em ampla concorrência por ordem decrescente de nota. Propostas submetidas a mais de uma microrregião serão desclassificadas. Cada proposta deverá vincular um único aluno sob orientação do proponente. O proponente que indicar alunos orientados vinculados a outra IES deverá apresentar declaração de autorização tanto da sua IES de vínculo quanto da IES à qual os alunos orientados estão vinculados. Propostas com Nota Final (NF) inferior a 70 (setenta) pontos serão desclassificadas. Não será permitido o acúmulo de bolsas Fapes pelo aluno orientado, exceto com bolsas do Programa Nossa Bolsa, do Programa Universidade para Todos (Prouni) e com Bolsas de Extensão (Ext-E e Ext-F) da Fapes.</t>
         </is>
       </c>
-      <c r="M9" s="2" t="inlineStr">
+      <c r="M10" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_Nº_01.2026_TCC_EMPREENDEDOR_INOVADOR-2.pdf</t>
         </is>
       </c>
-      <c r="N9" s="2" t="inlineStr">
+      <c r="N10" s="2" t="inlineStr">
         <is>
           <t>extensao/EDITAL_FAPES_No_01_2026_–_TCC_EMPREENDEDOR_INOVADOR.pdf</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 08/2026 - NOVA ECONOMIA CAPIXABA 2026</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="2" t="inlineStr"/>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr"/>
+      <c r="E11" s="2" t="inlineStr"/>
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>Promover o aumento da competitividade dos setores econômicos capixabas por meio de projetos de inovação, desenvolvidos por empresas (incluindo cooperativas de trabalho) em colaboração com Instituições de Ciência e Tecnologia (ICT) ou Instituições de Ensino Superior (IES) capixabas. O apoio se dará por meio de um modelo de coinvestimento tripartite (FAPES, empresa/cooperativa, ICT/IES), com projetos alinhados ao Plano ES 500 Anos e ao Plano Estadual de Ciência, Tecnologia e Inovação do Espírito Santo (PCTI-ES).</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>Empresas com sede administrativa ou filial no Espírito Santo, individualmente ou em associação com outras empresas ou cooperativas de trabalho capixabas.</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>R$ 40.000.000,00</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>R$ 500.000,00 a R$ 3.000.000,00</t>
         </is>
       </c>
-      <c r="J10" s="2" t="inlineStr">
+      <c r="J11" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K10" s="2" t="inlineStr">
+      <c r="K11" s="2" t="inlineStr">
         <is>
           <t>2026-03-30: Submissão das propostas no SIGFAPES (Fluxo contínuo)
 ?: Prazo de submissão dos recursos administrativos (Habilitação) (5 dias úteis a partir da publicação do resultado preliminar da habilitação.)
@@ -1142,70 +1221,70 @@
 ?: Submissão das documentações para contratação (Até 30 dias a partir da publicação do resultado homologado do julgamento de mérito.)</t>
         </is>
       </c>
-      <c r="L10" s="2" t="inlineStr">
+      <c r="L11" s="2" t="inlineStr">
         <is>
           <t>O prazo de execução do projeto é de 24 meses, com possibilidade de prorrogação por até 12 meses. As empresas proponentes e coexecutoras devem ter receita bruta operacional superior a R$ 360.000,00 nos dois últimos exercícios fiscais; cooperativas de trabalho devem apresentar Demonstração de Sobras ou Perdas (DSP). As empresas devem estar ativas há pelo menos 6 meses e não podem ter sido contratadas em editais FAPES nº 07/2024, nº 10/2025 e nº 06/2026, a menos que o projeto, coordenador e equipe executora sejam distintos. É permitida apenas uma proposta por empresa. Em caso de inabilitação ou desclassificação, a empresa poderá realizar uma nova submissão, exceto se reprovada pelo Comitê de Conformidade, o que impede nova submissão nesta chamada. A aprovação da proposta não garante a contratação, que está sujeita à disponibilidade financeira da FAPES, ordem de submissão e visita técnica. O critério de desempate é a data de submissão da proposta no SIGFAPES. Propostas com Nota Final inferior a 80 pontos ou notas individuais inferiores a 4 em critérios específicos serão desclassificadas. A impugnação dos termos do edital deve ser feita em até 5 dias úteis antes do encerramento do prazo de submissão das propostas do primeiro ciclo (considerando o fluxo contínuo, esta observação se refere a um prazo inicial para impugnação do edital em si).</t>
         </is>
       </c>
-      <c r="M10" s="2" t="inlineStr">
+      <c r="M11" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_08-2026_-_Nova_Economia_Capixaba_-_2_Edição_-_Lançamento.pdf</t>
         </is>
       </c>
-      <c r="N10" s="2" t="inlineStr">
+      <c r="N11" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_No_08_2026_-_NOVA_ECONOMIA_CAPIXABA_2026.pdf</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES N° 23/2026 - APOIO ÀS INCUBADORAS DO ESPÍRITO SANTO</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>2026-09-17: Prazo para impugnação do edital (Até 5 dias úteis anteriores ao encerramento do prazo de envio das propostas. O pedido deve ser enviado no E-Flow por meio do Formulário de Impugnação de Edital.)</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr"/>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="E12" s="2" t="inlineStr"/>
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>O edital visa apoiar incubadoras públicas ou privadas sem fins lucrativos, localizadas no Espírito Santo, que buscam estimular e prestar apoio logístico, gerencial e/ou tecnológico a empreendedores e empresas com produtos, serviços ou modelos de negócio inovadores. Este apoio busca ampliar, aperfeiçoar e consolidar as atividades de pré-incubação, incubação e pós-incubação, promovendo a capacitação de novos empreendedores e o desenvolvimento socioeconômico do estado.</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>Incubadoras, sem fins lucrativos, sediadas no Espírito Santo, que atendam aos requisitos do edital.</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="H12" s="2" t="inlineStr">
         <is>
           <t>R$ 4.500.000,00</t>
         </is>
       </c>
-      <c r="I11" s="2" t="inlineStr">
+      <c r="I12" s="2" t="inlineStr">
         <is>
           <t>R$ 252.000,00</t>
         </is>
       </c>
-      <c r="J11" s="2" t="inlineStr">
+      <c r="J12" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K11" s="2" t="inlineStr">
+      <c r="K12" s="2" t="inlineStr">
         <is>
           <t>2026-09-17: Prazo para impugnação do edital (Até 5 dias úteis anteriores ao encerramento do prazo de envio das propostas. O pedido deve ser enviado no E-Flow por meio do Formulário de Impugnação de Edital.)
 2026-08-25 a 2026-09-24: Envio da proposta e documentos (Até as 17h59, via SigFapes)
@@ -1213,83 +1292,19 @@
 2026-11-04: Contratação dos projetos selecionados (A partir desta data)</t>
         </is>
       </c>
-      <c r="L11" s="2" t="inlineStr">
+      <c r="L12" s="2" t="inlineStr">
         <is>
           <t>O projeto terá prazo de vigência de 24 meses, sem prorrogação. Os recursos financeiros remanescentes, caso o número de propostas previstas para contratação nos níveis de maturidade I, II ou III não seja alcançado, serão redirecionados para propostas suplentes. Os recursos destinados ao custeio (exceto bolsas) serão liberados em 2 parcelas. Caso a proposta seja enquadrada em nível de maturidade distinto do indicado pelo proponente, os valores financiáveis serão ajustados proporcionalmente. É obrigatório destinar no mínimo 20% do valor total solicitado para bolsas. As incubadoras beneficiárias devem destinar parte dos recursos de custeio à associação à Anprotec. Propostas com nota final inferior a 60 pontos serão desclassificadas. A classificação por nível de maturidade é a seguinte: Nível Avançado (86 a 100 pontos), Nível Intermediário (76 a 85 pontos), Nível Básico (60 a 75 pontos).</t>
         </is>
       </c>
-      <c r="M11" s="2" t="inlineStr">
+      <c r="M12" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_23-2026_Apoio%20a%20Incubadoras_(Versão%20Final).pdf</t>
         </is>
       </c>
-      <c r="N11" s="2" t="inlineStr">
+      <c r="N12" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_N°_23_2026_-_APOIO_ÀS_INCUBADORAS_DO_ESPÍRITO_SANTO.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>Chamadas Internacionais</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>CHAMADA CONFAP CDTI 2026</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-08: Submissão de propostas (Até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Os formulários devem ser preenchidos em língua inglesa.)</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr"/>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>Apoiar projetos colaborativos de pesquisa e inovação tecnológica entre o Brasil e a Espanha, abrangendo qualquer setor de atividade. Destina-se a profissionais vinculados a universidades, centros de pesquisa ou empresas do Espírito Santo que desenvolvam atividades de P,D&amp;I e que apresentem propostas conjuntas com empresas espanholas.</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores principais ou coordenadores de projetos, brasileiros ou estrangeiros com visto permanente, residentes no Espírito Santo, com vínculo ativo a universidades, centros de pesquisa ou empresas localizadas no estado do Espírito Santo, que realizem atividades de pesquisa, desenvolvimento e inovação tecnológica e que integrem proposta conjunta com empresa espanhola.</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="n"/>
-      <c r="I12" s="2" t="inlineStr">
-        <is>
-          <t>€ 75.000,00</t>
-        </is>
-      </c>
-      <c r="J12" s="2" t="inlineStr">
-        <is>
-          <t>internacional.confap@gmail.com, brasil@cdti.es, carlos.quintana@cdti.es, global4@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K12" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-08: Submissão de propostas (Até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Os formulários devem ser preenchidos em língua inglesa.)</t>
-        </is>
-      </c>
-      <c r="L12" s="2" t="inlineStr">
-        <is>
-          <t>A FAPES apoiará um único projeto. Os projetos terão duração de 12 a 36 meses. O apoio financeiro da FAPES destina-se a despesas de capital e custeio, excluindo bolsas, conforme Resolução nº 309/2022. Cada proponente pode submeter apenas uma proposta. A submissão à FAPES (via SigFapes) para contratação ocorrerá somente após a aprovação da proposta pelo CDTI. Os projetos devem ter um orçamento total mínimo de € 250.000,00, e o apoio da FAPES deve corresponder a no mínimo 30% da contrapartida do valor total da proposta.</t>
-        </is>
-      </c>
-      <c r="M12" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes_Chamada%20Internacional_CDTI.2026.pdf</t>
-        </is>
-      </c>
-      <c r="N12" s="2" t="inlineStr">
-        <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_CDTI_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1301,7 +1316,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA CONFAP &amp; WBI - BÉLGICA 2026</t>
+          <t>CHAMADA CONFAP CDTI 2026</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -1311,53 +1326,49 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília), exclusivamente por meio da plataforma https://sistema.confap.org.br.)</t>
+          <t>2026-10-08: Submissão de propostas (Até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Os formulários devem ser preenchidos em língua inglesa.)</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Apoiar projetos conjuntos de Pesquisa e Inovação, promovendo o intercâmbio científico entre grupos de pesquisa do Espírito Santo e da região da Valônia-Bruxelas, na Bélgica, em áreas como inovação em saúde, energia sustentável, gestão ambiental e aeronáutica. Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas.</t>
+          <t>Apoiar projetos colaborativos de pesquisa e inovação tecnológica entre o Brasil e a Espanha, abrangendo qualquer setor de atividade. Destina-se a profissionais vinculados a universidades, centros de pesquisa ou empresas do Espírito Santo que desenvolvam atividades de P,D&amp;I e que apresentem propostas conjuntas com empresas espanholas.</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores brasileiros com doutorado, vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) localizadas no estado do Espírito Santo, residentes no estado, que atuem como pesquisador principal ou coordenador do projeto, e que participem de propostas conjuntas com pesquisadores da Valônia-Bruxelas, Bélgica.</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>R$ 300.000,00</t>
-        </is>
-      </c>
+          <t>Pesquisadores principais ou coordenadores de projetos, brasileiros ou estrangeiros com visto permanente, residentes no Espírito Santo, com vínculo ativo a universidades, centros de pesquisa ou empresas localizadas no estado do Espírito Santo, que realizem atividades de pesquisa, desenvolvimento e inovação tecnológica e que integrem proposta conjunta com empresa espanhola.</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="n"/>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>R$ 150.000,00</t>
+          <t>€ 75.000,00</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
+          <t>internacional.confap@gmail.com, brasil@cdti.es, carlos.quintana@cdti.es, global4@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília), exclusivamente por meio da plataforma https://sistema.confap.org.br.)</t>
+          <t>2026-10-08: Submissão de propostas (Até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Os formulários devem ser preenchidos em língua inglesa.)</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas. O prazo de vigência máximo para cada projeto é de 24 meses. O apoio financeiro da Fapes destina-se exclusivamente a despesas de mobilidade, excluindo bolsas. Cada proponente pode submeter apenas uma proposta; em caso de múltiplas submissões, apenas a última será considerada. As propostas devem ser submetidas utilizando o modelo do Anexo I (Application Form Template) em ambas as plataformas (CONFAP).</t>
+          <t>A FAPES apoiará um único projeto. Os projetos terão duração de 12 a 36 meses. O apoio financeiro da FAPES destina-se a despesas de capital e custeio, excluindo bolsas, conforme Resolução nº 309/2022. Cada proponente pode submeter apenas uma proposta. A submissão à FAPES (via SigFapes) para contratação ocorrerá somente após a aprovação da proposta pelo CDTI. Os projetos devem ter um orçamento total mínimo de € 250.000,00, e o apoio da FAPES deve corresponder a no mínimo 30% da contrapartida do valor total da proposta.</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20WBI%20-2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes_Chamada%20Internacional_CDTI.2026.pdf</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WBI_-_BÉLGICA_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_CDTI_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1369,7 +1380,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA CONFAP &amp; DAAD 2026</t>
+          <t>CHAMADA CONFAP &amp; WBI - BÉLGICA 2026</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1377,20 +1388,32 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr"/>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília), exclusivamente por meio da plataforma https://sistema.confap.org.br.)</t>
+        </is>
+      </c>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Apoiar a manutenção de bolsas de doutorado da FAPES para bolsistas que forem selecionados pelo Serviço Alemão de Intercâmbio Acadêmico (DAAD). O suporte visa permitir que esses bolsistas realizem suas pesquisas em instituições na Alemanha, no âmbito da Chamada DAAD 2026.</t>
+          <t>Apoiar projetos conjuntos de Pesquisa e Inovação, promovendo o intercâmbio científico entre grupos de pesquisa do Espírito Santo e da região da Valônia-Bruxelas, na Bélgica, em áreas como inovação em saúde, energia sustentável, gestão ambiental e aeronáutica. Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas.</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Bolsistas de doutorado da FAPES que forem selecionados pelo DAAD, que estejam adimplentes junto à FAPES e que não estejam no primeiro nem no último ano do doutorado.</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="n"/>
-      <c r="I14" s="2" t="n"/>
+          <t>Pesquisadores brasileiros com doutorado, vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) localizadas no estado do Espírito Santo, residentes no estado, que atuem como pesquisador principal ou coordenador do projeto, e que participem de propostas conjuntas com pesquisadores da Valônia-Bruxelas, Bélgica.</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>R$ 300.000,00</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>R$ 150.000,00</t>
+        </is>
+      </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
           <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
@@ -1398,22 +1421,22 @@
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>?: Submissão de propostas (As propostas deverão ser submetidas na Plataforma do DAAD, conforme item 3.1.)</t>
+          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília), exclusivamente por meio da plataforma https://sistema.confap.org.br.)</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>Este documento apresenta as diretrizes específicas da FAPES para a Chamada DAAD 2026, complementando o edital completo disponível no site do CONFAP.</t>
+          <t>Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas. O prazo de vigência máximo para cada projeto é de 24 meses. O apoio financeiro da Fapes destina-se exclusivamente a despesas de mobilidade, excluindo bolsas. Cada proponente pode submeter apenas uma proposta; em caso de múltiplas submissões, apenas a última será considerada. As propostas devem ser submetidas utilizando o modelo do Anexo I (Application Form Template) em ambas as plataformas (CONFAP).</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20-%20FAPES%202026-1.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20WBI%20-2026.pdf</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_DAAD_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WBI_-_BÉLGICA_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1425,7 +1448,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA MOBILITY CONFAP ITALY 2026</t>
+          <t>CHAMADA CONFAP &amp; DAAD 2026</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1437,39 +1460,39 @@
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>O edital MOBILITY CONFAP ITALY CALL 2026 visa apoiar pesquisadores do Brasil, vinculados a instituições de ensino superior e pesquisa brasileiras, que desejam desenvolver atividades de pesquisa na Itália em colaboração com colegas locais. O objetivo é facilitar e apoiar a colaboração científica, tecnológica e de inovação por meio da mobilidade de estudantes de doutorado, mestrado e pós-doutorado. O suporte é oferecido na forma de bolsas de estudo para fortalecer grupos de pesquisa brasileiros através de colaborações e visitas a grupos de pesquisa na Itália, parte da rede MCI.</t>
+          <t>Apoiar a manutenção de bolsas de doutorado da FAPES para bolsistas que forem selecionados pelo Serviço Alemão de Intercâmbio Acadêmico (DAAD). O suporte visa permitir que esses bolsistas realizem suas pesquisas em instituições na Alemanha, no âmbito da Chamada DAAD 2026.</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores de doutorado, mestrado e pós-doutorado vinculados a universidades e instituições de pesquisa nos Estados brasileiros participantes, que possuam um supervisor associado a uma universidade italiana parte da rede MCI.</t>
+          <t>Bolsistas de doutorado da FAPES que forem selecionados pelo DAAD, que estejam adimplentes junto à FAPES e que não estejam no primeiro nem no último ano do doutorado.</t>
         </is>
       </c>
       <c r="H15" s="2" t="n"/>
       <c r="I15" s="2" t="n"/>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com</t>
+          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04: Submissão de propostas (Até as 11:59 (horário de Brasília) via https://sistema.confap.org.br. Proponentes devem verificar com suas FAPs sobre submissão em plataformas próprias.)</t>
+          <t>?: Submissão de propostas (As propostas deverão ser submetidas na Plataforma do DAAD, conforme item 3.1.)</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>As FAPs participantes podem exigir critérios de elegibilidade adicionais e definir as modalidades de apoio, incluindo os valores das bolsas mensais, em suas próprias diretrizes ou orientações, devendo ser consultadas pelos candidatos antes da preparação da proposta. Não serão cobradas taxas de matrícula por nenhuma das partes para qualquer mobilidade de intercâmbio. Em caso de mobilidade no âmbito de projetos com potencial valor comercial e direitos de propriedade intelectual, as instituições anfitriãs e de envio deverão assinar um acordo de colaboração específico. As propostas devem incluir: projeto de pesquisa, Curriculum Vitae do candidato (Brasil), Curriculum Vitae do supervisor (Itália) e carta de apoio do supervisor na universidade italiana. As FAPs podem solicitar documentos adicionais. As vagas e oportunidades de pesquisa nas universidades italianas da rede MCI estão disponíveis em https://site.unibo.it/mobility-confap-italy/en/research-opportunity-offers-in-italy. Detalhes da rede MCI italiana em https://site.unibo.it/mobility-confap-italy/en/mci-program/network-of-italian-university. As FAPs associadas a esta chamada são: Alagoas - FAPEAL, Amazonas - FAPEAM, Bahia - FAPESB, Ceará - FUNCAP, Espírito Santo – FAPES, Goiás - FAPEG, Maranhão - FAPEMA, Pará - FAPESPA, Paraná - Fundação Araucária, Pernambuco – FACEPE, Rio Grande do Sul - FAPERGS, Santa Catarina - FAPESC. Outras FAPs podem confirmar sua participação.</t>
+          <t>Este documento apresenta as diretrizes específicas da FAPES para a Chamada DAAD 2026, complementando o edital completo disponível no site do CONFAP.</t>
         </is>
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-MCI-–-MOBILITY-CONFAP-ITALY-2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20-%20FAPES%202026-1.pdf</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_MOBILITY_CONFAP_ITALY_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_DAAD_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1481,7 +1504,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA ERC-CONFAP 2026</t>
+          <t>CHAMADA MOBILITY CONFAP ITALY 2026</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -1493,48 +1516,39 @@
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Apoiar a mobilidade de pesquisadores do estado do Espírito Santo para integrar equipes de pesquisa na Europa, em projetos financiados pelo Conselho Europeu de Pesquisa (ERC). O objetivo é possibilitar colaborações de pesquisa, promover oportunidades em equipes internacionais de excelência e fortalecer a internacionalização da ciência, tecnologia e inovação desenvolvida no Espírito Santo.</t>
+          <t>O edital MOBILITY CONFAP ITALY CALL 2026 visa apoiar pesquisadores do Brasil, vinculados a instituições de ensino superior e pesquisa brasileiras, que desejam desenvolver atividades de pesquisa na Itália em colaboração com colegas locais. O objetivo é facilitar e apoiar a colaboração científica, tecnológica e de inovação por meio da mobilidade de estudantes de doutorado, mestrado e pós-doutorado. O suporte é oferecido na forma de bolsas de estudo para fortalecer grupos de pesquisa brasileiros através de colaborações e visitas a grupos de pesquisa na Itália, parte da rede MCI.</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores ativos do Brasil, com título de doutor, que implementam atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros. Para FAPES, o proponente deve ser pesquisador principal ou coordenador do projeto, vinculado a IES/P no Espírito Santo, residente no estado, brasileiro ou estrangeiro com visto permanente, com currículo Lattes atualizado, adimplente com a FAPES e em regularidade perante as normas legais vigentes.</t>
-        </is>
-      </c>
-      <c r="H16" s="2" t="inlineStr">
-        <is>
-          <t>US$ 18.000,00</t>
-        </is>
-      </c>
-      <c r="I16" s="2" t="inlineStr">
-        <is>
-          <t>US$ 6.000,00</t>
-        </is>
-      </c>
+          <t>Pesquisadores de doutorado, mestrado e pós-doutorado vinculados a universidades e instituições de pesquisa nos Estados brasileiros participantes, que possuam um supervisor associado a uma universidade italiana parte da rede MCI.</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="n"/>
+      <c r="I16" s="2" t="n"/>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com, global@fapes.es.gov.br</t>
+          <t>internacional.confap@gmail.com</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>2026-08-10: Submissão de propostas (CONFAP) (Propostas completas, incluindo todos os documentos solicitados no Item 6 do edital geral, devem ser submetidas via portal https://sistema.confap.org.br/.)
-2026-08-10: Submissão de documentação para verificação de elegibilidade (FAPES) (Submeter via SigFapes a documentação exigida conforme Instrução de Serviços nº 082/2025 e Item 4, alínea B do edital específico da FAPES.)</t>
+          <t>2026-09-04: Submissão de propostas (Até as 11:59 (horário de Brasília) via https://sistema.confap.org.br. Proponentes devem verificar com suas FAPs sobre submissão em plataformas próprias.)</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>A FAPES apoiará até 3 projetos selecionados. Os recursos podem ser usados como auxílios individuais para estágios ou visitas técnicas de curta duração. O acesso à lista de projetos ERC é liberado após análise de elegibilidade básica pelo CONFAP. Os pesquisadores devem contatar os PIs dos projetos ERC para definir o Plano de Trabalho e condições.</t>
+          <t>As FAPs participantes podem exigir critérios de elegibilidade adicionais e definir as modalidades de apoio, incluindo os valores das bolsas mensais, em suas próprias diretrizes ou orientações, devendo ser consultadas pelos candidatos antes da preparação da proposta. Não serão cobradas taxas de matrícula por nenhuma das partes para qualquer mobilidade de intercâmbio. Em caso de mobilidade no âmbito de projetos com potencial valor comercial e direitos de propriedade intelectual, as instituições anfitriãs e de envio deverão assinar um acordo de colaboração específico. As propostas devem incluir: projeto de pesquisa, Curriculum Vitae do candidato (Brasil), Curriculum Vitae do supervisor (Itália) e carta de apoio do supervisor na universidade italiana. As FAPs podem solicitar documentos adicionais. As vagas e oportunidades de pesquisa nas universidades italianas da rede MCI estão disponíveis em https://site.unibo.it/mobility-confap-italy/en/research-opportunity-offers-in-italy. Detalhes da rede MCI italiana em https://site.unibo.it/mobility-confap-italy/en/mci-program/network-of-italian-university. As FAPs associadas a esta chamada são: Alagoas - FAPEAL, Amazonas - FAPEAM, Bahia - FAPESB, Ceará - FUNCAP, Espírito Santo – FAPES, Goiás - FAPEG, Maranhão - FAPEMA, Pará - FAPESPA, Paraná - Fundação Araucária, Pernambuco – FACEPE, Rio Grande do Sul - FAPERGS, Santa Catarina - FAPESC. Outras FAPs podem confirmar sua participação.</t>
         </is>
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-MCI-–-MOBILITY-CONFAP-ITALY-2026.pdf</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_MOBILITY_CONFAP_ITALY_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1546,7 +1560,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA HORIZON EUROPE</t>
+          <t>CHAMADA ERC-CONFAP 2026</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -1558,92 +1572,157 @@
       <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="2" t="inlineStr">
         <is>
+          <t>Apoiar a mobilidade de pesquisadores do estado do Espírito Santo para integrar equipes de pesquisa na Europa, em projetos financiados pelo Conselho Europeu de Pesquisa (ERC). O objetivo é possibilitar colaborações de pesquisa, promover oportunidades em equipes internacionais de excelência e fortalecer a internacionalização da ciência, tecnologia e inovação desenvolvida no Espírito Santo.</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores ativos do Brasil, com título de doutor, que implementam atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros. Para FAPES, o proponente deve ser pesquisador principal ou coordenador do projeto, vinculado a IES/P no Espírito Santo, residente no estado, brasileiro ou estrangeiro com visto permanente, com currículo Lattes atualizado, adimplente com a FAPES e em regularidade perante as normas legais vigentes.</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>US$ 18.000,00</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>US$ 6.000,00</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>internacional.confap@gmail.com, global@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-10: Submissão de propostas (CONFAP) (Propostas completas, incluindo todos os documentos solicitados no Item 6 do edital geral, devem ser submetidas via portal https://sistema.confap.org.br/.)
+2026-08-10: Submissão de documentação para verificação de elegibilidade (FAPES) (Submeter via SigFapes a documentação exigida conforme Instrução de Serviços nº 082/2025 e Item 4, alínea B do edital específico da FAPES.)</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>A FAPES apoiará até 3 projetos selecionados. Os recursos podem ser usados como auxílios individuais para estágios ou visitas técnicas de curta duração. O acesso à lista de projetos ERC é liberado após análise de elegibilidade básica pelo CONFAP. Os pesquisadores devem contatar os PIs dos projetos ERC para definir o Plano de Trabalho e condições.</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
+        </is>
+      </c>
+      <c r="N17" s="2" t="inlineStr">
+        <is>
+          <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Chamadas Internacionais</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>CHAMADA HORIZON EUROPE</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr"/>
+      <c r="E18" s="2" t="inlineStr"/>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
           <t>Este edital da FAPES visa apoiar a participação de pesquisadores do estado do Espírito Santo, na condição de co-PI (co-Principal Investigator), em projetos de pesquisa e inovação executados por consórcios de parceiros europeus e associados no âmbito do Programa Horizonte Europa. As diretrizes orientam exclusivamente a submissão de propostas na categoria “C - Projetos Colaborativos (Pilar II)”, que se refere a projetos de pesquisa e inovação em grande escala para desenvolver soluções para desafios globais.</t>
         </is>
       </c>
-      <c r="G17" s="2" t="inlineStr">
+      <c r="G18" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores proponentes do estado do Espírito Santo, na condição de co-PI, vinculados a instituições de pesquisa ou acadêmicas, para participação em consórcios de projetos colaborativos da categoria 'C - Projetos Colaborativos (Pilar II)' do Horizonte Europa.</t>
         </is>
       </c>
-      <c r="H17" s="2" t="n"/>
-      <c r="I17" s="2" t="inlineStr">
+      <c r="H18" s="2" t="n"/>
+      <c r="I18" s="2" t="inlineStr">
         <is>
           <t>€ 25.000,00 por ano de projeto</t>
         </is>
       </c>
-      <c r="J17" s="2" t="inlineStr">
+      <c r="J18" s="2" t="inlineStr">
         <is>
           <t>parcerias@fapes.es.gov.br, internacional.confap@confap.org.br</t>
         </is>
       </c>
-      <c r="K17" s="2" t="inlineStr">
+      <c r="K18" s="2" t="inlineStr">
         <is>
           <t>?: Consulta de Elegibilidade à FAPES (Pesquisadores devem consultar a FAPES sobre sua elegibilidade antes de iniciar a preparação da proposta, enviando informações como CV em inglês, nome e instituição do coordenador da proposta do Horizonte Europa, título da proposta, orçamento estimado, duração do projeto e descrição resumida.)
 ?: Submissão da Proposta à FAPES (A FAPES receberá propostas associadas às chamadas do Horizonte Europa a qualquer momento. A proposta deve incluir cópia da proposta em inglês submetida ao Horizonte Europa, seguir diretrizes da FAPES e indicar detalhes da proposta vinculada.)
 ?: Assinatura do Termo de Outorga FAPES (Disponível somente após a submissão do Acordo de Subvenção com o qual a UE concede o apoio financeiro ao consórcio. O cofinanciamento por parte da Fapes somente poderá ser contratado até o término da vigência do Arranjo Administrativo Horizonte Europa 2021–2027.)</t>
         </is>
       </c>
-      <c r="L17" s="2" t="inlineStr">
+      <c r="L18" s="2" t="inlineStr">
         <is>
           <t>Os parceiros do Brasil não podem ser coordenadores das propostas submetidas ao Horizonte Europa, pois não são automaticamente elegíveis para receber financiamento da UE. Portanto, eles não podem ser responsáveis pela gestão administrativa e financeira geral do projeto; eles só podem participar como parceiros (ou co-PIs). A referência da chamada é o título (Programa/Tópico) e o número da chamada. Os recursos financeiros aplicados pela Fapes para financiamento de projetos no contexto do Horizonte Europa serão oriundos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo - Funcitec, fonte 0159, recursos vinculados ao Tesouro do Estado. Outros recursos financeiros, decorrentes de parcerias futuras ou de disponibilidade da Fapes e/ou do Funcitec, poderão ser aplicados na suplementação de propostas aprovadas no âmbito do Horizonte Europa 2021-2027. O número máximo de propostas a serem apoiadas no âmbito destas Diretrizes é de até 2 (DOIS) projetos por ano do Horizonte Europa 2021-2027. Os recursos financeiros aprovados pela Fundação poderão abranger despesas com passagens e diárias, observando suas respectivas regulamentações disponíveis na Resolução CCAF nº 309/2022.</t>
         </is>
       </c>
-      <c r="M17" s="2" t="inlineStr">
+      <c r="M18" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20Horizon%20Europe%202021-2027-1.pdf</t>
         </is>
       </c>
-      <c r="N17" s="2" t="inlineStr">
+      <c r="N18" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_HORIZON_EUROPE.pdf</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>Chamadas Internacionais</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="B19" s="2" t="inlineStr">
         <is>
           <t>CHAMADA DA PARCERIA DE MATÉRIAS-PRIMAS PARA A TRANSIÇÃO VERDE E DIGITAL (RAMP)</t>
         </is>
       </c>
-      <c r="C18" s="2" t="inlineStr">
+      <c r="C19" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr">
+      <c r="D19" s="2" t="inlineStr">
         <is>
           <t>2026-09-22: Prazo final para submissão de pré-propostas (Até as 15:00 CEST)</t>
         </is>
       </c>
-      <c r="E18" s="2" t="inlineStr"/>
-      <c r="F18" s="2" t="inlineStr">
+      <c r="E19" s="2" t="inlineStr"/>
+      <c r="F19" s="2" t="inlineStr">
         <is>
           <t>Este edital visa financiar projetos transnacionais de pesquisa e inovação em matérias-primas para a transição verde e digital. Os projetos devem focar em melhorar o acesso a matérias-primas, promover práticas de economia circular, alcançar a sustentabilidade e minimizar custos sociais e ambientais, agregando valor e contribuindo para o desenvolvimento industrial.</t>
         </is>
       </c>
-      <c r="G18" s="2" t="inlineStr">
+      <c r="G19" s="2" t="inlineStr">
         <is>
           <t>Organizações de ensino superior e centros de pesquisa públicos. Os consórcios devem ser compostos por, no mínimo, três parceiros de três países diferentes (sendo pelo menos dois da UE ou países associados).</t>
         </is>
       </c>
-      <c r="H18" s="2" t="n"/>
-      <c r="I18" s="2" t="inlineStr">
+      <c r="H19" s="2" t="n"/>
+      <c r="I19" s="2" t="inlineStr">
         <is>
           <t>EUR 100.000,00</t>
         </is>
       </c>
-      <c r="J18" s="2" t="inlineStr">
+      <c r="J19" s="2" t="inlineStr">
         <is>
           <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K18" s="2" t="inlineStr">
+      <c r="K19" s="2" t="inlineStr">
         <is>
           <t>2026-09-22: Prazo final para submissão de pré-propostas (Até as 15:00 CEST)
 2026-09-22: Submissão de propostas nacionais FAPES (Etapa 1) (Recomendado verificar requisitos da FAPES para submissão na plataforma nacional, prazo idêntico ao da submissão da pré-proposta internacional.)
@@ -1657,17 +1736,17 @@
 2027-06-01 a 2027-09-30: Negociações de contrato nacional/regional / Início dos projetos (esperado)</t>
         </is>
       </c>
-      <c r="L18" s="2" t="inlineStr">
+      <c r="L19" s="2" t="inlineStr">
         <is>
           <t>O edital é um Joint Transnational Call (JTC) 2026 da Parceria Europeia em Matérias-Primas para a Transição Verde e Digital (RAMP). A FAPES (Fundação de Amparo à Pesquisa e Inovação do Espírito Santo) participa sob o guarda-chuva do CONFAP. Cada parceiro de projeto é financiado diretamente por sua respectiva agência nacional/regional. A Comissão Europeia cofinancia os JTCs da RAMP, com o cofinanciamento sendo redistribuído pelas agências financiadoras aos seus beneficiários. A duração máxima dos projetos é de 36 meses. Propostas devem se enquadrar em um dos seis tópicos temáticos e adotar princípios de 'Safe and Sustainable by Design'. Conforme a tabela de elegibilidade de parceiros do CONFAP, empresas (SMEs e grandes) e entidades sem fins lucrativos (ONGs, associações, sociedades, fundações) não são elegíveis para financiamento pela FAPES.</t>
         </is>
       </c>
-      <c r="M18" s="2" t="inlineStr">
+      <c r="M19" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20-%20Chamada%20RAMP%202026.pdf</t>
         </is>
       </c>
-      <c r="N18" s="2" t="inlineStr">
+      <c r="N19" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_DA_PARCERIA_DE_MATÉRIAS-PRIMAS_PARA_A_TRANSIÇÃO_VERDE_E_DIGITAL_(RAMP).pdf</t>
         </is>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-09-12 10:50
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -949,11 +949,7 @@
           <t>Removido (nao mais aberto)</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-04 a 2026-09-11: Submissão de propostas (Até as 17h:59. Para 3ª Chamada (eventos com início entre 04/01/2027 a 30/04/2027))</t>
-        </is>
-      </c>
+      <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-09-14 13:47
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,12 +29,17 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -49,12 +54,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -422,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N19"/>
+  <dimension ref="A1:N20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1014,46 +1022,117 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>EDITAL FAPES Nº 28/2025 - PUBLICAÇÃO DE ARTIGOS TÉCNICO-CIENTÍFICOS</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>Removido (nao mais aberto)</t>
+          <t>EDITAL FAPES Nº 25/2026 - CIÊNCIA ABERTA CAPIXABA</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Novo - e-mail enviado em 14/09/2026</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-06 a 2026-10-26: Submissão de propostas (4ª Chamada, até as 17h59)</t>
+          <t>2026-10-08: Prazo para envio de dúvidas a respeito do edital (até as 17h59)</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr"/>
       <c r="F9" s="2" t="inlineStr">
         <is>
+          <t>Apoiar projetos voltados à organização, disponibilização, disseminação e aplicação de dados, informações e evidências científicas de interesse público. O edital busca ampliar o acesso ao conhecimento científico produzido no Espírito Santo, fortalecer sua integração a redes e sistemas de informação nacionais e internacionais e promover sua comunicação para diferentes segmentos da sociedade. O foco é construir uma infraestrutura pública de dados e conhecimento científico sobre temáticas estabelecidas, não financiar pesquisas.</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Profissionais/pesquisadores doutores, vinculados a Instituições de Ensino Superior/ou de Pesquisa (IES/P) públicas ou privadas, sediadas no Estado do Espírito Santo ou em município limítrofe, com vínculo estatutário ou celetista por tempo indeterminado. A equipe executora deve incluir o coordenador e, no mínimo, dois pesquisadores doutores de IES/P de fora do Estado.</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>R$ 3.000.000,00</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>R$ 200.000,00</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>editais.duvidas@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08: Prazo para envio de dúvidas a respeito do edital (até as 17h59)
+2026-09-14 a 2026-10-15: Submissão de propostas e documentos (até as 17h59 via SigFapes)
+?: Prazo para interposição de recursos (habilitação) (5 dias úteis após a divulgação do resultado preliminar da habilitação)
+?: Prazo para interposição de recursos (análise de mérito) (5 dias úteis após a divulgação do resultado preliminar da análise de mérito)</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>As propostas devem estar enquadradas em uma das seguintes linhas temáticas: Saúde e Saúde Pública; Sustentabilidade Socioambiental, Descarbonização e Clima; Biodiversidade e Recursos Naturais; Cidades e Territórios Sustentáveis e Resilientes; Agricultura, Produção de Alimentos e Segurança Alimentar. A distribuição dos recursos financeiros prevê a seleção das 2 (duas) propostas com as maiores Notas Finais em cada linha temática, e após, as demais propostas serão selecionadas conforme a ordem decrescente de Nota Final, independentemente da linha temática, até o limite dos recursos. A Fapes pode alterar as datas e os prazos do cronograma por necessidade administrativa ou decisão institucional.</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_25-2026_Ciência_Aberta_Capixaba.pdf</t>
+        </is>
+      </c>
+      <c r="N9" s="2" t="inlineStr">
+        <is>
+          <t>difusao_do_conhecimento/EDITAL_FAPES_No_25_2026_-_CIÊNCIA_ABERTA_CAPIXABA.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Difusão do Conhecimento</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>EDITAL FAPES Nº 28/2025 - PUBLICAÇÃO DE ARTIGOS TÉCNICO-CIENTÍFICOS</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Removido (nao mais aberto)</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06 a 2026-10-26: Submissão de propostas (4ª Chamada, até as 17h59)</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
           <t>O objetivo geral deste edital é incentivar a publicação científica e tecnológica no Espírito Santo por meio da concessão de auxílio financeiro para publicação de artigos técnico-científicos que apresentem resultados de pesquisa desenvolvidas em Instituições de Ensino e/ou Pesquisa no estado. A chamada pública visa selecionar propostas para concessão de auxílio financeiro para tal finalidade, valorizando a produção técnico-científica e ampliando a visibilidade das atividades de pesquisa e inovação.</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>Pesquisador ou aluno em atividade de pesquisa ou desenvolvimento inovador em Instituição de Ensino e/ou Pesquisa (IES/P) localizada no estado do Espírito Santo.</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>R$ 800.000,00</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>US$ 1.500,00</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr">
+      <c r="J10" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K9" s="2" t="inlineStr">
+      <c r="K10" s="2" t="inlineStr">
         <is>
           <t>2025-12-22 a 2026-02-25: Submissão de propostas (1ª Chamada, até as 17h59)
 2026-02-17: Prazo para impugnação do edital (Até 5 dias úteis antes do encerramento do prazo de submissão da primeira chamada)
@@ -1069,70 +1148,70 @@
 ?: Prestação de contas (Até 30 dias após o término de vigência do Termo de Outorga (prazo máximo de execução do projeto é de 12 meses))</t>
         </is>
       </c>
-      <c r="L9" s="2" t="inlineStr">
+      <c r="L10" s="2" t="inlineStr">
         <is>
           <t>O artigo deve ter sido aceito em periódico classificado entre A1 e A4 no Qualis-Capes (2021-2024) ou com percentil igual ou superior a 50% nas plataformas Scopus ou ISI Web of Science. O proponente poderá ser contratado para no máximo 2 propostas, desde que submetidas em chamadas distintas. Cada coordenador pode apresentar apenas uma proposta por chamada; caso envie mais de uma, apenas a última será considerada. O prazo máximo para execução de cada projeto é de 12 meses.</t>
         </is>
       </c>
-      <c r="M9" s="2" t="inlineStr">
+      <c r="M10" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_28_2025_Publicação_de_Artigos_Técnico-Científicos.pdf</t>
         </is>
       </c>
-      <c r="N9" s="2" t="inlineStr">
+      <c r="N10" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_28_2025_-_PUBLICAÇÃO_DE_ARTIGOS_TÉCNICO-CIENTÍFICOS.pdf</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>Extensão</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 01/2026 – TCC EMPREENDEDOR INOVADOR</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>2026-09-02 a 2026-10-27: Período de submissão das propostas (Segunda Chamada) (Até 17h59)</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr"/>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr"/>
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>Incentivar o desenvolvimento de Trabalhos de Conclusão de Curso (TCCs) com foco em inovação, empreendedorismo e aplicabilidade prática. O edital visa a concessão de Bolsas de Apoio a Trabalho de Conclusão de Curso (BTCC) para a execução de TCCs que apresentem soluções inovadoras e empreendedoras. As propostas devem ter fundamentação teórico-metodológica consistente, voltadas para aplicação prática e impacto econômico, social e/ou ambiental no Estado do Espírito Santo, alinhados aos ODS da ONU e ao Plano ES 500 Anos.</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>Professores orientadores com vínculo estatutário ou celetista por tempo indeterminado com Instituição de Ensino Superior (IES) reconhecida pelo Ministério da Educação (MEC), localizada no Espírito Santo, que submetam entre 3 (três) e 5 (cinco) propostas.</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>R$ 1.600.000,00</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>R$ 11.000,00</t>
         </is>
       </c>
-      <c r="J10" s="2" t="inlineStr">
+      <c r="J11" s="2" t="inlineStr">
         <is>
           <t>editais.extensao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K10" s="2" t="inlineStr">
+      <c r="K11" s="2" t="inlineStr">
         <is>
           <t>?: Impugnação do Edital (Até 5 (cinco) dias úteis antes do encerramento do prazo de submissão das propostas de cada chamada.)
 2026-02-02 a 2026-03-30: Período de submissão das propostas (Primeira Chamada) (Até 17h59)
@@ -1149,66 +1228,66 @@
 ?: Prazo para solicitação de ofício para abertura de conta (Até 3 (três) dias úteis para o Outorgado.)</t>
         </is>
       </c>
-      <c r="L10" s="2" t="inlineStr">
+      <c r="L11" s="2" t="inlineStr">
         <is>
           <t>O prazo de execução dos projetos será de um semestre letivo, acrescido de até 3 (três) meses apenas para apresentação da Declaração ou Ata de Defesa do TCC. Cada projeto de TCC deve demonstrar potencial de geração de valor, criação de negócios ou produtos inovadores; estar alinhado aos ODS da ONU (especialmente ODS 4, 8, 9, 10 e 17) e ao Plano ES 500 Anos, e ser desenvolvido em consonância com os Projetos Pedagógicos dos respectivos cursos de graduação. As propostas concorrerão com as demais de suas respectivas microrregiões, sendo apoiados, na primeira chamada, no máximo 20 (vinte) projetos de TCC por microrregião e, na segunda e terceira chamadas, até 10 (dez) projetos de TCC por microrregião. Recursos remanescentes serão destinados a projetos em ampla concorrência por ordem decrescente de nota. Propostas submetidas a mais de uma microrregião serão desclassificadas. Cada proposta deverá vincular um único aluno sob orientação do proponente. O proponente que indicar alunos orientados vinculados a outra IES deverá apresentar declaração de autorização tanto da sua IES de vínculo quanto da IES à qual os alunos orientados estão vinculados. Propostas com Nota Final (NF) inferior a 70 (setenta) pontos serão desclassificadas. Não será permitido o acúmulo de bolsas Fapes pelo aluno orientado, exceto com bolsas do Programa Nossa Bolsa, do Programa Universidade para Todos (Prouni) e com Bolsas de Extensão (Ext-E e Ext-F) da Fapes.</t>
         </is>
       </c>
-      <c r="M10" s="2" t="inlineStr">
+      <c r="M11" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_Nº_01.2026_TCC_EMPREENDEDOR_INOVADOR-2.pdf</t>
         </is>
       </c>
-      <c r="N10" s="2" t="inlineStr">
+      <c r="N11" s="2" t="inlineStr">
         <is>
           <t>extensao/EDITAL_FAPES_No_01_2026_–_TCC_EMPREENDEDOR_INOVADOR.pdf</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 08/2026 - NOVA ECONOMIA CAPIXABA 2026</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr"/>
-      <c r="E11" s="2" t="inlineStr"/>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr"/>
+      <c r="E12" s="2" t="inlineStr"/>
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>Promover o aumento da competitividade dos setores econômicos capixabas por meio de projetos de inovação, desenvolvidos por empresas (incluindo cooperativas de trabalho) em colaboração com Instituições de Ciência e Tecnologia (ICT) ou Instituições de Ensino Superior (IES) capixabas. O apoio se dará por meio de um modelo de coinvestimento tripartite (FAPES, empresa/cooperativa, ICT/IES), com projetos alinhados ao Plano ES 500 Anos e ao Plano Estadual de Ciência, Tecnologia e Inovação do Espírito Santo (PCTI-ES).</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>Empresas com sede administrativa ou filial no Espírito Santo, individualmente ou em associação com outras empresas ou cooperativas de trabalho capixabas.</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="H12" s="2" t="inlineStr">
         <is>
           <t>R$ 40.000.000,00</t>
         </is>
       </c>
-      <c r="I11" s="2" t="inlineStr">
+      <c r="I12" s="2" t="inlineStr">
         <is>
           <t>R$ 500.000,00 a R$ 3.000.000,00</t>
         </is>
       </c>
-      <c r="J11" s="2" t="inlineStr">
+      <c r="J12" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K11" s="2" t="inlineStr">
+      <c r="K12" s="2" t="inlineStr">
         <is>
           <t>2026-03-30: Submissão das propostas no SIGFAPES (Fluxo contínuo)
 ?: Prazo de submissão dos recursos administrativos (Habilitação) (5 dias úteis a partir da publicação do resultado preliminar da habilitação.)
@@ -1217,70 +1296,70 @@
 ?: Submissão das documentações para contratação (Até 30 dias a partir da publicação do resultado homologado do julgamento de mérito.)</t>
         </is>
       </c>
-      <c r="L11" s="2" t="inlineStr">
+      <c r="L12" s="2" t="inlineStr">
         <is>
           <t>O prazo de execução do projeto é de 24 meses, com possibilidade de prorrogação por até 12 meses. As empresas proponentes e coexecutoras devem ter receita bruta operacional superior a R$ 360.000,00 nos dois últimos exercícios fiscais; cooperativas de trabalho devem apresentar Demonstração de Sobras ou Perdas (DSP). As empresas devem estar ativas há pelo menos 6 meses e não podem ter sido contratadas em editais FAPES nº 07/2024, nº 10/2025 e nº 06/2026, a menos que o projeto, coordenador e equipe executora sejam distintos. É permitida apenas uma proposta por empresa. Em caso de inabilitação ou desclassificação, a empresa poderá realizar uma nova submissão, exceto se reprovada pelo Comitê de Conformidade, o que impede nova submissão nesta chamada. A aprovação da proposta não garante a contratação, que está sujeita à disponibilidade financeira da FAPES, ordem de submissão e visita técnica. O critério de desempate é a data de submissão da proposta no SIGFAPES. Propostas com Nota Final inferior a 80 pontos ou notas individuais inferiores a 4 em critérios específicos serão desclassificadas. A impugnação dos termos do edital deve ser feita em até 5 dias úteis antes do encerramento do prazo de submissão das propostas do primeiro ciclo (considerando o fluxo contínuo, esta observação se refere a um prazo inicial para impugnação do edital em si).</t>
         </is>
       </c>
-      <c r="M11" s="2" t="inlineStr">
+      <c r="M12" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_08-2026_-_Nova_Economia_Capixaba_-_2_Edição_-_Lançamento.pdf</t>
         </is>
       </c>
-      <c r="N11" s="2" t="inlineStr">
+      <c r="N12" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_No_08_2026_-_NOVA_ECONOMIA_CAPIXABA_2026.pdf</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B13" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES N° 23/2026 - APOIO ÀS INCUBADORAS DO ESPÍRITO SANTO</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C13" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="D13" s="2" t="inlineStr">
         <is>
           <t>2026-09-17: Prazo para impugnação do edital (Até 5 dias úteis anteriores ao encerramento do prazo de envio das propostas. O pedido deve ser enviado no E-Flow por meio do Formulário de Impugnação de Edital.)</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr"/>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="E13" s="2" t="inlineStr"/>
+      <c r="F13" s="2" t="inlineStr">
         <is>
           <t>O edital visa apoiar incubadoras públicas ou privadas sem fins lucrativos, localizadas no Espírito Santo, que buscam estimular e prestar apoio logístico, gerencial e/ou tecnológico a empreendedores e empresas com produtos, serviços ou modelos de negócio inovadores. Este apoio busca ampliar, aperfeiçoar e consolidar as atividades de pré-incubação, incubação e pós-incubação, promovendo a capacitação de novos empreendedores e o desenvolvimento socioeconômico do estado.</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G13" s="2" t="inlineStr">
         <is>
           <t>Incubadoras, sem fins lucrativos, sediadas no Espírito Santo, que atendam aos requisitos do edital.</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="H13" s="2" t="inlineStr">
         <is>
           <t>R$ 4.500.000,00</t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr">
+      <c r="I13" s="2" t="inlineStr">
         <is>
           <t>R$ 252.000,00</t>
         </is>
       </c>
-      <c r="J12" s="2" t="inlineStr">
+      <c r="J13" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K12" s="2" t="inlineStr">
+      <c r="K13" s="2" t="inlineStr">
         <is>
           <t>2026-09-17: Prazo para impugnação do edital (Até 5 dias úteis anteriores ao encerramento do prazo de envio das propostas. O pedido deve ser enviado no E-Flow por meio do Formulário de Impugnação de Edital.)
 2026-08-25 a 2026-09-24: Envio da proposta e documentos (Até as 17h59, via SigFapes)
@@ -1288,83 +1367,19 @@
 2026-11-04: Contratação dos projetos selecionados (A partir desta data)</t>
         </is>
       </c>
-      <c r="L12" s="2" t="inlineStr">
+      <c r="L13" s="2" t="inlineStr">
         <is>
           <t>O projeto terá prazo de vigência de 24 meses, sem prorrogação. Os recursos financeiros remanescentes, caso o número de propostas previstas para contratação nos níveis de maturidade I, II ou III não seja alcançado, serão redirecionados para propostas suplentes. Os recursos destinados ao custeio (exceto bolsas) serão liberados em 2 parcelas. Caso a proposta seja enquadrada em nível de maturidade distinto do indicado pelo proponente, os valores financiáveis serão ajustados proporcionalmente. É obrigatório destinar no mínimo 20% do valor total solicitado para bolsas. As incubadoras beneficiárias devem destinar parte dos recursos de custeio à associação à Anprotec. Propostas com nota final inferior a 60 pontos serão desclassificadas. A classificação por nível de maturidade é a seguinte: Nível Avançado (86 a 100 pontos), Nível Intermediário (76 a 85 pontos), Nível Básico (60 a 75 pontos).</t>
         </is>
       </c>
-      <c r="M12" s="2" t="inlineStr">
+      <c r="M13" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_23-2026_Apoio%20a%20Incubadoras_(Versão%20Final).pdf</t>
         </is>
       </c>
-      <c r="N12" s="2" t="inlineStr">
+      <c r="N13" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_N°_23_2026_-_APOIO_ÀS_INCUBADORAS_DO_ESPÍRITO_SANTO.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>Chamadas Internacionais</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>CHAMADA CONFAP CDTI 2026</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-08: Submissão de propostas (Até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Os formulários devem ser preenchidos em língua inglesa.)</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr"/>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>Apoiar projetos colaborativos de pesquisa e inovação tecnológica entre o Brasil e a Espanha, abrangendo qualquer setor de atividade. Destina-se a profissionais vinculados a universidades, centros de pesquisa ou empresas do Espírito Santo que desenvolvam atividades de P,D&amp;I e que apresentem propostas conjuntas com empresas espanholas.</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores principais ou coordenadores de projetos, brasileiros ou estrangeiros com visto permanente, residentes no Espírito Santo, com vínculo ativo a universidades, centros de pesquisa ou empresas localizadas no estado do Espírito Santo, que realizem atividades de pesquisa, desenvolvimento e inovação tecnológica e que integrem proposta conjunta com empresa espanhola.</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="n"/>
-      <c r="I13" s="2" t="inlineStr">
-        <is>
-          <t>€ 75.000,00</t>
-        </is>
-      </c>
-      <c r="J13" s="2" t="inlineStr">
-        <is>
-          <t>internacional.confap@gmail.com, brasil@cdti.es, carlos.quintana@cdti.es, global4@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K13" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-08: Submissão de propostas (Até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Os formulários devem ser preenchidos em língua inglesa.)</t>
-        </is>
-      </c>
-      <c r="L13" s="2" t="inlineStr">
-        <is>
-          <t>A FAPES apoiará um único projeto. Os projetos terão duração de 12 a 36 meses. O apoio financeiro da FAPES destina-se a despesas de capital e custeio, excluindo bolsas, conforme Resolução nº 309/2022. Cada proponente pode submeter apenas uma proposta. A submissão à FAPES (via SigFapes) para contratação ocorrerá somente após a aprovação da proposta pelo CDTI. Os projetos devem ter um orçamento total mínimo de € 250.000,00, e o apoio da FAPES deve corresponder a no mínimo 30% da contrapartida do valor total da proposta.</t>
-        </is>
-      </c>
-      <c r="M13" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes_Chamada%20Internacional_CDTI.2026.pdf</t>
-        </is>
-      </c>
-      <c r="N13" s="2" t="inlineStr">
-        <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_CDTI_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1376,7 +1391,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA CONFAP &amp; WBI - BÉLGICA 2026</t>
+          <t>CHAMADA CONFAP CDTI 2026</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1386,53 +1401,49 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília), exclusivamente por meio da plataforma https://sistema.confap.org.br.)</t>
+          <t>2026-10-08: Submissão de propostas (Até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Os formulários devem ser preenchidos em língua inglesa.)</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Apoiar projetos conjuntos de Pesquisa e Inovação, promovendo o intercâmbio científico entre grupos de pesquisa do Espírito Santo e da região da Valônia-Bruxelas, na Bélgica, em áreas como inovação em saúde, energia sustentável, gestão ambiental e aeronáutica. Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas.</t>
+          <t>Apoiar projetos colaborativos de pesquisa e inovação tecnológica entre o Brasil e a Espanha, abrangendo qualquer setor de atividade. Destina-se a profissionais vinculados a universidades, centros de pesquisa ou empresas do Espírito Santo que desenvolvam atividades de P,D&amp;I e que apresentem propostas conjuntas com empresas espanholas.</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores brasileiros com doutorado, vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) localizadas no estado do Espírito Santo, residentes no estado, que atuem como pesquisador principal ou coordenador do projeto, e que participem de propostas conjuntas com pesquisadores da Valônia-Bruxelas, Bélgica.</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="inlineStr">
-        <is>
-          <t>R$ 300.000,00</t>
-        </is>
-      </c>
+          <t>Pesquisadores principais ou coordenadores de projetos, brasileiros ou estrangeiros com visto permanente, residentes no Espírito Santo, com vínculo ativo a universidades, centros de pesquisa ou empresas localizadas no estado do Espírito Santo, que realizem atividades de pesquisa, desenvolvimento e inovação tecnológica e que integrem proposta conjunta com empresa espanhola.</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="n"/>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>R$ 150.000,00</t>
+          <t>€ 75.000,00</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
+          <t>internacional.confap@gmail.com, brasil@cdti.es, carlos.quintana@cdti.es, global4@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília), exclusivamente por meio da plataforma https://sistema.confap.org.br.)</t>
+          <t>2026-10-08: Submissão de propostas (Até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Os formulários devem ser preenchidos em língua inglesa.)</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas. O prazo de vigência máximo para cada projeto é de 24 meses. O apoio financeiro da Fapes destina-se exclusivamente a despesas de mobilidade, excluindo bolsas. Cada proponente pode submeter apenas uma proposta; em caso de múltiplas submissões, apenas a última será considerada. As propostas devem ser submetidas utilizando o modelo do Anexo I (Application Form Template) em ambas as plataformas (CONFAP).</t>
+          <t>A FAPES apoiará um único projeto. Os projetos terão duração de 12 a 36 meses. O apoio financeiro da FAPES destina-se a despesas de capital e custeio, excluindo bolsas, conforme Resolução nº 309/2022. Cada proponente pode submeter apenas uma proposta. A submissão à FAPES (via SigFapes) para contratação ocorrerá somente após a aprovação da proposta pelo CDTI. Os projetos devem ter um orçamento total mínimo de € 250.000,00, e o apoio da FAPES deve corresponder a no mínimo 30% da contrapartida do valor total da proposta.</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20WBI%20-2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes_Chamada%20Internacional_CDTI.2026.pdf</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WBI_-_BÉLGICA_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_CDTI_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1444,7 +1455,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA CONFAP &amp; DAAD 2026</t>
+          <t>CHAMADA CONFAP &amp; WBI - BÉLGICA 2026</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1452,20 +1463,32 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr"/>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília), exclusivamente por meio da plataforma https://sistema.confap.org.br.)</t>
+        </is>
+      </c>
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Apoiar a manutenção de bolsas de doutorado da FAPES para bolsistas que forem selecionados pelo Serviço Alemão de Intercâmbio Acadêmico (DAAD). O suporte visa permitir que esses bolsistas realizem suas pesquisas em instituições na Alemanha, no âmbito da Chamada DAAD 2026.</t>
+          <t>Apoiar projetos conjuntos de Pesquisa e Inovação, promovendo o intercâmbio científico entre grupos de pesquisa do Espírito Santo e da região da Valônia-Bruxelas, na Bélgica, em áreas como inovação em saúde, energia sustentável, gestão ambiental e aeronáutica. Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas.</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Bolsistas de doutorado da FAPES que forem selecionados pelo DAAD, que estejam adimplentes junto à FAPES e que não estejam no primeiro nem no último ano do doutorado.</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="n"/>
-      <c r="I15" s="2" t="n"/>
+          <t>Pesquisadores brasileiros com doutorado, vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) localizadas no estado do Espírito Santo, residentes no estado, que atuem como pesquisador principal ou coordenador do projeto, e que participem de propostas conjuntas com pesquisadores da Valônia-Bruxelas, Bélgica.</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>R$ 300.000,00</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>R$ 150.000,00</t>
+        </is>
+      </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
           <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
@@ -1473,22 +1496,22 @@
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>?: Submissão de propostas (As propostas deverão ser submetidas na Plataforma do DAAD, conforme item 3.1.)</t>
+          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília), exclusivamente por meio da plataforma https://sistema.confap.org.br.)</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>Este documento apresenta as diretrizes específicas da FAPES para a Chamada DAAD 2026, complementando o edital completo disponível no site do CONFAP.</t>
+          <t>Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas. O prazo de vigência máximo para cada projeto é de 24 meses. O apoio financeiro da Fapes destina-se exclusivamente a despesas de mobilidade, excluindo bolsas. Cada proponente pode submeter apenas uma proposta; em caso de múltiplas submissões, apenas a última será considerada. As propostas devem ser submetidas utilizando o modelo do Anexo I (Application Form Template) em ambas as plataformas (CONFAP).</t>
         </is>
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20-%20FAPES%202026-1.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20WBI%20-2026.pdf</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_DAAD_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WBI_-_BÉLGICA_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1500,7 +1523,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA MOBILITY CONFAP ITALY 2026</t>
+          <t>CHAMADA CONFAP &amp; DAAD 2026</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -1512,39 +1535,39 @@
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>O edital MOBILITY CONFAP ITALY CALL 2026 visa apoiar pesquisadores do Brasil, vinculados a instituições de ensino superior e pesquisa brasileiras, que desejam desenvolver atividades de pesquisa na Itália em colaboração com colegas locais. O objetivo é facilitar e apoiar a colaboração científica, tecnológica e de inovação por meio da mobilidade de estudantes de doutorado, mestrado e pós-doutorado. O suporte é oferecido na forma de bolsas de estudo para fortalecer grupos de pesquisa brasileiros através de colaborações e visitas a grupos de pesquisa na Itália, parte da rede MCI.</t>
+          <t>Apoiar a manutenção de bolsas de doutorado da FAPES para bolsistas que forem selecionados pelo Serviço Alemão de Intercâmbio Acadêmico (DAAD). O suporte visa permitir que esses bolsistas realizem suas pesquisas em instituições na Alemanha, no âmbito da Chamada DAAD 2026.</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores de doutorado, mestrado e pós-doutorado vinculados a universidades e instituições de pesquisa nos Estados brasileiros participantes, que possuam um supervisor associado a uma universidade italiana parte da rede MCI.</t>
+          <t>Bolsistas de doutorado da FAPES que forem selecionados pelo DAAD, que estejam adimplentes junto à FAPES e que não estejam no primeiro nem no último ano do doutorado.</t>
         </is>
       </c>
       <c r="H16" s="2" t="n"/>
       <c r="I16" s="2" t="n"/>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com</t>
+          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04: Submissão de propostas (Até as 11:59 (horário de Brasília) via https://sistema.confap.org.br. Proponentes devem verificar com suas FAPs sobre submissão em plataformas próprias.)</t>
+          <t>?: Submissão de propostas (As propostas deverão ser submetidas na Plataforma do DAAD, conforme item 3.1.)</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>As FAPs participantes podem exigir critérios de elegibilidade adicionais e definir as modalidades de apoio, incluindo os valores das bolsas mensais, em suas próprias diretrizes ou orientações, devendo ser consultadas pelos candidatos antes da preparação da proposta. Não serão cobradas taxas de matrícula por nenhuma das partes para qualquer mobilidade de intercâmbio. Em caso de mobilidade no âmbito de projetos com potencial valor comercial e direitos de propriedade intelectual, as instituições anfitriãs e de envio deverão assinar um acordo de colaboração específico. As propostas devem incluir: projeto de pesquisa, Curriculum Vitae do candidato (Brasil), Curriculum Vitae do supervisor (Itália) e carta de apoio do supervisor na universidade italiana. As FAPs podem solicitar documentos adicionais. As vagas e oportunidades de pesquisa nas universidades italianas da rede MCI estão disponíveis em https://site.unibo.it/mobility-confap-italy/en/research-opportunity-offers-in-italy. Detalhes da rede MCI italiana em https://site.unibo.it/mobility-confap-italy/en/mci-program/network-of-italian-university. As FAPs associadas a esta chamada são: Alagoas - FAPEAL, Amazonas - FAPEAM, Bahia - FAPESB, Ceará - FUNCAP, Espírito Santo – FAPES, Goiás - FAPEG, Maranhão - FAPEMA, Pará - FAPESPA, Paraná - Fundação Araucária, Pernambuco – FACEPE, Rio Grande do Sul - FAPERGS, Santa Catarina - FAPESC. Outras FAPs podem confirmar sua participação.</t>
+          <t>Este documento apresenta as diretrizes específicas da FAPES para a Chamada DAAD 2026, complementando o edital completo disponível no site do CONFAP.</t>
         </is>
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-MCI-–-MOBILITY-CONFAP-ITALY-2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20-%20FAPES%202026-1.pdf</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_MOBILITY_CONFAP_ITALY_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_DAAD_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1556,7 +1579,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA ERC-CONFAP 2026</t>
+          <t>CHAMADA MOBILITY CONFAP ITALY 2026</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -1568,48 +1591,39 @@
       <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Apoiar a mobilidade de pesquisadores do estado do Espírito Santo para integrar equipes de pesquisa na Europa, em projetos financiados pelo Conselho Europeu de Pesquisa (ERC). O objetivo é possibilitar colaborações de pesquisa, promover oportunidades em equipes internacionais de excelência e fortalecer a internacionalização da ciência, tecnologia e inovação desenvolvida no Espírito Santo.</t>
+          <t>O edital MOBILITY CONFAP ITALY CALL 2026 visa apoiar pesquisadores do Brasil, vinculados a instituições de ensino superior e pesquisa brasileiras, que desejam desenvolver atividades de pesquisa na Itália em colaboração com colegas locais. O objetivo é facilitar e apoiar a colaboração científica, tecnológica e de inovação por meio da mobilidade de estudantes de doutorado, mestrado e pós-doutorado. O suporte é oferecido na forma de bolsas de estudo para fortalecer grupos de pesquisa brasileiros através de colaborações e visitas a grupos de pesquisa na Itália, parte da rede MCI.</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores ativos do Brasil, com título de doutor, que implementam atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros. Para FAPES, o proponente deve ser pesquisador principal ou coordenador do projeto, vinculado a IES/P no Espírito Santo, residente no estado, brasileiro ou estrangeiro com visto permanente, com currículo Lattes atualizado, adimplente com a FAPES e em regularidade perante as normas legais vigentes.</t>
-        </is>
-      </c>
-      <c r="H17" s="2" t="inlineStr">
-        <is>
-          <t>US$ 18.000,00</t>
-        </is>
-      </c>
-      <c r="I17" s="2" t="inlineStr">
-        <is>
-          <t>US$ 6.000,00</t>
-        </is>
-      </c>
+          <t>Pesquisadores de doutorado, mestrado e pós-doutorado vinculados a universidades e instituições de pesquisa nos Estados brasileiros participantes, que possuam um supervisor associado a uma universidade italiana parte da rede MCI.</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="n"/>
+      <c r="I17" s="2" t="n"/>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com, global@fapes.es.gov.br</t>
+          <t>internacional.confap@gmail.com</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>2026-08-10: Submissão de propostas (CONFAP) (Propostas completas, incluindo todos os documentos solicitados no Item 6 do edital geral, devem ser submetidas via portal https://sistema.confap.org.br/.)
-2026-08-10: Submissão de documentação para verificação de elegibilidade (FAPES) (Submeter via SigFapes a documentação exigida conforme Instrução de Serviços nº 082/2025 e Item 4, alínea B do edital específico da FAPES.)</t>
+          <t>2026-09-04: Submissão de propostas (Até as 11:59 (horário de Brasília) via https://sistema.confap.org.br. Proponentes devem verificar com suas FAPs sobre submissão em plataformas próprias.)</t>
         </is>
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>A FAPES apoiará até 3 projetos selecionados. Os recursos podem ser usados como auxílios individuais para estágios ou visitas técnicas de curta duração. O acesso à lista de projetos ERC é liberado após análise de elegibilidade básica pelo CONFAP. Os pesquisadores devem contatar os PIs dos projetos ERC para definir o Plano de Trabalho e condições.</t>
+          <t>As FAPs participantes podem exigir critérios de elegibilidade adicionais e definir as modalidades de apoio, incluindo os valores das bolsas mensais, em suas próprias diretrizes ou orientações, devendo ser consultadas pelos candidatos antes da preparação da proposta. Não serão cobradas taxas de matrícula por nenhuma das partes para qualquer mobilidade de intercâmbio. Em caso de mobilidade no âmbito de projetos com potencial valor comercial e direitos de propriedade intelectual, as instituições anfitriãs e de envio deverão assinar um acordo de colaboração específico. As propostas devem incluir: projeto de pesquisa, Curriculum Vitae do candidato (Brasil), Curriculum Vitae do supervisor (Itália) e carta de apoio do supervisor na universidade italiana. As FAPs podem solicitar documentos adicionais. As vagas e oportunidades de pesquisa nas universidades italianas da rede MCI estão disponíveis em https://site.unibo.it/mobility-confap-italy/en/research-opportunity-offers-in-italy. Detalhes da rede MCI italiana em https://site.unibo.it/mobility-confap-italy/en/mci-program/network-of-italian-university. As FAPs associadas a esta chamada são: Alagoas - FAPEAL, Amazonas - FAPEAM, Bahia - FAPESB, Ceará - FUNCAP, Espírito Santo – FAPES, Goiás - FAPEG, Maranhão - FAPEMA, Pará - FAPESPA, Paraná - Fundação Araucária, Pernambuco – FACEPE, Rio Grande do Sul - FAPERGS, Santa Catarina - FAPESC. Outras FAPs podem confirmar sua participação.</t>
         </is>
       </c>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-MCI-–-MOBILITY-CONFAP-ITALY-2026.pdf</t>
         </is>
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_MOBILITY_CONFAP_ITALY_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1621,7 +1635,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA HORIZON EUROPE</t>
+          <t>CHAMADA ERC-CONFAP 2026</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -1633,92 +1647,157 @@
       <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="2" t="inlineStr">
         <is>
+          <t>Apoiar a mobilidade de pesquisadores do estado do Espírito Santo para integrar equipes de pesquisa na Europa, em projetos financiados pelo Conselho Europeu de Pesquisa (ERC). O objetivo é possibilitar colaborações de pesquisa, promover oportunidades em equipes internacionais de excelência e fortalecer a internacionalização da ciência, tecnologia e inovação desenvolvida no Espírito Santo.</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores ativos do Brasil, com título de doutor, que implementam atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros. Para FAPES, o proponente deve ser pesquisador principal ou coordenador do projeto, vinculado a IES/P no Espírito Santo, residente no estado, brasileiro ou estrangeiro com visto permanente, com currículo Lattes atualizado, adimplente com a FAPES e em regularidade perante as normas legais vigentes.</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>US$ 18.000,00</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>US$ 6.000,00</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>internacional.confap@gmail.com, global@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-10: Submissão de propostas (CONFAP) (Propostas completas, incluindo todos os documentos solicitados no Item 6 do edital geral, devem ser submetidas via portal https://sistema.confap.org.br/.)
+2026-08-10: Submissão de documentação para verificação de elegibilidade (FAPES) (Submeter via SigFapes a documentação exigida conforme Instrução de Serviços nº 082/2025 e Item 4, alínea B do edital específico da FAPES.)</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>A FAPES apoiará até 3 projetos selecionados. Os recursos podem ser usados como auxílios individuais para estágios ou visitas técnicas de curta duração. O acesso à lista de projetos ERC é liberado após análise de elegibilidade básica pelo CONFAP. Os pesquisadores devem contatar os PIs dos projetos ERC para definir o Plano de Trabalho e condições.</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
+        </is>
+      </c>
+      <c r="N18" s="2" t="inlineStr">
+        <is>
+          <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Chamadas Internacionais</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>CHAMADA HORIZON EUROPE</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr"/>
+      <c r="E19" s="2" t="inlineStr"/>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
           <t>Este edital da FAPES visa apoiar a participação de pesquisadores do estado do Espírito Santo, na condição de co-PI (co-Principal Investigator), em projetos de pesquisa e inovação executados por consórcios de parceiros europeus e associados no âmbito do Programa Horizonte Europa. As diretrizes orientam exclusivamente a submissão de propostas na categoria “C - Projetos Colaborativos (Pilar II)”, que se refere a projetos de pesquisa e inovação em grande escala para desenvolver soluções para desafios globais.</t>
         </is>
       </c>
-      <c r="G18" s="2" t="inlineStr">
+      <c r="G19" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores proponentes do estado do Espírito Santo, na condição de co-PI, vinculados a instituições de pesquisa ou acadêmicas, para participação em consórcios de projetos colaborativos da categoria 'C - Projetos Colaborativos (Pilar II)' do Horizonte Europa.</t>
         </is>
       </c>
-      <c r="H18" s="2" t="n"/>
-      <c r="I18" s="2" t="inlineStr">
+      <c r="H19" s="2" t="n"/>
+      <c r="I19" s="2" t="inlineStr">
         <is>
           <t>€ 25.000,00 por ano de projeto</t>
         </is>
       </c>
-      <c r="J18" s="2" t="inlineStr">
+      <c r="J19" s="2" t="inlineStr">
         <is>
           <t>parcerias@fapes.es.gov.br, internacional.confap@confap.org.br</t>
         </is>
       </c>
-      <c r="K18" s="2" t="inlineStr">
+      <c r="K19" s="2" t="inlineStr">
         <is>
           <t>?: Consulta de Elegibilidade à FAPES (Pesquisadores devem consultar a FAPES sobre sua elegibilidade antes de iniciar a preparação da proposta, enviando informações como CV em inglês, nome e instituição do coordenador da proposta do Horizonte Europa, título da proposta, orçamento estimado, duração do projeto e descrição resumida.)
 ?: Submissão da Proposta à FAPES (A FAPES receberá propostas associadas às chamadas do Horizonte Europa a qualquer momento. A proposta deve incluir cópia da proposta em inglês submetida ao Horizonte Europa, seguir diretrizes da FAPES e indicar detalhes da proposta vinculada.)
 ?: Assinatura do Termo de Outorga FAPES (Disponível somente após a submissão do Acordo de Subvenção com o qual a UE concede o apoio financeiro ao consórcio. O cofinanciamento por parte da Fapes somente poderá ser contratado até o término da vigência do Arranjo Administrativo Horizonte Europa 2021–2027.)</t>
         </is>
       </c>
-      <c r="L18" s="2" t="inlineStr">
+      <c r="L19" s="2" t="inlineStr">
         <is>
           <t>Os parceiros do Brasil não podem ser coordenadores das propostas submetidas ao Horizonte Europa, pois não são automaticamente elegíveis para receber financiamento da UE. Portanto, eles não podem ser responsáveis pela gestão administrativa e financeira geral do projeto; eles só podem participar como parceiros (ou co-PIs). A referência da chamada é o título (Programa/Tópico) e o número da chamada. Os recursos financeiros aplicados pela Fapes para financiamento de projetos no contexto do Horizonte Europa serão oriundos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo - Funcitec, fonte 0159, recursos vinculados ao Tesouro do Estado. Outros recursos financeiros, decorrentes de parcerias futuras ou de disponibilidade da Fapes e/ou do Funcitec, poderão ser aplicados na suplementação de propostas aprovadas no âmbito do Horizonte Europa 2021-2027. O número máximo de propostas a serem apoiadas no âmbito destas Diretrizes é de até 2 (DOIS) projetos por ano do Horizonte Europa 2021-2027. Os recursos financeiros aprovados pela Fundação poderão abranger despesas com passagens e diárias, observando suas respectivas regulamentações disponíveis na Resolução CCAF nº 309/2022.</t>
         </is>
       </c>
-      <c r="M18" s="2" t="inlineStr">
+      <c r="M19" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20Horizon%20Europe%202021-2027-1.pdf</t>
         </is>
       </c>
-      <c r="N18" s="2" t="inlineStr">
+      <c r="N19" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_HORIZON_EUROPE.pdf</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>Chamadas Internacionais</t>
         </is>
       </c>
-      <c r="B19" s="2" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t>CHAMADA DA PARCERIA DE MATÉRIAS-PRIMAS PARA A TRANSIÇÃO VERDE E DIGITAL (RAMP)</t>
         </is>
       </c>
-      <c r="C19" s="2" t="inlineStr">
+      <c r="C20" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D19" s="2" t="inlineStr">
+      <c r="D20" s="2" t="inlineStr">
         <is>
           <t>2026-09-22: Prazo final para submissão de pré-propostas (Até as 15:00 CEST)</t>
         </is>
       </c>
-      <c r="E19" s="2" t="inlineStr"/>
-      <c r="F19" s="2" t="inlineStr">
+      <c r="E20" s="2" t="inlineStr"/>
+      <c r="F20" s="2" t="inlineStr">
         <is>
           <t>Este edital visa financiar projetos transnacionais de pesquisa e inovação em matérias-primas para a transição verde e digital. Os projetos devem focar em melhorar o acesso a matérias-primas, promover práticas de economia circular, alcançar a sustentabilidade e minimizar custos sociais e ambientais, agregando valor e contribuindo para o desenvolvimento industrial.</t>
         </is>
       </c>
-      <c r="G19" s="2" t="inlineStr">
+      <c r="G20" s="2" t="inlineStr">
         <is>
           <t>Organizações de ensino superior e centros de pesquisa públicos. Os consórcios devem ser compostos por, no mínimo, três parceiros de três países diferentes (sendo pelo menos dois da UE ou países associados).</t>
         </is>
       </c>
-      <c r="H19" s="2" t="n"/>
-      <c r="I19" s="2" t="inlineStr">
+      <c r="H20" s="2" t="n"/>
+      <c r="I20" s="2" t="inlineStr">
         <is>
           <t>EUR 100.000,00</t>
         </is>
       </c>
-      <c r="J19" s="2" t="inlineStr">
+      <c r="J20" s="2" t="inlineStr">
         <is>
           <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K19" s="2" t="inlineStr">
+      <c r="K20" s="2" t="inlineStr">
         <is>
           <t>2026-09-22: Prazo final para submissão de pré-propostas (Até as 15:00 CEST)
 2026-09-22: Submissão de propostas nacionais FAPES (Etapa 1) (Recomendado verificar requisitos da FAPES para submissão na plataforma nacional, prazo idêntico ao da submissão da pré-proposta internacional.)
@@ -1732,17 +1811,17 @@
 2027-06-01 a 2027-09-30: Negociações de contrato nacional/regional / Início dos projetos (esperado)</t>
         </is>
       </c>
-      <c r="L19" s="2" t="inlineStr">
+      <c r="L20" s="2" t="inlineStr">
         <is>
           <t>O edital é um Joint Transnational Call (JTC) 2026 da Parceria Europeia em Matérias-Primas para a Transição Verde e Digital (RAMP). A FAPES (Fundação de Amparo à Pesquisa e Inovação do Espírito Santo) participa sob o guarda-chuva do CONFAP. Cada parceiro de projeto é financiado diretamente por sua respectiva agência nacional/regional. A Comissão Europeia cofinancia os JTCs da RAMP, com o cofinanciamento sendo redistribuído pelas agências financiadoras aos seus beneficiários. A duração máxima dos projetos é de 36 meses. Propostas devem se enquadrar em um dos seis tópicos temáticos e adotar princípios de 'Safe and Sustainable by Design'. Conforme a tabela de elegibilidade de parceiros do CONFAP, empresas (SMEs e grandes) e entidades sem fins lucrativos (ONGs, associações, sociedades, fundações) não são elegíveis para financiamento pela FAPES.</t>
         </is>
       </c>
-      <c r="M19" s="2" t="inlineStr">
+      <c r="M20" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20-%20Chamada%20RAMP%202026.pdf</t>
         </is>
       </c>
-      <c r="N19" s="2" t="inlineStr">
+      <c r="N20" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_DA_PARCERIA_DE_MATÉRIAS-PRIMAS_PARA_A_TRANSIÇÃO_VERDE_E_DIGITAL_(RAMP).pdf</t>
         </is>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-09-15 12:22
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,17 +29,12 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -54,15 +49,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -743,11 +735,7 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-07 a 2026-09-14: Submissão de propostas (Até as 17h59, via SigFapes)</t>
-        </is>
-      </c>
+      <c r="D5" s="2" t="inlineStr"/>
       <c r="E5" s="2" t="inlineStr"/>
       <c r="F5" s="2" t="inlineStr">
         <is>
@@ -1025,9 +1013,9 @@
           <t>EDITAL FAPES Nº 25/2026 - CIÊNCIA ABERTA CAPIXABA</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>Novo - e-mail enviado em 14/09/2026</t>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-09-16 12:16
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,12 +29,17 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEB9C"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -49,12 +54,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -422,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N20"/>
+  <dimension ref="A1:N16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -727,7 +735,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>EDITAL FAPES Nº 21/2026 - REDES DE PESQUISA, DESENVOLVIMENTO E INOVAÇÃO EM SETORES ESTRATÉGICOS</t>
+          <t>EDITAL FAPES Nº 24/2026 - PRIMEIROS PROJETOS DE PESQUISA - ESPÍRITO SANTO (PPP-ES)</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -735,26 +743,30 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr"/>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28: Prazo para envio de dúvidas a respeito do edital (até as 17h59)</t>
+        </is>
+      </c>
       <c r="E5" s="2" t="inlineStr"/>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>O edital Redes de Pesquisa, Desenvolvimento e Inovação (PD&amp;I) em Setores Estratégicos da Fapes tem como finalidade apoiar financeiramente a criação e o fortalecimento de redes que promovam ações coletivas de PD&amp;I. O objetivo geral é selecionar projetos para criar e fortalecer redes estruturantes de PD&amp;I em setores estratégicos e de interesse do Espírito Santo, consolidando grupos de referência em áreas do conhecimento.</t>
+          <t>Apoiar o primeiro projeto de pesquisa científica de pesquisadores doutores em início de carreira, vinculados a Instituições de Ensino Superior e/ou de Pesquisa (IES/P) públicas ou privadas no Espírito Santo. O edital visa fortalecer a pesquisa científica no estado, promover o acesso a recursos e consolidar novos grupos de pesquisa, com projetos de até 24 meses de duração.</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores doutores vinculados a Instituições de Ensino Superior e/ou de Pesquisa (IES/P) públicas ou privadas, sediadas no Estado do Espírito Santo, que atuem como coordenadores de propostas.</t>
+          <t>Pesquisadores doutores em início de carreira, que tenham obtido o título de doutor a partir de 28/08/2018, vinculados a Instituições de Ensino Superior e/ou de Pesquisa (IES/P) públicas ou privadas, sediadas no Estado do Espírito Santo. Os proponentes não devem ter atuado como coordenadores de projetos de pesquisa, extensão ou inovação no âmbito da Fapes ou do CNPq, com exceção de projetos PICJr, PIBIC, PIBITI, auxílios e/ou bolsas de pós-graduação.</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>R$ 12.000.000,00</t>
+          <t>R$ 4.000.000,00</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>R$ 1.200.000,00</t>
+          <t>R$ 180.000,00</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
@@ -763,77 +775,6 @@
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-10: Envio de dúvidas sobre o edital (Até as 17h59)
-2026-08-07 a 2026-09-14: Submissão de propostas (Até as 17h59, via SigFapes)
-?: Interposição de recursos (habilitação) (Até 5 dias úteis após a divulgação do resultado preliminar da habilitação)
-?: Interposição de recursos (análise de mérito) (Até 5 dias úteis após a divulgação do resultado preliminar da análise de mérito)</t>
-        </is>
-      </c>
-      <c r="L5" s="2" t="inlineStr">
-        <is>
-          <t>As propostas devem ter prazo de execução de até 36 meses e prever no orçamento 1 bolsista pós-doutorado (POSDOC) e 1 estudante de graduação (ICT). As linhas temáticas incluem: Saúde Única, Saúde de Precisão, Imunobiológicos e Biofármacos, Preservação e Restauração ecológica do bioma da Mata Atlântica, Transformação digital e rastreabilidade ambiental, Economia Circular e Soberania digital e cibersegurança. A equipe executora deve ser exclusiva e composta por no mínimo 7 pesquisadores além do coordenador, com distribuição específica de doutores de diferentes IES/P e um pesquisador de órgão público estadual. Os recursos serão distribuídos garantindo ao menos uma proposta contemplada por linha temática, e as demais por ordem decrescente de nota final. Somente propostas com nota final igual ou superior a 70,0 pontos serão classificadas. Despesas de custeio com serviços de terceiros são limitadas a 30% do valor máximo por proposta. Despesas de capital financiáveis devem ter vida útil superior a dois anos e valor superior a 80 VRTEs. Não são financiáveis mobiliário (exceto se indispensável à pesquisa) e veículos motorizados (exceto se objeto da pesquisa).</t>
-        </is>
-      </c>
-      <c r="M5" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_21-2026_-_Redes_de_PDI_em_Setores_Estratégicos.pdf</t>
-        </is>
-      </c>
-      <c r="N5" s="2" t="inlineStr">
-        <is>
-          <t>pesquisa/EDITAL_FAPES_No_21_2026_-_REDES_DE_PESQUISA,_DESENVOLVIMENTO_E_INOVAÇÃO_EM_SETORES_ESTRATÉGICOS.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisa</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>EDITAL FAPES Nº 24/2026 - PRIMEIROS PROJETOS DE PESQUISA - ESPÍRITO SANTO (PPP-ES)</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28: Prazo para envio de dúvidas a respeito do edital (até as 17h59)</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr"/>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>Apoiar o primeiro projeto de pesquisa científica de pesquisadores doutores em início de carreira, vinculados a Instituições de Ensino Superior e/ou de Pesquisa (IES/P) públicas ou privadas no Espírito Santo. O edital visa fortalecer a pesquisa científica no estado, promover o acesso a recursos e consolidar novos grupos de pesquisa, com projetos de até 24 meses de duração.</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores doutores em início de carreira, que tenham obtido o título de doutor a partir de 28/08/2018, vinculados a Instituições de Ensino Superior e/ou de Pesquisa (IES/P) públicas ou privadas, sediadas no Estado do Espírito Santo. Os proponentes não devem ter atuado como coordenadores de projetos de pesquisa, extensão ou inovação no âmbito da Fapes ou do CNPq, com exceção de projetos PICJr, PIBIC, PIBITI, auxílios e/ou bolsas de pós-graduação.</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>R$ 4.000.000,00</t>
-        </is>
-      </c>
-      <c r="I6" s="2" t="inlineStr">
-        <is>
-          <t>R$ 180.000,00</t>
-        </is>
-      </c>
-      <c r="J6" s="2" t="inlineStr">
-        <is>
-          <t>editais.duvidas@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K6" s="2" t="inlineStr">
         <is>
           <t>2026-09-28: Prazo para envio de dúvidas a respeito do edital (até as 17h59)
 2026-08-29 a 2026-09-30: Envio da proposta e documentos via SigFapes (até as 17h59)
@@ -842,19 +783,94 @@
 2026-12-10: Início da contratação dos projetos selecionados (Prazo de até 30 dias para a Fapes contratar as propostas aprovadas após a publicação do resultado final homologado.)</t>
         </is>
       </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>Os projetos aprovados terão duração de até 24 meses. Os coordenadores devem ter obtido o título de doutor a partir de 28/08/2018 e não podem ter atuado como coordenadores de projetos de pesquisa, extensão ou inovação no âmbito da Fapes ou do CNPq, exceto em projetos PICJr, PIBIC, PIBITI, auxílios e/ou bolsas de pós-graduação. As propostas devem estar enquadradas em uma das 8 grandes áreas do conhecimento do CNPq. Documentos de aprovação ética e legal, quando aplicáveis, devem estar emitidos ou aprovados no momento da contratação.</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Fapes%2024-2026%20PPP-ES.pdf</t>
+        </is>
+      </c>
+      <c r="N5" s="2" t="inlineStr">
+        <is>
+          <t>pesquisa/EDITAL_FAPES_No_24_2026_-_PRIMEIROS_PROJETOS_DE_PESQUISA_-_ESPÍRITO_SANTO_(PPP-ES).pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Difusão do Conhecimento</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>EDITAL FAPES Nº 17/2026 - PRÊMIO FAPES DE CIÊNCIA, TECNOLOGIA, INOVAÇÃO E JORNALISMO – EDIÇÃO 2026</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Atualizado - e-mail enviado em 16/09/2026</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22 a 2026-09-28: Envio das inscrições – Categoria Jornalismo (até 17h59)</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Objetivo: "O Prêmio Fapes tem como objetivo reconhecer e premiar projetos de destaque e trajetórias profissionais nas áreas de pesquisa, extensão e inovação, bem como premiar matérias jornalísticas sobre a Fapes ou programas e projetos fomentados pela Fundação, valorizando a relevância e o impacto da ciência, tecnologia e inovação para o desenvolvimento do Espírito Santo." → "Reconhecer e premiar projetos de destaque e trajetórias profissionais nas áreas de pesquisa, extensão e inovação, bem como matérias jornalísticas sobre a Fapes ou programas e projetos fomentados pela Fundação. O objetivo é valorizar a relevância, o impacto, a excelência e a divulgação da Ciência, Tecnologia e Inovação (CT&amp;I) no Espírito Santo."
+Público-alvo: "Pesquisadores, extensionistas e empreendedores vinculados a projetos contratados pela Fapes (executados entre 01/01/2019 e 31/12/2025), e profissionais de jornalismo residentes no Espírito Santo, autores de matérias relacionadas à Fapes ou a projetos fomentados." → "Pesquisadores, extensionistas e empreendedores vinculados a projetos contratados pela Fapes (executados a partir de 01/01/2019 e concluídos até 31/12/2025), e profissionais de jornalismo residentes no Espírito Santo, autores de matérias relacionadas à Fapes ou aos programas e projetos fomentados pela Fundação."</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Reconhecer e premiar projetos de destaque e trajetórias profissionais nas áreas de pesquisa, extensão e inovação, bem como matérias jornalísticas sobre a Fapes ou programas e projetos fomentados pela Fundação. O objetivo é valorizar a relevância, o impacto, a excelência e a divulgação da Ciência, Tecnologia e Inovação (CT&amp;I) no Espírito Santo.</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores, extensionistas e empreendedores vinculados a projetos contratados pela Fapes (executados a partir de 01/01/2019 e concluídos até 31/12/2025), e profissionais de jornalismo residentes no Espírito Santo, autores de matérias relacionadas à Fapes ou aos programas e projetos fomentados pela Fundação.</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>R$ 308.000,00</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>R$ 12.000,00</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>editais.duvidas@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22 a 2026-08-06: Envio das inscrições – Categorias Projetos e Destaque (até 17h59)
+2026-06-22 a 2026-09-28: Envio das inscrições – Categoria Jornalismo (até 17h59)
+?: Prazo para recurso administrativo (5 (cinco) dias úteis após a divulgação do resultado preliminar)</t>
+        </is>
+      </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>Os projetos aprovados terão duração de até 24 meses. Os coordenadores devem ter obtido o título de doutor a partir de 28/08/2018 e não podem ter atuado como coordenadores de projetos de pesquisa, extensão ou inovação no âmbito da Fapes ou do CNPq, exceto em projetos PICJr, PIBIC, PIBITI, auxílios e/ou bolsas de pós-graduação. As propostas devem estar enquadradas em uma das 8 grandes áreas do conhecimento do CNPq. Documentos de aprovação ética e legal, quando aplicáveis, devem estar emitidos ou aprovados no momento da contratação.</t>
+          <t>Os valores das premiações possuem natureza bruta e estão sujeitos à incidência do Imposto de Renda Retido na Fonte – IRRF. A premiação tem caráter exclusivamente honorífico, meritório e eventual. O comparecimento do premiado à cerimônia é obrigatório, ou deve-se indicar um representante. A solicitação de pagamento deve ser protocolada em até 90 dias após a publicação do resultado final. Para a categoria Jornalismo, a matéria deve ter sido veiculada e disponibilizada no canal oficial do veículo de comunicação entre 01/09/2025 e 28/09/2026. As etapas de votação final (Comitê de Especialistas e Votação Popular) considerarão as 3 (três) propostas/matérias com as maiores notas em cada subcategoria.</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Fapes%2024-2026%20PPP-ES.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_17.2026_Prêmio_Fapes_Edição_2026_Professora_Jurema_José_de_Oliveira.pdf</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>pesquisa/EDITAL_FAPES_No_24_2026_-_PRIMEIROS_PROJETOS_DE_PESQUISA_-_ESPÍRITO_SANTO_(PPP-ES).pdf</t>
+          <t>difusao_do_conhecimento/EDITAL_FAPES_No_17_2026_-_PRÊMIO_FAPES_DE_CIÊNCIA,_TECNOLOGIA,_INOVAÇÃO_E_JORNALISMO_–_EDIÇÃO_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -866,7 +882,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>EDITAL FAPES Nº 17/2026 - PRÊMIO FAPES DE CIÊNCIA, TECNOLOGIA, INOVAÇÃO E JORNALISMO – EDIÇÃO 2026</t>
+          <t>EDITAL FAPES Nº 25/2026 - CIÊNCIA ABERTA CAPIXABA</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -876,28 +892,28 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22 a 2026-09-15: Envio das inscrições – Categoria Jornalismo (até 17h59. A matéria deve ter sido veiculada entre 01/09/2025 a 15/09/2026 e disponibilizada no canal oficial do veículo de comunicação.)</t>
+          <t>2026-10-08: Prazo para envio de dúvidas a respeito do edital (até as 17h59)</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr"/>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>O Prêmio Fapes tem como objetivo reconhecer e premiar projetos de destaque e trajetórias profissionais nas áreas de pesquisa, extensão e inovação, bem como premiar matérias jornalísticas sobre a Fapes ou programas e projetos fomentados pela Fundação, valorizando a relevância e o impacto da ciência, tecnologia e inovação para o desenvolvimento do Espírito Santo.</t>
+          <t>Apoiar projetos voltados à organização, disponibilização, disseminação e aplicação de dados, informações e evidências científicas de interesse público. O edital busca ampliar o acesso ao conhecimento científico produzido no Espírito Santo, fortalecer sua integração a redes e sistemas de informação nacionais e internacionais e promover sua comunicação para diferentes segmentos da sociedade. O foco é construir uma infraestrutura pública de dados e conhecimento científico sobre temáticas estabelecidas, não financiar pesquisas.</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores, extensionistas e empreendedores vinculados a projetos contratados pela Fapes (executados entre 01/01/2019 e 31/12/2025), e profissionais de jornalismo residentes no Espírito Santo, autores de matérias relacionadas à Fapes ou a projetos fomentados.</t>
+          <t>Profissionais/pesquisadores doutores, vinculados a Instituições de Ensino Superior/ou de Pesquisa (IES/P) públicas ou privadas, sediadas no Estado do Espírito Santo ou em município limítrofe, com vínculo estatutário ou celetista por tempo indeterminado. A equipe executora deve incluir o coordenador e, no mínimo, dois pesquisadores doutores de IES/P de fora do Estado.</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>R$ 308.000,00</t>
+          <t>R$ 3.000.000,00</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>R$ 12.000,00</t>
+          <t>R$ 200.000,00</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
@@ -906,150 +922,6 @@
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-22 a 2026-08-06: Envio das inscrições – Categorias Projetos e Destaque (até 17h59)
-2026-06-22 a 2026-09-15: Envio das inscrições – Categoria Jornalismo (até 17h59. A matéria deve ter sido veiculada entre 01/09/2025 a 15/09/2026 e disponibilizada no canal oficial do veículo de comunicação.)
-?: Prazo para recurso administrativo (5 dias úteis após a divulgação do resultado preliminar)
-2026-11-03 a 2026-11-09: Votação popular – Categoria Jornalismo</t>
-        </is>
-      </c>
-      <c r="L7" s="2" t="inlineStr">
-        <is>
-          <t>Edição em homenagem à Professora Jurema José de Oliveira. Os valores das premiações possuem natureza bruta e estão sujeitos à incidência do Imposto de Renda Retido na Fonte – IRRF, na forma da legislação tributária vigente. A premiação prevista neste edital possui caráter exclusivamente honorífico, meritório e eventual, destinando-se ao reconhecimento institucional dos trabalhos classificados. A Fapes pode alterar datas e prazos do cronograma por necessidade administrativa ou decisão institucional. O comparecimento do premiado é obrigatório. Caso não possa comparecer, deve indicar formalmente um representante para o recebimento da premiação, com comunicação prévia à Fapes, pelo e-mail gabinete@fapes.es.gov.br. Para as categorias Projetos e Destaque, as 3 (três) propostas com as maiores notas seguem para votação pelo Comitê de Especialistas. Para a categoria Jornalismo, as 3 (três) matérias com maiores notas seguem para votação popular.</t>
-        </is>
-      </c>
-      <c r="M7" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_17.2026_Prêmio_Fapes_Edição_2026_Professora_Jurema_José_de_Oliveira.pdf</t>
-        </is>
-      </c>
-      <c r="N7" s="2" t="inlineStr">
-        <is>
-          <t>difusao_do_conhecimento/EDITAL_FAPES_No_17_2026_-_PRÊMIO_FAPES_DE_CIÊNCIA,_TECNOLOGIA,_INOVAÇÃO_E_JORNALISMO_–_EDIÇÃO_2026.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>Difusão do Conhecimento</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>EDITAL FAPES N° 25/2025 - PARTICIPAÇÃO DE EQUIPES DE ESTUDANTES EM MOSTRAS E COMPETIÇÕES TÉCNICO-CIENTÍFICAS</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>Removido (nao mais aberto)</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr"/>
-      <c r="E8" s="2" t="inlineStr"/>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>Conceder apoio financeiro a equipes formadas por estudantes de nível médio, de graduação e pós-graduação, coordenadas por um professor orientador. O objetivo é permitir a participação dessas equipes em mostras e competições técnico-científicas de âmbito regional, nacional ou internacional, visando a divulgação e difusão de resultados obtidos por instituições de ensino do Espírito Santo.</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr">
-        <is>
-          <t>Professores(as) coordenadores(as) de equipes de 3 a 5 estudantes, vinculados(as) a instituições de ensino médio públicas ou instituições de ensino superior públicas ou privadas localizadas no estado do Espírito Santo. O proponente deve ter formação mínima de nível superior, vínculo ativo com a instituição, atuar em sala de aula na mesma instituição dos estudantes, ter Lattes atualizado há menos de 6 meses, estar regularizado junto à Fapes e morar no Espírito Santo ou municípios limítrofes. Estudantes de instituições privadas devem ser bolsistas integrais financiados por programas governamentais estaduais ou federais.</t>
-        </is>
-      </c>
-      <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t>R$ 500.000,00</t>
-        </is>
-      </c>
-      <c r="I8" s="2" t="inlineStr">
-        <is>
-          <t>US$ 1.500,00</t>
-        </is>
-      </c>
-      <c r="J8" s="2" t="inlineStr">
-        <is>
-          <t>editais.duvidas@fapes.es.gov.br, sucon@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K8" s="2" t="inlineStr">
-        <is>
-          <t>?: Prazo para impugnação do edital (5 dias úteis antes do encerramento do prazo de submissão da 1ª Chamada)
-2025-11-10 a 2025-12-16: Submissão de propostas (Até as 17h:59. Para 1ª Chamada (eventos com início entre 01/03/2026 a 30/06/2026))
-?: Interposição de recursos administrativos (5 dias úteis a partir da publicação do resultado preliminar. Para 1ª Chamada (eventos com início entre 01/03/2026 a 30/06/2026))
-2026-03-04 a 2026-04-09: Submissão de propostas (Até as 17:59h. Para 2ª Chamada (eventos com início entre 01/07/2026 a 31/12/2026))
-?: Interposição de recursos administrativos (5 dias úteis a partir da publicação do resultado preliminar. Para 2ª Chamada (eventos com início entre 01/07/2026 a 31/12/2026))
-2026-08-04 a 2026-09-11: Submissão de propostas (Até as 17h:59. Para 3ª Chamada (eventos com início entre 04/01/2027 a 30/04/2027))
-?: Interposição de recursos administrativos (5 dias úteis a partir da publicação do resultado preliminar. Para 3ª Chamada (eventos com início entre 04/01/2027 a 30/04/2027))
-?: Contratação e assinatura do Termo de Outorga (Até 30 dias após a publicação do resultado final homologado. Período específico de assinatura será definido após a homologação.)
-?: Prazo para informar dados bancários (Até 30 dias após a assinatura e publicação do Termo de Outorga)
-?: Prazo para prestação de contas (Até 30 dias após o término da vigência do Termo de Outorga)</t>
-        </is>
-      </c>
-      <c r="L8" s="2" t="inlineStr">
-        <is>
-          <t>O valor por proposta varia conforme a categoria do evento: R$ 500,00 para eventos regionais, R$ 1.200,00 para eventos nacionais e US$ 1.500,00 para eventos internacionais. O edital prevê três chamadas com períodos de submissão e eventos distintos. O início do evento proposto deve corresponder ao período da chamada selecionada. A Fapes pode alterar as datas e prazos definidos no cronograma. Cada coordenador pode apresentar apenas uma proposta. Não são contempladas propostas para participação em concursos ou premiações sem natureza acadêmica, técnico-científica ou tecnológica, ou competições esportivas.</t>
-        </is>
-      </c>
-      <c r="M8" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_N_25_2025_Participação_Equipe_em_Mostras_e_Competições-2.pdf</t>
-        </is>
-      </c>
-      <c r="N8" s="2" t="inlineStr">
-        <is>
-          <t>difusao_do_conhecimento/EDITAL_FAPES_N°_25_2025_-_PARTICIPAÇÃO_DE_EQUIPES_DE_ESTUDANTES_EM_MOSTRAS_E_COMPETIÇÕES_TÉCNICO-CIENTÍFICAS.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>Difusão do Conhecimento</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>EDITAL FAPES Nº 25/2026 - CIÊNCIA ABERTA CAPIXABA</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-08: Prazo para envio de dúvidas a respeito do edital (até as 17h59)</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr"/>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>Apoiar projetos voltados à organização, disponibilização, disseminação e aplicação de dados, informações e evidências científicas de interesse público. O edital busca ampliar o acesso ao conhecimento científico produzido no Espírito Santo, fortalecer sua integração a redes e sistemas de informação nacionais e internacionais e promover sua comunicação para diferentes segmentos da sociedade. O foco é construir uma infraestrutura pública de dados e conhecimento científico sobre temáticas estabelecidas, não financiar pesquisas.</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>Profissionais/pesquisadores doutores, vinculados a Instituições de Ensino Superior/ou de Pesquisa (IES/P) públicas ou privadas, sediadas no Estado do Espírito Santo ou em município limítrofe, com vínculo estatutário ou celetista por tempo indeterminado. A equipe executora deve incluir o coordenador e, no mínimo, dois pesquisadores doutores de IES/P de fora do Estado.</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>R$ 3.000.000,00</t>
-        </is>
-      </c>
-      <c r="I9" s="2" t="inlineStr">
-        <is>
-          <t>R$ 200.000,00</t>
-        </is>
-      </c>
-      <c r="J9" s="2" t="inlineStr">
-        <is>
-          <t>editais.duvidas@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K9" s="2" t="inlineStr">
         <is>
           <t>2026-10-08: Prazo para envio de dúvidas a respeito do edital (até as 17h59)
 2026-09-14 a 2026-10-15: Submissão de propostas e documentos (até as 17h59 via SigFapes)
@@ -1057,70 +929,70 @@
 ?: Prazo para interposição de recursos (análise de mérito) (5 dias úteis após a divulgação do resultado preliminar da análise de mérito)</t>
         </is>
       </c>
-      <c r="L9" s="2" t="inlineStr">
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>As propostas devem estar enquadradas em uma das seguintes linhas temáticas: Saúde e Saúde Pública; Sustentabilidade Socioambiental, Descarbonização e Clima; Biodiversidade e Recursos Naturais; Cidades e Territórios Sustentáveis e Resilientes; Agricultura, Produção de Alimentos e Segurança Alimentar. A distribuição dos recursos financeiros prevê a seleção das 2 (duas) propostas com as maiores Notas Finais em cada linha temática, e após, as demais propostas serão selecionadas conforme a ordem decrescente de Nota Final, independentemente da linha temática, até o limite dos recursos. A Fapes pode alterar as datas e os prazos do cronograma por necessidade administrativa ou decisão institucional.</t>
         </is>
       </c>
-      <c r="M9" s="2" t="inlineStr">
+      <c r="M7" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_25-2026_Ciência_Aberta_Capixaba.pdf</t>
         </is>
       </c>
-      <c r="N9" s="2" t="inlineStr">
+      <c r="N7" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_25_2026_-_CIÊNCIA_ABERTA_CAPIXABA.pdf</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Difusão do Conhecimento</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 28/2025 - PUBLICAÇÃO DE ARTIGOS TÉCNICO-CIENTÍFICOS</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>Removido (nao mais aberto)</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>2026-09-06 a 2026-10-26: Submissão de propostas (4ª Chamada, até as 17h59)</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr"/>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>O objetivo geral deste edital é incentivar a publicação científica e tecnológica no Espírito Santo por meio da concessão de auxílio financeiro para publicação de artigos técnico-científicos que apresentem resultados de pesquisa desenvolvidas em Instituições de Ensino e/ou Pesquisa no estado. A chamada pública visa selecionar propostas para concessão de auxílio financeiro para tal finalidade, valorizando a produção técnico-científica e ampliando a visibilidade das atividades de pesquisa e inovação.</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>Pesquisador ou aluno em atividade de pesquisa ou desenvolvimento inovador em Instituição de Ensino e/ou Pesquisa (IES/P) localizada no estado do Espírito Santo.</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>R$ 800.000,00</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>US$ 1.500,00</t>
         </is>
       </c>
-      <c r="J10" s="2" t="inlineStr">
+      <c r="J8" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K10" s="2" t="inlineStr">
+      <c r="K8" s="2" t="inlineStr">
         <is>
           <t>2025-12-22 a 2026-02-25: Submissão de propostas (1ª Chamada, até as 17h59)
 2026-02-17: Prazo para impugnação do edital (Até 5 dias úteis antes do encerramento do prazo de submissão da primeira chamada)
@@ -1136,70 +1008,70 @@
 ?: Prestação de contas (Até 30 dias após o término de vigência do Termo de Outorga (prazo máximo de execução do projeto é de 12 meses))</t>
         </is>
       </c>
-      <c r="L10" s="2" t="inlineStr">
+      <c r="L8" s="2" t="inlineStr">
         <is>
           <t>O artigo deve ter sido aceito em periódico classificado entre A1 e A4 no Qualis-Capes (2021-2024) ou com percentil igual ou superior a 50% nas plataformas Scopus ou ISI Web of Science. O proponente poderá ser contratado para no máximo 2 propostas, desde que submetidas em chamadas distintas. Cada coordenador pode apresentar apenas uma proposta por chamada; caso envie mais de uma, apenas a última será considerada. O prazo máximo para execução de cada projeto é de 12 meses.</t>
         </is>
       </c>
-      <c r="M10" s="2" t="inlineStr">
+      <c r="M8" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_28_2025_Publicação_de_Artigos_Técnico-Científicos.pdf</t>
         </is>
       </c>
-      <c r="N10" s="2" t="inlineStr">
+      <c r="N8" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_28_2025_-_PUBLICAÇÃO_DE_ARTIGOS_TÉCNICO-CIENTÍFICOS.pdf</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Extensão</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 01/2026 – TCC EMPREENDEDOR INOVADOR</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>2026-09-02 a 2026-10-27: Período de submissão das propostas (Segunda Chamada) (Até 17h59)</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr"/>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="E9" s="2" t="inlineStr"/>
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>Incentivar o desenvolvimento de Trabalhos de Conclusão de Curso (TCCs) com foco em inovação, empreendedorismo e aplicabilidade prática. O edital visa a concessão de Bolsas de Apoio a Trabalho de Conclusão de Curso (BTCC) para a execução de TCCs que apresentem soluções inovadoras e empreendedoras. As propostas devem ter fundamentação teórico-metodológica consistente, voltadas para aplicação prática e impacto econômico, social e/ou ambiental no Estado do Espírito Santo, alinhados aos ODS da ONU e ao Plano ES 500 Anos.</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>Professores orientadores com vínculo estatutário ou celetista por tempo indeterminado com Instituição de Ensino Superior (IES) reconhecida pelo Ministério da Educação (MEC), localizada no Espírito Santo, que submetam entre 3 (três) e 5 (cinco) propostas.</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>R$ 1.600.000,00</t>
         </is>
       </c>
-      <c r="I11" s="2" t="inlineStr">
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>R$ 11.000,00</t>
         </is>
       </c>
-      <c r="J11" s="2" t="inlineStr">
+      <c r="J9" s="2" t="inlineStr">
         <is>
           <t>editais.extensao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K11" s="2" t="inlineStr">
+      <c r="K9" s="2" t="inlineStr">
         <is>
           <t>?: Impugnação do Edital (Até 5 (cinco) dias úteis antes do encerramento do prazo de submissão das propostas de cada chamada.)
 2026-02-02 a 2026-03-30: Período de submissão das propostas (Primeira Chamada) (Até 17h59)
@@ -1216,66 +1088,66 @@
 ?: Prazo para solicitação de ofício para abertura de conta (Até 3 (três) dias úteis para o Outorgado.)</t>
         </is>
       </c>
-      <c r="L11" s="2" t="inlineStr">
+      <c r="L9" s="2" t="inlineStr">
         <is>
           <t>O prazo de execução dos projetos será de um semestre letivo, acrescido de até 3 (três) meses apenas para apresentação da Declaração ou Ata de Defesa do TCC. Cada projeto de TCC deve demonstrar potencial de geração de valor, criação de negócios ou produtos inovadores; estar alinhado aos ODS da ONU (especialmente ODS 4, 8, 9, 10 e 17) e ao Plano ES 500 Anos, e ser desenvolvido em consonância com os Projetos Pedagógicos dos respectivos cursos de graduação. As propostas concorrerão com as demais de suas respectivas microrregiões, sendo apoiados, na primeira chamada, no máximo 20 (vinte) projetos de TCC por microrregião e, na segunda e terceira chamadas, até 10 (dez) projetos de TCC por microrregião. Recursos remanescentes serão destinados a projetos em ampla concorrência por ordem decrescente de nota. Propostas submetidas a mais de uma microrregião serão desclassificadas. Cada proposta deverá vincular um único aluno sob orientação do proponente. O proponente que indicar alunos orientados vinculados a outra IES deverá apresentar declaração de autorização tanto da sua IES de vínculo quanto da IES à qual os alunos orientados estão vinculados. Propostas com Nota Final (NF) inferior a 70 (setenta) pontos serão desclassificadas. Não será permitido o acúmulo de bolsas Fapes pelo aluno orientado, exceto com bolsas do Programa Nossa Bolsa, do Programa Universidade para Todos (Prouni) e com Bolsas de Extensão (Ext-E e Ext-F) da Fapes.</t>
         </is>
       </c>
-      <c r="M11" s="2" t="inlineStr">
+      <c r="M9" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_Nº_01.2026_TCC_EMPREENDEDOR_INOVADOR-2.pdf</t>
         </is>
       </c>
-      <c r="N11" s="2" t="inlineStr">
+      <c r="N9" s="2" t="inlineStr">
         <is>
           <t>extensao/EDITAL_FAPES_No_01_2026_–_TCC_EMPREENDEDOR_INOVADOR.pdf</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 08/2026 - NOVA ECONOMIA CAPIXABA 2026</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr"/>
-      <c r="E12" s="2" t="inlineStr"/>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr"/>
+      <c r="E10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>Promover o aumento da competitividade dos setores econômicos capixabas por meio de projetos de inovação, desenvolvidos por empresas (incluindo cooperativas de trabalho) em colaboração com Instituições de Ciência e Tecnologia (ICT) ou Instituições de Ensino Superior (IES) capixabas. O apoio se dará por meio de um modelo de coinvestimento tripartite (FAPES, empresa/cooperativa, ICT/IES), com projetos alinhados ao Plano ES 500 Anos e ao Plano Estadual de Ciência, Tecnologia e Inovação do Espírito Santo (PCTI-ES).</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>Empresas com sede administrativa ou filial no Espírito Santo, individualmente ou em associação com outras empresas ou cooperativas de trabalho capixabas.</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>R$ 40.000.000,00</t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr">
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>R$ 500.000,00 a R$ 3.000.000,00</t>
         </is>
       </c>
-      <c r="J12" s="2" t="inlineStr">
+      <c r="J10" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K12" s="2" t="inlineStr">
+      <c r="K10" s="2" t="inlineStr">
         <is>
           <t>2026-03-30: Submissão das propostas no SIGFAPES (Fluxo contínuo)
 ?: Prazo de submissão dos recursos administrativos (Habilitação) (5 dias úteis a partir da publicação do resultado preliminar da habilitação.)
@@ -1284,70 +1156,70 @@
 ?: Submissão das documentações para contratação (Até 30 dias a partir da publicação do resultado homologado do julgamento de mérito.)</t>
         </is>
       </c>
-      <c r="L12" s="2" t="inlineStr">
+      <c r="L10" s="2" t="inlineStr">
         <is>
           <t>O prazo de execução do projeto é de 24 meses, com possibilidade de prorrogação por até 12 meses. As empresas proponentes e coexecutoras devem ter receita bruta operacional superior a R$ 360.000,00 nos dois últimos exercícios fiscais; cooperativas de trabalho devem apresentar Demonstração de Sobras ou Perdas (DSP). As empresas devem estar ativas há pelo menos 6 meses e não podem ter sido contratadas em editais FAPES nº 07/2024, nº 10/2025 e nº 06/2026, a menos que o projeto, coordenador e equipe executora sejam distintos. É permitida apenas uma proposta por empresa. Em caso de inabilitação ou desclassificação, a empresa poderá realizar uma nova submissão, exceto se reprovada pelo Comitê de Conformidade, o que impede nova submissão nesta chamada. A aprovação da proposta não garante a contratação, que está sujeita à disponibilidade financeira da FAPES, ordem de submissão e visita técnica. O critério de desempate é a data de submissão da proposta no SIGFAPES. Propostas com Nota Final inferior a 80 pontos ou notas individuais inferiores a 4 em critérios específicos serão desclassificadas. A impugnação dos termos do edital deve ser feita em até 5 dias úteis antes do encerramento do prazo de submissão das propostas do primeiro ciclo (considerando o fluxo contínuo, esta observação se refere a um prazo inicial para impugnação do edital em si).</t>
         </is>
       </c>
-      <c r="M12" s="2" t="inlineStr">
+      <c r="M10" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_08-2026_-_Nova_Economia_Capixaba_-_2_Edição_-_Lançamento.pdf</t>
         </is>
       </c>
-      <c r="N12" s="2" t="inlineStr">
+      <c r="N10" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_No_08_2026_-_NOVA_ECONOMIA_CAPIXABA_2026.pdf</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES N° 23/2026 - APOIO ÀS INCUBADORAS DO ESPÍRITO SANTO</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>2026-09-17: Prazo para impugnação do edital (Até 5 dias úteis anteriores ao encerramento do prazo de envio das propostas. O pedido deve ser enviado no E-Flow por meio do Formulário de Impugnação de Edital.)</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr"/>
-      <c r="F13" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr"/>
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>O edital visa apoiar incubadoras públicas ou privadas sem fins lucrativos, localizadas no Espírito Santo, que buscam estimular e prestar apoio logístico, gerencial e/ou tecnológico a empreendedores e empresas com produtos, serviços ou modelos de negócio inovadores. Este apoio busca ampliar, aperfeiçoar e consolidar as atividades de pré-incubação, incubação e pós-incubação, promovendo a capacitação de novos empreendedores e o desenvolvimento socioeconômico do estado.</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>Incubadoras, sem fins lucrativos, sediadas no Espírito Santo, que atendam aos requisitos do edital.</t>
         </is>
       </c>
-      <c r="H13" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>R$ 4.500.000,00</t>
         </is>
       </c>
-      <c r="I13" s="2" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>R$ 252.000,00</t>
         </is>
       </c>
-      <c r="J13" s="2" t="inlineStr">
+      <c r="J11" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K13" s="2" t="inlineStr">
+      <c r="K11" s="2" t="inlineStr">
         <is>
           <t>2026-09-17: Prazo para impugnação do edital (Até 5 dias úteis anteriores ao encerramento do prazo de envio das propostas. O pedido deve ser enviado no E-Flow por meio do Formulário de Impugnação de Edital.)
 2026-08-25 a 2026-09-24: Envio da proposta e documentos (Até as 17h59, via SigFapes)
@@ -1355,19 +1227,151 @@
 2026-11-04: Contratação dos projetos selecionados (A partir desta data)</t>
         </is>
       </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>O projeto terá prazo de vigência de 24 meses, sem prorrogação. Os recursos financeiros remanescentes, caso o número de propostas previstas para contratação nos níveis de maturidade I, II ou III não seja alcançado, serão redirecionados para propostas suplentes. Os recursos destinados ao custeio (exceto bolsas) serão liberados em 2 parcelas. Caso a proposta seja enquadrada em nível de maturidade distinto do indicado pelo proponente, os valores financiáveis serão ajustados proporcionalmente. É obrigatório destinar no mínimo 20% do valor total solicitado para bolsas. As incubadoras beneficiárias devem destinar parte dos recursos de custeio à associação à Anprotec. Propostas com nota final inferior a 60 pontos serão desclassificadas. A classificação por nível de maturidade é a seguinte: Nível Avançado (86 a 100 pontos), Nível Intermediário (76 a 85 pontos), Nível Básico (60 a 75 pontos).</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_23-2026_Apoio%20a%20Incubadoras_(Versão%20Final).pdf</t>
+        </is>
+      </c>
+      <c r="N11" s="2" t="inlineStr">
+        <is>
+          <t>inovacao/EDITAL_FAPES_N°_23_2026_-_APOIO_ÀS_INCUBADORAS_DO_ESPÍRITO_SANTO.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Chamadas Internacionais</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>CHAMADA CONFAP CDTI 2026</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08: Submissão de propostas (Até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Os formulários devem ser preenchidos em língua inglesa.)</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr"/>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Apoiar projetos colaborativos de pesquisa e inovação tecnológica entre o Brasil e a Espanha, abrangendo qualquer setor de atividade. Destina-se a profissionais vinculados a universidades, centros de pesquisa ou empresas do Espírito Santo que desenvolvam atividades de P,D&amp;I e que apresentem propostas conjuntas com empresas espanholas.</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores principais ou coordenadores de projetos, brasileiros ou estrangeiros com visto permanente, residentes no Espírito Santo, com vínculo ativo a universidades, centros de pesquisa ou empresas localizadas no estado do Espírito Santo, que realizem atividades de pesquisa, desenvolvimento e inovação tecnológica e que integrem proposta conjunta com empresa espanhola.</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="n"/>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>€ 75.000,00</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>internacional.confap@gmail.com, brasil@cdti.es, carlos.quintana@cdti.es, global4@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08: Submissão de propostas (Até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Os formulários devem ser preenchidos em língua inglesa.)</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>A FAPES apoiará um único projeto. Os projetos terão duração de 12 a 36 meses. O apoio financeiro da FAPES destina-se a despesas de capital e custeio, excluindo bolsas, conforme Resolução nº 309/2022. Cada proponente pode submeter apenas uma proposta. A submissão à FAPES (via SigFapes) para contratação ocorrerá somente após a aprovação da proposta pelo CDTI. Os projetos devem ter um orçamento total mínimo de € 250.000,00, e o apoio da FAPES deve corresponder a no mínimo 30% da contrapartida do valor total da proposta.</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes_Chamada%20Internacional_CDTI.2026.pdf</t>
+        </is>
+      </c>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_CDTI_2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Chamadas Internacionais</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>CHAMADA CONFAP &amp; WBI - BÉLGICA 2026</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília), exclusivamente por meio da plataforma https://sistema.confap.org.br.)</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr"/>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Apoiar projetos conjuntos de Pesquisa e Inovação, promovendo o intercâmbio científico entre grupos de pesquisa do Espírito Santo e da região da Valônia-Bruxelas, na Bélgica, em áreas como inovação em saúde, energia sustentável, gestão ambiental e aeronáutica. Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas.</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores brasileiros com doutorado, vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) localizadas no estado do Espírito Santo, residentes no estado, que atuem como pesquisador principal ou coordenador do projeto, e que participem de propostas conjuntas com pesquisadores da Valônia-Bruxelas, Bélgica.</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>R$ 300.000,00</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>R$ 150.000,00</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília), exclusivamente por meio da plataforma https://sistema.confap.org.br.)</t>
+        </is>
+      </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>O projeto terá prazo de vigência de 24 meses, sem prorrogação. Os recursos financeiros remanescentes, caso o número de propostas previstas para contratação nos níveis de maturidade I, II ou III não seja alcançado, serão redirecionados para propostas suplentes. Os recursos destinados ao custeio (exceto bolsas) serão liberados em 2 parcelas. Caso a proposta seja enquadrada em nível de maturidade distinto do indicado pelo proponente, os valores financiáveis serão ajustados proporcionalmente. É obrigatório destinar no mínimo 20% do valor total solicitado para bolsas. As incubadoras beneficiárias devem destinar parte dos recursos de custeio à associação à Anprotec. Propostas com nota final inferior a 60 pontos serão desclassificadas. A classificação por nível de maturidade é a seguinte: Nível Avançado (86 a 100 pontos), Nível Intermediário (76 a 85 pontos), Nível Básico (60 a 75 pontos).</t>
+          <t>Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas. O prazo de vigência máximo para cada projeto é de 24 meses. O apoio financeiro da Fapes destina-se exclusivamente a despesas de mobilidade, excluindo bolsas. Cada proponente pode submeter apenas uma proposta; em caso de múltiplas submissões, apenas a última será considerada. As propostas devem ser submetidas utilizando o modelo do Anexo I (Application Form Template) em ambas as plataformas (CONFAP).</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_23-2026_Apoio%20a%20Incubadoras_(Versão%20Final).pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20WBI%20-2026.pdf</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>inovacao/EDITAL_FAPES_N°_23_2026_-_APOIO_ÀS_INCUBADORAS_DO_ESPÍRITO_SANTO.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WBI_-_BÉLGICA_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1379,7 +1383,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA CONFAP CDTI 2026</t>
+          <t>CHAMADA ERC-CONFAP 2026</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1387,51 +1391,52 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-08: Submissão de propostas (Até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Os formulários devem ser preenchidos em língua inglesa.)</t>
-        </is>
-      </c>
+      <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Apoiar projetos colaborativos de pesquisa e inovação tecnológica entre o Brasil e a Espanha, abrangendo qualquer setor de atividade. Destina-se a profissionais vinculados a universidades, centros de pesquisa ou empresas do Espírito Santo que desenvolvam atividades de P,D&amp;I e que apresentem propostas conjuntas com empresas espanholas.</t>
+          <t>Apoiar a mobilidade de pesquisadores do estado do Espírito Santo para integrar equipes de pesquisa na Europa, em projetos financiados pelo Conselho Europeu de Pesquisa (ERC). O objetivo é possibilitar colaborações de pesquisa, promover oportunidades em equipes internacionais de excelência e fortalecer a internacionalização da ciência, tecnologia e inovação desenvolvida no Espírito Santo.</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores principais ou coordenadores de projetos, brasileiros ou estrangeiros com visto permanente, residentes no Espírito Santo, com vínculo ativo a universidades, centros de pesquisa ou empresas localizadas no estado do Espírito Santo, que realizem atividades de pesquisa, desenvolvimento e inovação tecnológica e que integrem proposta conjunta com empresa espanhola.</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="n"/>
+          <t>Pesquisadores ativos do Brasil, com título de doutor, que implementam atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros. Para FAPES, o proponente deve ser pesquisador principal ou coordenador do projeto, vinculado a IES/P no Espírito Santo, residente no estado, brasileiro ou estrangeiro com visto permanente, com currículo Lattes atualizado, adimplente com a FAPES e em regularidade perante as normas legais vigentes.</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>US$ 18.000,00</t>
+        </is>
+      </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>€ 75.000,00</t>
+          <t>US$ 6.000,00</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com, brasil@cdti.es, carlos.quintana@cdti.es, global4@fapes.es.gov.br</t>
+          <t>internacional.confap@gmail.com, global@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08: Submissão de propostas (Até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Os formulários devem ser preenchidos em língua inglesa.)</t>
+          <t>2026-08-10: Submissão de propostas (CONFAP) (Propostas completas, incluindo todos os documentos solicitados no Item 6 do edital geral, devem ser submetidas via portal https://sistema.confap.org.br/.)
+2026-08-10: Submissão de documentação para verificação de elegibilidade (FAPES) (Submeter via SigFapes a documentação exigida conforme Instrução de Serviços nº 082/2025 e Item 4, alínea B do edital específico da FAPES.)</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>A FAPES apoiará um único projeto. Os projetos terão duração de 12 a 36 meses. O apoio financeiro da FAPES destina-se a despesas de capital e custeio, excluindo bolsas, conforme Resolução nº 309/2022. Cada proponente pode submeter apenas uma proposta. A submissão à FAPES (via SigFapes) para contratação ocorrerá somente após a aprovação da proposta pelo CDTI. Os projetos devem ter um orçamento total mínimo de € 250.000,00, e o apoio da FAPES deve corresponder a no mínimo 30% da contrapartida do valor total da proposta.</t>
+          <t>A FAPES apoiará até 3 projetos selecionados. Os recursos podem ser usados como auxílios individuais para estágios ou visitas técnicas de curta duração. O acesso à lista de projetos ERC é liberado após análise de elegibilidade básica pelo CONFAP. Os pesquisadores devem contatar os PIs dos projetos ERC para definir o Plano de Trabalho e condições.</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes_Chamada%20Internacional_CDTI.2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_CDTI_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1443,7 +1448,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA CONFAP &amp; WBI - BÉLGICA 2026</t>
+          <t>CHAMADA HORIZON EUROPE</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1451,55 +1456,49 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília), exclusivamente por meio da plataforma https://sistema.confap.org.br.)</t>
-        </is>
-      </c>
+      <c r="D15" s="2" t="inlineStr"/>
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Apoiar projetos conjuntos de Pesquisa e Inovação, promovendo o intercâmbio científico entre grupos de pesquisa do Espírito Santo e da região da Valônia-Bruxelas, na Bélgica, em áreas como inovação em saúde, energia sustentável, gestão ambiental e aeronáutica. Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas.</t>
+          <t>Este edital da FAPES visa apoiar a participação de pesquisadores do estado do Espírito Santo, na condição de co-PI (co-Principal Investigator), em projetos de pesquisa e inovação executados por consórcios de parceiros europeus e associados no âmbito do Programa Horizonte Europa. As diretrizes orientam exclusivamente a submissão de propostas na categoria “C - Projetos Colaborativos (Pilar II)”, que se refere a projetos de pesquisa e inovação em grande escala para desenvolver soluções para desafios globais.</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores brasileiros com doutorado, vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) localizadas no estado do Espírito Santo, residentes no estado, que atuem como pesquisador principal ou coordenador do projeto, e que participem de propostas conjuntas com pesquisadores da Valônia-Bruxelas, Bélgica.</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="inlineStr">
-        <is>
-          <t>R$ 300.000,00</t>
-        </is>
-      </c>
+          <t>Pesquisadores proponentes do estado do Espírito Santo, na condição de co-PI, vinculados a instituições de pesquisa ou acadêmicas, para participação em consórcios de projetos colaborativos da categoria 'C - Projetos Colaborativos (Pilar II)' do Horizonte Europa.</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="n"/>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>R$ 150.000,00</t>
+          <t>€ 25.000,00 por ano de projeto</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
+          <t>parcerias@fapes.es.gov.br, internacional.confap@confap.org.br</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília), exclusivamente por meio da plataforma https://sistema.confap.org.br.)</t>
+          <t>?: Consulta de Elegibilidade à FAPES (Pesquisadores devem consultar a FAPES sobre sua elegibilidade antes de iniciar a preparação da proposta, enviando informações como CV em inglês, nome e instituição do coordenador da proposta do Horizonte Europa, título da proposta, orçamento estimado, duração do projeto e descrição resumida.)
+?: Submissão da Proposta à FAPES (A FAPES receberá propostas associadas às chamadas do Horizonte Europa a qualquer momento. A proposta deve incluir cópia da proposta em inglês submetida ao Horizonte Europa, seguir diretrizes da FAPES e indicar detalhes da proposta vinculada.)
+?: Assinatura do Termo de Outorga FAPES (Disponível somente após a submissão do Acordo de Subvenção com o qual a UE concede o apoio financeiro ao consórcio. O cofinanciamento por parte da Fapes somente poderá ser contratado até o término da vigência do Arranjo Administrativo Horizonte Europa 2021–2027.)</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas. O prazo de vigência máximo para cada projeto é de 24 meses. O apoio financeiro da Fapes destina-se exclusivamente a despesas de mobilidade, excluindo bolsas. Cada proponente pode submeter apenas uma proposta; em caso de múltiplas submissões, apenas a última será considerada. As propostas devem ser submetidas utilizando o modelo do Anexo I (Application Form Template) em ambas as plataformas (CONFAP).</t>
+          <t>Os parceiros do Brasil não podem ser coordenadores das propostas submetidas ao Horizonte Europa, pois não são automaticamente elegíveis para receber financiamento da UE. Portanto, eles não podem ser responsáveis pela gestão administrativa e financeira geral do projeto; eles só podem participar como parceiros (ou co-PIs). A referência da chamada é o título (Programa/Tópico) e o número da chamada. Os recursos financeiros aplicados pela Fapes para financiamento de projetos no contexto do Horizonte Europa serão oriundos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo - Funcitec, fonte 0159, recursos vinculados ao Tesouro do Estado. Outros recursos financeiros, decorrentes de parcerias futuras ou de disponibilidade da Fapes e/ou do Funcitec, poderão ser aplicados na suplementação de propostas aprovadas no âmbito do Horizonte Europa 2021-2027. O número máximo de propostas a serem apoiadas no âmbito destas Diretrizes é de até 2 (DOIS) projetos por ano do Horizonte Europa 2021-2027. Os recursos financeiros aprovados pela Fundação poderão abranger despesas com passagens e diárias, observando suas respectivas regulamentações disponíveis na Resolução CCAF nº 309/2022.</t>
         </is>
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20WBI%20-2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20Horizon%20Europe%202021-2027-1.pdf</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WBI_-_BÉLGICA_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_HORIZON_EUROPE.pdf</t>
         </is>
       </c>
     </row>
@@ -1511,7 +1510,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA CONFAP &amp; DAAD 2026</t>
+          <t>CHAMADA DA PARCERIA DE MATÉRIAS-PRIMAS PARA A TRANSIÇÃO VERDE E DIGITAL (RAMP)</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -1519,273 +1518,34 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr"/>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22: Prazo final para submissão de pré-propostas (Até as 15:00 CEST)</t>
+        </is>
+      </c>
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Apoiar a manutenção de bolsas de doutorado da FAPES para bolsistas que forem selecionados pelo Serviço Alemão de Intercâmbio Acadêmico (DAAD). O suporte visa permitir que esses bolsistas realizem suas pesquisas em instituições na Alemanha, no âmbito da Chamada DAAD 2026.</t>
+          <t>Este edital visa financiar projetos transnacionais de pesquisa e inovação em matérias-primas para a transição verde e digital. Os projetos devem focar em melhorar o acesso a matérias-primas, promover práticas de economia circular, alcançar a sustentabilidade e minimizar custos sociais e ambientais, agregando valor e contribuindo para o desenvolvimento industrial.</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Bolsistas de doutorado da FAPES que forem selecionados pelo DAAD, que estejam adimplentes junto à FAPES e que não estejam no primeiro nem no último ano do doutorado.</t>
+          <t>Organizações de ensino superior e centros de pesquisa públicos. Os consórcios devem ser compostos por, no mínimo, três parceiros de três países diferentes (sendo pelo menos dois da UE ou países associados).</t>
         </is>
       </c>
       <c r="H16" s="2" t="n"/>
-      <c r="I16" s="2" t="n"/>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>EUR 100.000,00</t>
+        </is>
+      </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
           <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
-        <is>
-          <t>?: Submissão de propostas (As propostas deverão ser submetidas na Plataforma do DAAD, conforme item 3.1.)</t>
-        </is>
-      </c>
-      <c r="L16" s="2" t="inlineStr">
-        <is>
-          <t>Este documento apresenta as diretrizes específicas da FAPES para a Chamada DAAD 2026, complementando o edital completo disponível no site do CONFAP.</t>
-        </is>
-      </c>
-      <c r="M16" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20-%20FAPES%202026-1.pdf</t>
-        </is>
-      </c>
-      <c r="N16" s="2" t="inlineStr">
-        <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_DAAD_2026.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>Chamadas Internacionais</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>CHAMADA MOBILITY CONFAP ITALY 2026</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr"/>
-      <c r="E17" s="2" t="inlineStr"/>
-      <c r="F17" s="2" t="inlineStr">
-        <is>
-          <t>O edital MOBILITY CONFAP ITALY CALL 2026 visa apoiar pesquisadores do Brasil, vinculados a instituições de ensino superior e pesquisa brasileiras, que desejam desenvolver atividades de pesquisa na Itália em colaboração com colegas locais. O objetivo é facilitar e apoiar a colaboração científica, tecnológica e de inovação por meio da mobilidade de estudantes de doutorado, mestrado e pós-doutorado. O suporte é oferecido na forma de bolsas de estudo para fortalecer grupos de pesquisa brasileiros através de colaborações e visitas a grupos de pesquisa na Itália, parte da rede MCI.</t>
-        </is>
-      </c>
-      <c r="G17" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores de doutorado, mestrado e pós-doutorado vinculados a universidades e instituições de pesquisa nos Estados brasileiros participantes, que possuam um supervisor associado a uma universidade italiana parte da rede MCI.</t>
-        </is>
-      </c>
-      <c r="H17" s="2" t="n"/>
-      <c r="I17" s="2" t="n"/>
-      <c r="J17" s="2" t="inlineStr">
-        <is>
-          <t>internacional.confap@gmail.com</t>
-        </is>
-      </c>
-      <c r="K17" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-04: Submissão de propostas (Até as 11:59 (horário de Brasília) via https://sistema.confap.org.br. Proponentes devem verificar com suas FAPs sobre submissão em plataformas próprias.)</t>
-        </is>
-      </c>
-      <c r="L17" s="2" t="inlineStr">
-        <is>
-          <t>As FAPs participantes podem exigir critérios de elegibilidade adicionais e definir as modalidades de apoio, incluindo os valores das bolsas mensais, em suas próprias diretrizes ou orientações, devendo ser consultadas pelos candidatos antes da preparação da proposta. Não serão cobradas taxas de matrícula por nenhuma das partes para qualquer mobilidade de intercâmbio. Em caso de mobilidade no âmbito de projetos com potencial valor comercial e direitos de propriedade intelectual, as instituições anfitriãs e de envio deverão assinar um acordo de colaboração específico. As propostas devem incluir: projeto de pesquisa, Curriculum Vitae do candidato (Brasil), Curriculum Vitae do supervisor (Itália) e carta de apoio do supervisor na universidade italiana. As FAPs podem solicitar documentos adicionais. As vagas e oportunidades de pesquisa nas universidades italianas da rede MCI estão disponíveis em https://site.unibo.it/mobility-confap-italy/en/research-opportunity-offers-in-italy. Detalhes da rede MCI italiana em https://site.unibo.it/mobility-confap-italy/en/mci-program/network-of-italian-university. As FAPs associadas a esta chamada são: Alagoas - FAPEAL, Amazonas - FAPEAM, Bahia - FAPESB, Ceará - FUNCAP, Espírito Santo – FAPES, Goiás - FAPEG, Maranhão - FAPEMA, Pará - FAPESPA, Paraná - Fundação Araucária, Pernambuco – FACEPE, Rio Grande do Sul - FAPERGS, Santa Catarina - FAPESC. Outras FAPs podem confirmar sua participação.</t>
-        </is>
-      </c>
-      <c r="M17" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-MCI-–-MOBILITY-CONFAP-ITALY-2026.pdf</t>
-        </is>
-      </c>
-      <c r="N17" s="2" t="inlineStr">
-        <is>
-          <t>chamadas_internacionais/CHAMADA_MOBILITY_CONFAP_ITALY_2026.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>Chamadas Internacionais</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>CHAMADA ERC-CONFAP 2026</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr"/>
-      <c r="E18" s="2" t="inlineStr"/>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>Apoiar a mobilidade de pesquisadores do estado do Espírito Santo para integrar equipes de pesquisa na Europa, em projetos financiados pelo Conselho Europeu de Pesquisa (ERC). O objetivo é possibilitar colaborações de pesquisa, promover oportunidades em equipes internacionais de excelência e fortalecer a internacionalização da ciência, tecnologia e inovação desenvolvida no Espírito Santo.</t>
-        </is>
-      </c>
-      <c r="G18" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores ativos do Brasil, com título de doutor, que implementam atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros. Para FAPES, o proponente deve ser pesquisador principal ou coordenador do projeto, vinculado a IES/P no Espírito Santo, residente no estado, brasileiro ou estrangeiro com visto permanente, com currículo Lattes atualizado, adimplente com a FAPES e em regularidade perante as normas legais vigentes.</t>
-        </is>
-      </c>
-      <c r="H18" s="2" t="inlineStr">
-        <is>
-          <t>US$ 18.000,00</t>
-        </is>
-      </c>
-      <c r="I18" s="2" t="inlineStr">
-        <is>
-          <t>US$ 6.000,00</t>
-        </is>
-      </c>
-      <c r="J18" s="2" t="inlineStr">
-        <is>
-          <t>internacional.confap@gmail.com, global@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K18" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-10: Submissão de propostas (CONFAP) (Propostas completas, incluindo todos os documentos solicitados no Item 6 do edital geral, devem ser submetidas via portal https://sistema.confap.org.br/.)
-2026-08-10: Submissão de documentação para verificação de elegibilidade (FAPES) (Submeter via SigFapes a documentação exigida conforme Instrução de Serviços nº 082/2025 e Item 4, alínea B do edital específico da FAPES.)</t>
-        </is>
-      </c>
-      <c r="L18" s="2" t="inlineStr">
-        <is>
-          <t>A FAPES apoiará até 3 projetos selecionados. Os recursos podem ser usados como auxílios individuais para estágios ou visitas técnicas de curta duração. O acesso à lista de projetos ERC é liberado após análise de elegibilidade básica pelo CONFAP. Os pesquisadores devem contatar os PIs dos projetos ERC para definir o Plano de Trabalho e condições.</t>
-        </is>
-      </c>
-      <c r="M18" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
-        </is>
-      </c>
-      <c r="N18" s="2" t="inlineStr">
-        <is>
-          <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>Chamadas Internacionais</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>CHAMADA HORIZON EUROPE</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr"/>
-      <c r="E19" s="2" t="inlineStr"/>
-      <c r="F19" s="2" t="inlineStr">
-        <is>
-          <t>Este edital da FAPES visa apoiar a participação de pesquisadores do estado do Espírito Santo, na condição de co-PI (co-Principal Investigator), em projetos de pesquisa e inovação executados por consórcios de parceiros europeus e associados no âmbito do Programa Horizonte Europa. As diretrizes orientam exclusivamente a submissão de propostas na categoria “C - Projetos Colaborativos (Pilar II)”, que se refere a projetos de pesquisa e inovação em grande escala para desenvolver soluções para desafios globais.</t>
-        </is>
-      </c>
-      <c r="G19" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores proponentes do estado do Espírito Santo, na condição de co-PI, vinculados a instituições de pesquisa ou acadêmicas, para participação em consórcios de projetos colaborativos da categoria 'C - Projetos Colaborativos (Pilar II)' do Horizonte Europa.</t>
-        </is>
-      </c>
-      <c r="H19" s="2" t="n"/>
-      <c r="I19" s="2" t="inlineStr">
-        <is>
-          <t>€ 25.000,00 por ano de projeto</t>
-        </is>
-      </c>
-      <c r="J19" s="2" t="inlineStr">
-        <is>
-          <t>parcerias@fapes.es.gov.br, internacional.confap@confap.org.br</t>
-        </is>
-      </c>
-      <c r="K19" s="2" t="inlineStr">
-        <is>
-          <t>?: Consulta de Elegibilidade à FAPES (Pesquisadores devem consultar a FAPES sobre sua elegibilidade antes de iniciar a preparação da proposta, enviando informações como CV em inglês, nome e instituição do coordenador da proposta do Horizonte Europa, título da proposta, orçamento estimado, duração do projeto e descrição resumida.)
-?: Submissão da Proposta à FAPES (A FAPES receberá propostas associadas às chamadas do Horizonte Europa a qualquer momento. A proposta deve incluir cópia da proposta em inglês submetida ao Horizonte Europa, seguir diretrizes da FAPES e indicar detalhes da proposta vinculada.)
-?: Assinatura do Termo de Outorga FAPES (Disponível somente após a submissão do Acordo de Subvenção com o qual a UE concede o apoio financeiro ao consórcio. O cofinanciamento por parte da Fapes somente poderá ser contratado até o término da vigência do Arranjo Administrativo Horizonte Europa 2021–2027.)</t>
-        </is>
-      </c>
-      <c r="L19" s="2" t="inlineStr">
-        <is>
-          <t>Os parceiros do Brasil não podem ser coordenadores das propostas submetidas ao Horizonte Europa, pois não são automaticamente elegíveis para receber financiamento da UE. Portanto, eles não podem ser responsáveis pela gestão administrativa e financeira geral do projeto; eles só podem participar como parceiros (ou co-PIs). A referência da chamada é o título (Programa/Tópico) e o número da chamada. Os recursos financeiros aplicados pela Fapes para financiamento de projetos no contexto do Horizonte Europa serão oriundos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo - Funcitec, fonte 0159, recursos vinculados ao Tesouro do Estado. Outros recursos financeiros, decorrentes de parcerias futuras ou de disponibilidade da Fapes e/ou do Funcitec, poderão ser aplicados na suplementação de propostas aprovadas no âmbito do Horizonte Europa 2021-2027. O número máximo de propostas a serem apoiadas no âmbito destas Diretrizes é de até 2 (DOIS) projetos por ano do Horizonte Europa 2021-2027. Os recursos financeiros aprovados pela Fundação poderão abranger despesas com passagens e diárias, observando suas respectivas regulamentações disponíveis na Resolução CCAF nº 309/2022.</t>
-        </is>
-      </c>
-      <c r="M19" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20Horizon%20Europe%202021-2027-1.pdf</t>
-        </is>
-      </c>
-      <c r="N19" s="2" t="inlineStr">
-        <is>
-          <t>chamadas_internacionais/CHAMADA_HORIZON_EUROPE.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>Chamadas Internacionais</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>CHAMADA DA PARCERIA DE MATÉRIAS-PRIMAS PARA A TRANSIÇÃO VERDE E DIGITAL (RAMP)</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-22: Prazo final para submissão de pré-propostas (Até as 15:00 CEST)</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="inlineStr"/>
-      <c r="F20" s="2" t="inlineStr">
-        <is>
-          <t>Este edital visa financiar projetos transnacionais de pesquisa e inovação em matérias-primas para a transição verde e digital. Os projetos devem focar em melhorar o acesso a matérias-primas, promover práticas de economia circular, alcançar a sustentabilidade e minimizar custos sociais e ambientais, agregando valor e contribuindo para o desenvolvimento industrial.</t>
-        </is>
-      </c>
-      <c r="G20" s="2" t="inlineStr">
-        <is>
-          <t>Organizações de ensino superior e centros de pesquisa públicos. Os consórcios devem ser compostos por, no mínimo, três parceiros de três países diferentes (sendo pelo menos dois da UE ou países associados).</t>
-        </is>
-      </c>
-      <c r="H20" s="2" t="n"/>
-      <c r="I20" s="2" t="inlineStr">
-        <is>
-          <t>EUR 100.000,00</t>
-        </is>
-      </c>
-      <c r="J20" s="2" t="inlineStr">
-        <is>
-          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K20" s="2" t="inlineStr">
         <is>
           <t>2026-09-22: Prazo final para submissão de pré-propostas (Até as 15:00 CEST)
 2026-09-22: Submissão de propostas nacionais FAPES (Etapa 1) (Recomendado verificar requisitos da FAPES para submissão na plataforma nacional, prazo idêntico ao da submissão da pré-proposta internacional.)
@@ -1799,17 +1559,17 @@
 2027-06-01 a 2027-09-30: Negociações de contrato nacional/regional / Início dos projetos (esperado)</t>
         </is>
       </c>
-      <c r="L20" s="2" t="inlineStr">
+      <c r="L16" s="2" t="inlineStr">
         <is>
           <t>O edital é um Joint Transnational Call (JTC) 2026 da Parceria Europeia em Matérias-Primas para a Transição Verde e Digital (RAMP). A FAPES (Fundação de Amparo à Pesquisa e Inovação do Espírito Santo) participa sob o guarda-chuva do CONFAP. Cada parceiro de projeto é financiado diretamente por sua respectiva agência nacional/regional. A Comissão Europeia cofinancia os JTCs da RAMP, com o cofinanciamento sendo redistribuído pelas agências financiadoras aos seus beneficiários. A duração máxima dos projetos é de 36 meses. Propostas devem se enquadrar em um dos seis tópicos temáticos e adotar princípios de 'Safe and Sustainable by Design'. Conforme a tabela de elegibilidade de parceiros do CONFAP, empresas (SMEs e grandes) e entidades sem fins lucrativos (ONGs, associações, sociedades, fundações) não são elegíveis para financiamento pela FAPES.</t>
         </is>
       </c>
-      <c r="M20" s="2" t="inlineStr">
+      <c r="M16" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20-%20Chamada%20RAMP%202026.pdf</t>
         </is>
       </c>
-      <c r="N20" s="2" t="inlineStr">
+      <c r="N16" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_DA_PARCERIA_DE_MATÉRIAS-PRIMAS_PARA_A_TRANSIÇÃO_VERDE_E_DIGITAL_(RAMP).pdf</t>
         </is>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-09-17 12:26
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,17 +29,12 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFEB9C"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -54,15 +49,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -810,9 +802,9 @@
           <t>EDITAL FAPES Nº 17/2026 - PRÊMIO FAPES DE CIÊNCIA, TECNOLOGIA, INOVAÇÃO E JORNALISMO – EDIÇÃO 2026</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>Atualizado - e-mail enviado em 16/09/2026</t>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -820,12 +812,7 @@
           <t>2026-06-22 a 2026-09-28: Envio das inscrições – Categoria Jornalismo (até 17h59)</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>Objetivo: "O Prêmio Fapes tem como objetivo reconhecer e premiar projetos de destaque e trajetórias profissionais nas áreas de pesquisa, extensão e inovação, bem como premiar matérias jornalísticas sobre a Fapes ou programas e projetos fomentados pela Fundação, valorizando a relevância e o impacto da ciência, tecnologia e inovação para o desenvolvimento do Espírito Santo." → "Reconhecer e premiar projetos de destaque e trajetórias profissionais nas áreas de pesquisa, extensão e inovação, bem como matérias jornalísticas sobre a Fapes ou programas e projetos fomentados pela Fundação. O objetivo é valorizar a relevância, o impacto, a excelência e a divulgação da Ciência, Tecnologia e Inovação (CT&amp;I) no Espírito Santo."
-Público-alvo: "Pesquisadores, extensionistas e empreendedores vinculados a projetos contratados pela Fapes (executados entre 01/01/2019 e 31/12/2025), e profissionais de jornalismo residentes no Espírito Santo, autores de matérias relacionadas à Fapes ou a projetos fomentados." → "Pesquisadores, extensionistas e empreendedores vinculados a projetos contratados pela Fapes (executados a partir de 01/01/2019 e concluídos até 31/12/2025), e profissionais de jornalismo residentes no Espírito Santo, autores de matérias relacionadas à Fapes ou aos programas e projetos fomentados pela Fundação."</t>
-        </is>
-      </c>
+      <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr">
         <is>
           <t>Reconhecer e premiar projetos de destaque e trajetórias profissionais nas áreas de pesquisa, extensão e inovação, bem como matérias jornalísticas sobre a Fapes ou programas e projetos fomentados pela Fundação. O objetivo é valorizar a relevância, o impacto, a excelência e a divulgação da Ciência, Tecnologia e Inovação (CT&amp;I) no Espírito Santo.</t>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-09-18 11:45
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -869,117 +869,46 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>EDITAL FAPES Nº 25/2026 - CIÊNCIA ABERTA CAPIXABA</t>
+          <t>EDITAL FAPES Nº 28/2025 - PUBLICAÇÃO DE ARTIGOS TÉCNICO-CIENTÍFICOS</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Sem alteracoes</t>
+          <t>Removido (nao mais aberto)</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08: Prazo para envio de dúvidas a respeito do edital (até as 17h59)</t>
+          <t>2026-09-06 a 2026-10-26: Submissão de propostas (4ª Chamada, até as 17h59)</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr"/>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Apoiar projetos voltados à organização, disponibilização, disseminação e aplicação de dados, informações e evidências científicas de interesse público. O edital busca ampliar o acesso ao conhecimento científico produzido no Espírito Santo, fortalecer sua integração a redes e sistemas de informação nacionais e internacionais e promover sua comunicação para diferentes segmentos da sociedade. O foco é construir uma infraestrutura pública de dados e conhecimento científico sobre temáticas estabelecidas, não financiar pesquisas.</t>
+          <t>O objetivo geral deste edital é incentivar a publicação científica e tecnológica no Espírito Santo por meio da concessão de auxílio financeiro para publicação de artigos técnico-científicos que apresentem resultados de pesquisa desenvolvidas em Instituições de Ensino e/ou Pesquisa no estado. A chamada pública visa selecionar propostas para concessão de auxílio financeiro para tal finalidade, valorizando a produção técnico-científica e ampliando a visibilidade das atividades de pesquisa e inovação.</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Profissionais/pesquisadores doutores, vinculados a Instituições de Ensino Superior/ou de Pesquisa (IES/P) públicas ou privadas, sediadas no Estado do Espírito Santo ou em município limítrofe, com vínculo estatutário ou celetista por tempo indeterminado. A equipe executora deve incluir o coordenador e, no mínimo, dois pesquisadores doutores de IES/P de fora do Estado.</t>
+          <t>Pesquisador ou aluno em atividade de pesquisa ou desenvolvimento inovador em Instituição de Ensino e/ou Pesquisa (IES/P) localizada no estado do Espírito Santo.</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>R$ 3.000.000,00</t>
+          <t>R$ 800.000,00</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>R$ 200.000,00</t>
+          <t>US$ 1.500,00</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>editais.duvidas@fapes.es.gov.br</t>
+          <t>editais.duvidas@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-08: Prazo para envio de dúvidas a respeito do edital (até as 17h59)
-2026-09-14 a 2026-10-15: Submissão de propostas e documentos (até as 17h59 via SigFapes)
-?: Prazo para interposição de recursos (habilitação) (5 dias úteis após a divulgação do resultado preliminar da habilitação)
-?: Prazo para interposição de recursos (análise de mérito) (5 dias úteis após a divulgação do resultado preliminar da análise de mérito)</t>
-        </is>
-      </c>
-      <c r="L7" s="2" t="inlineStr">
-        <is>
-          <t>As propostas devem estar enquadradas em uma das seguintes linhas temáticas: Saúde e Saúde Pública; Sustentabilidade Socioambiental, Descarbonização e Clima; Biodiversidade e Recursos Naturais; Cidades e Territórios Sustentáveis e Resilientes; Agricultura, Produção de Alimentos e Segurança Alimentar. A distribuição dos recursos financeiros prevê a seleção das 2 (duas) propostas com as maiores Notas Finais em cada linha temática, e após, as demais propostas serão selecionadas conforme a ordem decrescente de Nota Final, independentemente da linha temática, até o limite dos recursos. A Fapes pode alterar as datas e os prazos do cronograma por necessidade administrativa ou decisão institucional.</t>
-        </is>
-      </c>
-      <c r="M7" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_25-2026_Ciência_Aberta_Capixaba.pdf</t>
-        </is>
-      </c>
-      <c r="N7" s="2" t="inlineStr">
-        <is>
-          <t>difusao_do_conhecimento/EDITAL_FAPES_No_25_2026_-_CIÊNCIA_ABERTA_CAPIXABA.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>Difusão do Conhecimento</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>EDITAL FAPES Nº 28/2025 - PUBLICAÇÃO DE ARTIGOS TÉCNICO-CIENTÍFICOS</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>Removido (nao mais aberto)</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-06 a 2026-10-26: Submissão de propostas (4ª Chamada, até as 17h59)</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr"/>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>O objetivo geral deste edital é incentivar a publicação científica e tecnológica no Espírito Santo por meio da concessão de auxílio financeiro para publicação de artigos técnico-científicos que apresentem resultados de pesquisa desenvolvidas em Instituições de Ensino e/ou Pesquisa no estado. A chamada pública visa selecionar propostas para concessão de auxílio financeiro para tal finalidade, valorizando a produção técnico-científica e ampliando a visibilidade das atividades de pesquisa e inovação.</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisador ou aluno em atividade de pesquisa ou desenvolvimento inovador em Instituição de Ensino e/ou Pesquisa (IES/P) localizada no estado do Espírito Santo.</t>
-        </is>
-      </c>
-      <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t>R$ 800.000,00</t>
-        </is>
-      </c>
-      <c r="I8" s="2" t="inlineStr">
-        <is>
-          <t>US$ 1.500,00</t>
-        </is>
-      </c>
-      <c r="J8" s="2" t="inlineStr">
-        <is>
-          <t>editais.duvidas@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K8" s="2" t="inlineStr">
         <is>
           <t>2025-12-22 a 2026-02-25: Submissão de propostas (1ª Chamada, até as 17h59)
 2026-02-17: Prazo para impugnação do edital (Até 5 dias úteis antes do encerramento do prazo de submissão da primeira chamada)
@@ -995,19 +924,90 @@
 ?: Prestação de contas (Até 30 dias após o término de vigência do Termo de Outorga (prazo máximo de execução do projeto é de 12 meses))</t>
         </is>
       </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>O artigo deve ter sido aceito em periódico classificado entre A1 e A4 no Qualis-Capes (2021-2024) ou com percentil igual ou superior a 50% nas plataformas Scopus ou ISI Web of Science. O proponente poderá ser contratado para no máximo 2 propostas, desde que submetidas em chamadas distintas. Cada coordenador pode apresentar apenas uma proposta por chamada; caso envie mais de uma, apenas a última será considerada. O prazo máximo para execução de cada projeto é de 12 meses.</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_28_2025_Publicação_de_Artigos_Técnico-Científicos.pdf</t>
+        </is>
+      </c>
+      <c r="N7" s="2" t="inlineStr">
+        <is>
+          <t>difusao_do_conhecimento/EDITAL_FAPES_No_28_2025_-_PUBLICAÇÃO_DE_ARTIGOS_TÉCNICO-CIENTÍFICOS.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Difusão do Conhecimento</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>EDITAL FAPES Nº 25/2026 - CIÊNCIA ABERTA CAPIXABA</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08: Prazo para envio de dúvidas a respeito do edital (até as 17h59)</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Apoiar projetos voltados à organização, disponibilização, disseminação e aplicação de dados, informações e evidências científicas de interesse público. O edital busca ampliar o acesso ao conhecimento científico produzido no Espírito Santo, fortalecer sua integração a redes e sistemas de informação nacionais e internacionais e promover sua comunicação para diferentes segmentos da sociedade. O foco é construir uma infraestrutura pública de dados e conhecimento científico sobre temáticas estabelecidas, não financiar pesquisas.</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Profissionais/pesquisadores doutores, vinculados a Instituições de Ensino Superior/ou de Pesquisa (IES/P) públicas ou privadas, sediadas no Estado do Espírito Santo ou em município limítrofe, com vínculo estatutário ou celetista por tempo indeterminado. A equipe executora deve incluir o coordenador e, no mínimo, dois pesquisadores doutores de IES/P de fora do Estado.</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>R$ 3.000.000,00</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>R$ 200.000,00</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>editais.duvidas@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08: Prazo para envio de dúvidas a respeito do edital (até as 17h59)
+2026-09-14 a 2026-10-15: Submissão de propostas e documentos (até as 17h59 via SigFapes)
+?: Prazo para interposição de recursos (habilitação) (5 dias úteis após a divulgação do resultado preliminar da habilitação)
+?: Prazo para interposição de recursos (análise de mérito) (5 dias úteis após a divulgação do resultado preliminar da análise de mérito)</t>
+        </is>
+      </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>O artigo deve ter sido aceito em periódico classificado entre A1 e A4 no Qualis-Capes (2021-2024) ou com percentil igual ou superior a 50% nas plataformas Scopus ou ISI Web of Science. O proponente poderá ser contratado para no máximo 2 propostas, desde que submetidas em chamadas distintas. Cada coordenador pode apresentar apenas uma proposta por chamada; caso envie mais de uma, apenas a última será considerada. O prazo máximo para execução de cada projeto é de 12 meses.</t>
+          <t>As propostas devem estar enquadradas em uma das seguintes linhas temáticas: Saúde e Saúde Pública; Sustentabilidade Socioambiental, Descarbonização e Clima; Biodiversidade e Recursos Naturais; Cidades e Territórios Sustentáveis e Resilientes; Agricultura, Produção de Alimentos e Segurança Alimentar. A distribuição dos recursos financeiros prevê a seleção das 2 (duas) propostas com as maiores Notas Finais em cada linha temática, e após, as demais propostas serão selecionadas conforme a ordem decrescente de Nota Final, independentemente da linha temática, até o limite dos recursos. A Fapes pode alterar as datas e os prazos do cronograma por necessidade administrativa ou decisão institucional.</t>
         </is>
       </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_28_2025_Publicação_de_Artigos_Técnico-Científicos.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_25-2026_Ciência_Aberta_Capixaba.pdf</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>difusao_do_conhecimento/EDITAL_FAPES_No_28_2025_-_PUBLICAÇÃO_DE_ARTIGOS_TÉCNICO-CIENTÍFICOS.pdf</t>
+          <t>difusao_do_conhecimento/EDITAL_FAPES_No_25_2026_-_CIÊNCIA_ABERTA_CAPIXABA.pdf</t>
         </is>
       </c>
     </row>
@@ -1177,7 +1177,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17: Prazo para impugnação do edital (Até 5 dias úteis anteriores ao encerramento do prazo de envio das propostas. O pedido deve ser enviado no E-Flow por meio do Formulário de Impugnação de Edital.)</t>
+          <t>2026-08-25 a 2026-09-24: Envio da proposta e documentos (Até as 17h59, via SigFapes)</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-09-19 11:05
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,12 +29,17 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEB9C"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -49,12 +54,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -422,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N16"/>
+  <dimension ref="A1:N17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -727,46 +735,123 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
+          <t>EDITAL FAPES Nº 21/2026 - REDES DE PESQUISA, DESENVOLVIMENTO E INOVAÇÃO EM SETORES ESTRATÉGICOS</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Atualizado - e-mail enviado em 19/09/2026</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-07 a 2026-09-21: Envio da proposta e documentos (até as 17h59, via SigFapes)</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Objetivo: "O edital Redes de Pesquisa, Desenvolvimento e Inovação (PD&amp;I) em Setores Estratégicos da Fapes tem como finalidade apoiar financeiramente a criação e o fortalecimento de redes que promovam ações coletivas de PD&amp;I. O objetivo geral é selecionar projetos para criar e fortalecer redes estruturantes de PD&amp;I em setores estratégicos e de interesse do Espírito Santo, consolidando grupos de referência em áreas do conhecimento." → "Apoiar financeiramente a criação e o fortalecimento de redes de Pesquisa, Desenvolvimento e Inovação (PD&amp;I) em Setores Estratégicos, visando a consolidação de grupos de referência e a geração de conhecimentos e soluções para aplicação em políticas públicas do Espírito Santo."
+Público-alvo: "Pesquisadores doutores vinculados a Instituições de Ensino Superior e/ou de Pesquisa (IES/P) públicas ou privadas, sediadas no Estado do Espírito Santo, que atuem como coordenadores de propostas." → "Pesquisadores doutores vinculados a Instituições de Ensino Superior e/ou de Pesquisa (IES/P) públicas ou privadas, sediadas no Estado do Espírito Santo, com vínculo estatutário ou celetista por tempo indeterminado, que residam no Espírito Santo ou em município limítrofe. As propostas devem ser articuladas com outras instituições científicas e tecnológicas e com a participação de órgão ou instituição que atue na gestão de políticas públicas do Estado."
+Submissão (removida): Submissão de propostas — 2026-08-07 a 2026-09-14</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Apoiar financeiramente a criação e o fortalecimento de redes de Pesquisa, Desenvolvimento e Inovação (PD&amp;I) em Setores Estratégicos, visando a consolidação de grupos de referência e a geração de conhecimentos e soluções para aplicação em políticas públicas do Espírito Santo.</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores doutores vinculados a Instituições de Ensino Superior e/ou de Pesquisa (IES/P) públicas ou privadas, sediadas no Estado do Espírito Santo, com vínculo estatutário ou celetista por tempo indeterminado, que residam no Espírito Santo ou em município limítrofe. As propostas devem ser articuladas com outras instituições científicas e tecnológicas e com a participação de órgão ou instituição que atue na gestão de políticas públicas do Estado.</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>R$ 12.000.000,00</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>R$ 1.200.000,00</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>editais.duvidas@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-07 a 2026-09-21: Envio da proposta e documentos (até as 17h59, via SigFapes)
+2026-09-10: Prazo para envio de dúvidas (até as 17h59)
+?: Prazo para recorrer (habilitação) (Até 5 dias úteis após a divulgação do resultado preliminar da habilitação)
+?: Prazo para recorrer (análise de mérito) (Até 5 dias úteis após a divulgação do resultado preliminar de análise de mérito)</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>As propostas devem estar enquadradas em uma das seguintes linhas temáticas: Saúde Única, Saúde de Precisão, Imunobiológicos e Biofármacos, Preservação e Restauração ecológica do bioma da Mata Atlântica, Transformação digital e rastreabilidade ambiental, Economia Circular, Soberania digital e cibersegurança. A distribuição dos recursos priorizará uma proposta por linha temática, e as demais serão selecionadas por ordem decrescente de nota final. Despesas de capital são financiáveis se os bens tiverem vida útil superior a dois anos e valor superior a 80 VRTEs. Mobiliário e veículos motorizados (exceto se objeto da pesquisa) não são financiáveis. É obrigatória a menção do apoio da Fapes em todas as publicações e divulgações relacionadas ao projeto.</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_21-2026_-_Redes_de_PDI_em_Setores_Estratégicos-1.pdf</t>
+        </is>
+      </c>
+      <c r="N5" s="2" t="inlineStr">
+        <is>
+          <t>pesquisa/EDITAL_FAPES_No_21_2026_-_REDES_DE_PESQUISA,_DESENVOLVIMENTO_E_INOVAÇÃO_EM_SETORES_ESTRATÉGICOS.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisa</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
           <t>EDITAL FAPES Nº 24/2026 - PRIMEIROS PROJETOS DE PESQUISA - ESPÍRITO SANTO (PPP-ES)</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>2026-09-28: Prazo para envio de dúvidas a respeito do edital (até as 17h59)</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr"/>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr"/>
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>Apoiar o primeiro projeto de pesquisa científica de pesquisadores doutores em início de carreira, vinculados a Instituições de Ensino Superior e/ou de Pesquisa (IES/P) públicas ou privadas no Espírito Santo. O edital visa fortalecer a pesquisa científica no estado, promover o acesso a recursos e consolidar novos grupos de pesquisa, com projetos de até 24 meses de duração.</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores doutores em início de carreira, que tenham obtido o título de doutor a partir de 28/08/2018, vinculados a Instituições de Ensino Superior e/ou de Pesquisa (IES/P) públicas ou privadas, sediadas no Estado do Espírito Santo. Os proponentes não devem ter atuado como coordenadores de projetos de pesquisa, extensão ou inovação no âmbito da Fapes ou do CNPq, com exceção de projetos PICJr, PIBIC, PIBITI, auxílios e/ou bolsas de pós-graduação.</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>R$ 4.000.000,00</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>R$ 180.000,00</t>
         </is>
       </c>
-      <c r="J5" s="2" t="inlineStr">
+      <c r="J6" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K5" s="2" t="inlineStr">
+      <c r="K6" s="2" t="inlineStr">
         <is>
           <t>2026-09-28: Prazo para envio de dúvidas a respeito do edital (até as 17h59)
 2026-08-29 a 2026-09-30: Envio da proposta e documentos via SigFapes (até as 17h59)
@@ -775,140 +860,140 @@
 2026-12-10: Início da contratação dos projetos selecionados (Prazo de até 30 dias para a Fapes contratar as propostas aprovadas após a publicação do resultado final homologado.)</t>
         </is>
       </c>
-      <c r="L5" s="2" t="inlineStr">
+      <c r="L6" s="2" t="inlineStr">
         <is>
           <t>Os projetos aprovados terão duração de até 24 meses. Os coordenadores devem ter obtido o título de doutor a partir de 28/08/2018 e não podem ter atuado como coordenadores de projetos de pesquisa, extensão ou inovação no âmbito da Fapes ou do CNPq, exceto em projetos PICJr, PIBIC, PIBITI, auxílios e/ou bolsas de pós-graduação. As propostas devem estar enquadradas em uma das 8 grandes áreas do conhecimento do CNPq. Documentos de aprovação ética e legal, quando aplicáveis, devem estar emitidos ou aprovados no momento da contratação.</t>
         </is>
       </c>
-      <c r="M5" s="2" t="inlineStr">
+      <c r="M6" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Fapes%2024-2026%20PPP-ES.pdf</t>
         </is>
       </c>
-      <c r="N5" s="2" t="inlineStr">
+      <c r="N6" s="2" t="inlineStr">
         <is>
           <t>pesquisa/EDITAL_FAPES_No_24_2026_-_PRIMEIROS_PROJETOS_DE_PESQUISA_-_ESPÍRITO_SANTO_(PPP-ES).pdf</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Difusão do Conhecimento</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 17/2026 - PRÊMIO FAPES DE CIÊNCIA, TECNOLOGIA, INOVAÇÃO E JORNALISMO – EDIÇÃO 2026</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>2026-06-22 a 2026-09-28: Envio das inscrições – Categoria Jornalismo (até 17h59)</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr"/>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr"/>
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>Reconhecer e premiar projetos de destaque e trajetórias profissionais nas áreas de pesquisa, extensão e inovação, bem como matérias jornalísticas sobre a Fapes ou programas e projetos fomentados pela Fundação. O objetivo é valorizar a relevância, o impacto, a excelência e a divulgação da Ciência, Tecnologia e Inovação (CT&amp;I) no Espírito Santo.</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores, extensionistas e empreendedores vinculados a projetos contratados pela Fapes (executados a partir de 01/01/2019 e concluídos até 31/12/2025), e profissionais de jornalismo residentes no Espírito Santo, autores de matérias relacionadas à Fapes ou aos programas e projetos fomentados pela Fundação.</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>R$ 308.000,00</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>R$ 12.000,00</t>
         </is>
       </c>
-      <c r="J6" s="2" t="inlineStr">
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K6" s="2" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>2026-06-22 a 2026-08-06: Envio das inscrições – Categorias Projetos e Destaque (até 17h59)
 2026-06-22 a 2026-09-28: Envio das inscrições – Categoria Jornalismo (até 17h59)
 ?: Prazo para recurso administrativo (5 (cinco) dias úteis após a divulgação do resultado preliminar)</t>
         </is>
       </c>
-      <c r="L6" s="2" t="inlineStr">
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>Os valores das premiações possuem natureza bruta e estão sujeitos à incidência do Imposto de Renda Retido na Fonte – IRRF. A premiação tem caráter exclusivamente honorífico, meritório e eventual. O comparecimento do premiado à cerimônia é obrigatório, ou deve-se indicar um representante. A solicitação de pagamento deve ser protocolada em até 90 dias após a publicação do resultado final. Para a categoria Jornalismo, a matéria deve ter sido veiculada e disponibilizada no canal oficial do veículo de comunicação entre 01/09/2025 e 28/09/2026. As etapas de votação final (Comitê de Especialistas e Votação Popular) considerarão as 3 (três) propostas/matérias com as maiores notas em cada subcategoria.</t>
         </is>
       </c>
-      <c r="M6" s="2" t="inlineStr">
+      <c r="M7" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_17.2026_Prêmio_Fapes_Edição_2026_Professora_Jurema_José_de_Oliveira.pdf</t>
         </is>
       </c>
-      <c r="N6" s="2" t="inlineStr">
+      <c r="N7" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_17_2026_-_PRÊMIO_FAPES_DE_CIÊNCIA,_TECNOLOGIA,_INOVAÇÃO_E_JORNALISMO_–_EDIÇÃO_2026.pdf</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Difusão do Conhecimento</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 28/2025 - PUBLICAÇÃO DE ARTIGOS TÉCNICO-CIENTÍFICOS</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>Removido (nao mais aberto)</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>2026-09-06 a 2026-10-26: Submissão de propostas (4ª Chamada, até as 17h59)</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr"/>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>O objetivo geral deste edital é incentivar a publicação científica e tecnológica no Espírito Santo por meio da concessão de auxílio financeiro para publicação de artigos técnico-científicos que apresentem resultados de pesquisa desenvolvidas em Instituições de Ensino e/ou Pesquisa no estado. A chamada pública visa selecionar propostas para concessão de auxílio financeiro para tal finalidade, valorizando a produção técnico-científica e ampliando a visibilidade das atividades de pesquisa e inovação.</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>Pesquisador ou aluno em atividade de pesquisa ou desenvolvimento inovador em Instituição de Ensino e/ou Pesquisa (IES/P) localizada no estado do Espírito Santo.</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>R$ 800.000,00</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>US$ 1.500,00</t>
         </is>
       </c>
-      <c r="J7" s="2" t="inlineStr">
+      <c r="J8" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K7" s="2" t="inlineStr">
+      <c r="K8" s="2" t="inlineStr">
         <is>
           <t>2025-12-22 a 2026-02-25: Submissão de propostas (1ª Chamada, até as 17h59)
 2026-02-17: Prazo para impugnação do edital (Até 5 dias úteis antes do encerramento do prazo de submissão da primeira chamada)
@@ -924,70 +1009,70 @@
 ?: Prestação de contas (Até 30 dias após o término de vigência do Termo de Outorga (prazo máximo de execução do projeto é de 12 meses))</t>
         </is>
       </c>
-      <c r="L7" s="2" t="inlineStr">
+      <c r="L8" s="2" t="inlineStr">
         <is>
           <t>O artigo deve ter sido aceito em periódico classificado entre A1 e A4 no Qualis-Capes (2021-2024) ou com percentil igual ou superior a 50% nas plataformas Scopus ou ISI Web of Science. O proponente poderá ser contratado para no máximo 2 propostas, desde que submetidas em chamadas distintas. Cada coordenador pode apresentar apenas uma proposta por chamada; caso envie mais de uma, apenas a última será considerada. O prazo máximo para execução de cada projeto é de 12 meses.</t>
         </is>
       </c>
-      <c r="M7" s="2" t="inlineStr">
+      <c r="M8" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_28_2025_Publicação_de_Artigos_Técnico-Científicos.pdf</t>
         </is>
       </c>
-      <c r="N7" s="2" t="inlineStr">
+      <c r="N8" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_28_2025_-_PUBLICAÇÃO_DE_ARTIGOS_TÉCNICO-CIENTÍFICOS.pdf</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Difusão do Conhecimento</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 25/2026 - CIÊNCIA ABERTA CAPIXABA</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>2026-10-08: Prazo para envio de dúvidas a respeito do edital (até as 17h59)</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr"/>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="E9" s="2" t="inlineStr"/>
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>Apoiar projetos voltados à organização, disponibilização, disseminação e aplicação de dados, informações e evidências científicas de interesse público. O edital busca ampliar o acesso ao conhecimento científico produzido no Espírito Santo, fortalecer sua integração a redes e sistemas de informação nacionais e internacionais e promover sua comunicação para diferentes segmentos da sociedade. O foco é construir uma infraestrutura pública de dados e conhecimento científico sobre temáticas estabelecidas, não financiar pesquisas.</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>Profissionais/pesquisadores doutores, vinculados a Instituições de Ensino Superior/ou de Pesquisa (IES/P) públicas ou privadas, sediadas no Estado do Espírito Santo ou em município limítrofe, com vínculo estatutário ou celetista por tempo indeterminado. A equipe executora deve incluir o coordenador e, no mínimo, dois pesquisadores doutores de IES/P de fora do Estado.</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>R$ 3.000.000,00</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>R$ 200.000,00</t>
         </is>
       </c>
-      <c r="J8" s="2" t="inlineStr">
+      <c r="J9" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K8" s="2" t="inlineStr">
+      <c r="K9" s="2" t="inlineStr">
         <is>
           <t>2026-10-08: Prazo para envio de dúvidas a respeito do edital (até as 17h59)
 2026-09-14 a 2026-10-15: Submissão de propostas e documentos (até as 17h59 via SigFapes)
@@ -995,70 +1080,70 @@
 ?: Prazo para interposição de recursos (análise de mérito) (5 dias úteis após a divulgação do resultado preliminar da análise de mérito)</t>
         </is>
       </c>
-      <c r="L8" s="2" t="inlineStr">
+      <c r="L9" s="2" t="inlineStr">
         <is>
           <t>As propostas devem estar enquadradas em uma das seguintes linhas temáticas: Saúde e Saúde Pública; Sustentabilidade Socioambiental, Descarbonização e Clima; Biodiversidade e Recursos Naturais; Cidades e Territórios Sustentáveis e Resilientes; Agricultura, Produção de Alimentos e Segurança Alimentar. A distribuição dos recursos financeiros prevê a seleção das 2 (duas) propostas com as maiores Notas Finais em cada linha temática, e após, as demais propostas serão selecionadas conforme a ordem decrescente de Nota Final, independentemente da linha temática, até o limite dos recursos. A Fapes pode alterar as datas e os prazos do cronograma por necessidade administrativa ou decisão institucional.</t>
         </is>
       </c>
-      <c r="M8" s="2" t="inlineStr">
+      <c r="M9" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_25-2026_Ciência_Aberta_Capixaba.pdf</t>
         </is>
       </c>
-      <c r="N8" s="2" t="inlineStr">
+      <c r="N9" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_25_2026_-_CIÊNCIA_ABERTA_CAPIXABA.pdf</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Extensão</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 01/2026 – TCC EMPREENDEDOR INOVADOR</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>2026-09-02 a 2026-10-27: Período de submissão das propostas (Segunda Chamada) (Até 17h59)</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr"/>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>Incentivar o desenvolvimento de Trabalhos de Conclusão de Curso (TCCs) com foco em inovação, empreendedorismo e aplicabilidade prática. O edital visa a concessão de Bolsas de Apoio a Trabalho de Conclusão de Curso (BTCC) para a execução de TCCs que apresentem soluções inovadoras e empreendedoras. As propostas devem ter fundamentação teórico-metodológica consistente, voltadas para aplicação prática e impacto econômico, social e/ou ambiental no Estado do Espírito Santo, alinhados aos ODS da ONU e ao Plano ES 500 Anos.</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>Professores orientadores com vínculo estatutário ou celetista por tempo indeterminado com Instituição de Ensino Superior (IES) reconhecida pelo Ministério da Educação (MEC), localizada no Espírito Santo, que submetam entre 3 (três) e 5 (cinco) propostas.</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>R$ 1.600.000,00</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>R$ 11.000,00</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr">
+      <c r="J10" s="2" t="inlineStr">
         <is>
           <t>editais.extensao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K9" s="2" t="inlineStr">
+      <c r="K10" s="2" t="inlineStr">
         <is>
           <t>?: Impugnação do Edital (Até 5 (cinco) dias úteis antes do encerramento do prazo de submissão das propostas de cada chamada.)
 2026-02-02 a 2026-03-30: Período de submissão das propostas (Primeira Chamada) (Até 17h59)
@@ -1075,66 +1160,66 @@
 ?: Prazo para solicitação de ofício para abertura de conta (Até 3 (três) dias úteis para o Outorgado.)</t>
         </is>
       </c>
-      <c r="L9" s="2" t="inlineStr">
+      <c r="L10" s="2" t="inlineStr">
         <is>
           <t>O prazo de execução dos projetos será de um semestre letivo, acrescido de até 3 (três) meses apenas para apresentação da Declaração ou Ata de Defesa do TCC. Cada projeto de TCC deve demonstrar potencial de geração de valor, criação de negócios ou produtos inovadores; estar alinhado aos ODS da ONU (especialmente ODS 4, 8, 9, 10 e 17) e ao Plano ES 500 Anos, e ser desenvolvido em consonância com os Projetos Pedagógicos dos respectivos cursos de graduação. As propostas concorrerão com as demais de suas respectivas microrregiões, sendo apoiados, na primeira chamada, no máximo 20 (vinte) projetos de TCC por microrregião e, na segunda e terceira chamadas, até 10 (dez) projetos de TCC por microrregião. Recursos remanescentes serão destinados a projetos em ampla concorrência por ordem decrescente de nota. Propostas submetidas a mais de uma microrregião serão desclassificadas. Cada proposta deverá vincular um único aluno sob orientação do proponente. O proponente que indicar alunos orientados vinculados a outra IES deverá apresentar declaração de autorização tanto da sua IES de vínculo quanto da IES à qual os alunos orientados estão vinculados. Propostas com Nota Final (NF) inferior a 70 (setenta) pontos serão desclassificadas. Não será permitido o acúmulo de bolsas Fapes pelo aluno orientado, exceto com bolsas do Programa Nossa Bolsa, do Programa Universidade para Todos (Prouni) e com Bolsas de Extensão (Ext-E e Ext-F) da Fapes.</t>
         </is>
       </c>
-      <c r="M9" s="2" t="inlineStr">
+      <c r="M10" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_Nº_01.2026_TCC_EMPREENDEDOR_INOVADOR-2.pdf</t>
         </is>
       </c>
-      <c r="N9" s="2" t="inlineStr">
+      <c r="N10" s="2" t="inlineStr">
         <is>
           <t>extensao/EDITAL_FAPES_No_01_2026_–_TCC_EMPREENDEDOR_INOVADOR.pdf</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 08/2026 - NOVA ECONOMIA CAPIXABA 2026</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="2" t="inlineStr"/>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr"/>
+      <c r="E11" s="2" t="inlineStr"/>
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>Promover o aumento da competitividade dos setores econômicos capixabas por meio de projetos de inovação, desenvolvidos por empresas (incluindo cooperativas de trabalho) em colaboração com Instituições de Ciência e Tecnologia (ICT) ou Instituições de Ensino Superior (IES) capixabas. O apoio se dará por meio de um modelo de coinvestimento tripartite (FAPES, empresa/cooperativa, ICT/IES), com projetos alinhados ao Plano ES 500 Anos e ao Plano Estadual de Ciência, Tecnologia e Inovação do Espírito Santo (PCTI-ES).</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>Empresas com sede administrativa ou filial no Espírito Santo, individualmente ou em associação com outras empresas ou cooperativas de trabalho capixabas.</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>R$ 40.000.000,00</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>R$ 500.000,00 a R$ 3.000.000,00</t>
         </is>
       </c>
-      <c r="J10" s="2" t="inlineStr">
+      <c r="J11" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K10" s="2" t="inlineStr">
+      <c r="K11" s="2" t="inlineStr">
         <is>
           <t>2026-03-30: Submissão das propostas no SIGFAPES (Fluxo contínuo)
 ?: Prazo de submissão dos recursos administrativos (Habilitação) (5 dias úteis a partir da publicação do resultado preliminar da habilitação.)
@@ -1143,70 +1228,70 @@
 ?: Submissão das documentações para contratação (Até 30 dias a partir da publicação do resultado homologado do julgamento de mérito.)</t>
         </is>
       </c>
-      <c r="L10" s="2" t="inlineStr">
+      <c r="L11" s="2" t="inlineStr">
         <is>
           <t>O prazo de execução do projeto é de 24 meses, com possibilidade de prorrogação por até 12 meses. As empresas proponentes e coexecutoras devem ter receita bruta operacional superior a R$ 360.000,00 nos dois últimos exercícios fiscais; cooperativas de trabalho devem apresentar Demonstração de Sobras ou Perdas (DSP). As empresas devem estar ativas há pelo menos 6 meses e não podem ter sido contratadas em editais FAPES nº 07/2024, nº 10/2025 e nº 06/2026, a menos que o projeto, coordenador e equipe executora sejam distintos. É permitida apenas uma proposta por empresa. Em caso de inabilitação ou desclassificação, a empresa poderá realizar uma nova submissão, exceto se reprovada pelo Comitê de Conformidade, o que impede nova submissão nesta chamada. A aprovação da proposta não garante a contratação, que está sujeita à disponibilidade financeira da FAPES, ordem de submissão e visita técnica. O critério de desempate é a data de submissão da proposta no SIGFAPES. Propostas com Nota Final inferior a 80 pontos ou notas individuais inferiores a 4 em critérios específicos serão desclassificadas. A impugnação dos termos do edital deve ser feita em até 5 dias úteis antes do encerramento do prazo de submissão das propostas do primeiro ciclo (considerando o fluxo contínuo, esta observação se refere a um prazo inicial para impugnação do edital em si).</t>
         </is>
       </c>
-      <c r="M10" s="2" t="inlineStr">
+      <c r="M11" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_08-2026_-_Nova_Economia_Capixaba_-_2_Edição_-_Lançamento.pdf</t>
         </is>
       </c>
-      <c r="N10" s="2" t="inlineStr">
+      <c r="N11" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_No_08_2026_-_NOVA_ECONOMIA_CAPIXABA_2026.pdf</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES N° 23/2026 - APOIO ÀS INCUBADORAS DO ESPÍRITO SANTO</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>2026-08-25 a 2026-09-24: Envio da proposta e documentos (Até as 17h59, via SigFapes)</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr"/>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="E12" s="2" t="inlineStr"/>
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>O edital visa apoiar incubadoras públicas ou privadas sem fins lucrativos, localizadas no Espírito Santo, que buscam estimular e prestar apoio logístico, gerencial e/ou tecnológico a empreendedores e empresas com produtos, serviços ou modelos de negócio inovadores. Este apoio busca ampliar, aperfeiçoar e consolidar as atividades de pré-incubação, incubação e pós-incubação, promovendo a capacitação de novos empreendedores e o desenvolvimento socioeconômico do estado.</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>Incubadoras, sem fins lucrativos, sediadas no Espírito Santo, que atendam aos requisitos do edital.</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="H12" s="2" t="inlineStr">
         <is>
           <t>R$ 4.500.000,00</t>
         </is>
       </c>
-      <c r="I11" s="2" t="inlineStr">
+      <c r="I12" s="2" t="inlineStr">
         <is>
           <t>R$ 252.000,00</t>
         </is>
       </c>
-      <c r="J11" s="2" t="inlineStr">
+      <c r="J12" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K11" s="2" t="inlineStr">
+      <c r="K12" s="2" t="inlineStr">
         <is>
           <t>2026-09-17: Prazo para impugnação do edital (Até 5 dias úteis anteriores ao encerramento do prazo de envio das propostas. O pedido deve ser enviado no E-Flow por meio do Formulário de Impugnação de Edital.)
 2026-08-25 a 2026-09-24: Envio da proposta e documentos (Até as 17h59, via SigFapes)
@@ -1214,83 +1299,19 @@
 2026-11-04: Contratação dos projetos selecionados (A partir desta data)</t>
         </is>
       </c>
-      <c r="L11" s="2" t="inlineStr">
+      <c r="L12" s="2" t="inlineStr">
         <is>
           <t>O projeto terá prazo de vigência de 24 meses, sem prorrogação. Os recursos financeiros remanescentes, caso o número de propostas previstas para contratação nos níveis de maturidade I, II ou III não seja alcançado, serão redirecionados para propostas suplentes. Os recursos destinados ao custeio (exceto bolsas) serão liberados em 2 parcelas. Caso a proposta seja enquadrada em nível de maturidade distinto do indicado pelo proponente, os valores financiáveis serão ajustados proporcionalmente. É obrigatório destinar no mínimo 20% do valor total solicitado para bolsas. As incubadoras beneficiárias devem destinar parte dos recursos de custeio à associação à Anprotec. Propostas com nota final inferior a 60 pontos serão desclassificadas. A classificação por nível de maturidade é a seguinte: Nível Avançado (86 a 100 pontos), Nível Intermediário (76 a 85 pontos), Nível Básico (60 a 75 pontos).</t>
         </is>
       </c>
-      <c r="M11" s="2" t="inlineStr">
+      <c r="M12" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_23-2026_Apoio%20a%20Incubadoras_(Versão%20Final).pdf</t>
         </is>
       </c>
-      <c r="N11" s="2" t="inlineStr">
+      <c r="N12" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_N°_23_2026_-_APOIO_ÀS_INCUBADORAS_DO_ESPÍRITO_SANTO.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>Chamadas Internacionais</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>CHAMADA CONFAP CDTI 2026</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-08: Submissão de propostas (Até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Os formulários devem ser preenchidos em língua inglesa.)</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr"/>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>Apoiar projetos colaborativos de pesquisa e inovação tecnológica entre o Brasil e a Espanha, abrangendo qualquer setor de atividade. Destina-se a profissionais vinculados a universidades, centros de pesquisa ou empresas do Espírito Santo que desenvolvam atividades de P,D&amp;I e que apresentem propostas conjuntas com empresas espanholas.</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores principais ou coordenadores de projetos, brasileiros ou estrangeiros com visto permanente, residentes no Espírito Santo, com vínculo ativo a universidades, centros de pesquisa ou empresas localizadas no estado do Espírito Santo, que realizem atividades de pesquisa, desenvolvimento e inovação tecnológica e que integrem proposta conjunta com empresa espanhola.</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="n"/>
-      <c r="I12" s="2" t="inlineStr">
-        <is>
-          <t>€ 75.000,00</t>
-        </is>
-      </c>
-      <c r="J12" s="2" t="inlineStr">
-        <is>
-          <t>internacional.confap@gmail.com, brasil@cdti.es, carlos.quintana@cdti.es, global4@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K12" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-08: Submissão de propostas (Até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Os formulários devem ser preenchidos em língua inglesa.)</t>
-        </is>
-      </c>
-      <c r="L12" s="2" t="inlineStr">
-        <is>
-          <t>A FAPES apoiará um único projeto. Os projetos terão duração de 12 a 36 meses. O apoio financeiro da FAPES destina-se a despesas de capital e custeio, excluindo bolsas, conforme Resolução nº 309/2022. Cada proponente pode submeter apenas uma proposta. A submissão à FAPES (via SigFapes) para contratação ocorrerá somente após a aprovação da proposta pelo CDTI. Os projetos devem ter um orçamento total mínimo de € 250.000,00, e o apoio da FAPES deve corresponder a no mínimo 30% da contrapartida do valor total da proposta.</t>
-        </is>
-      </c>
-      <c r="M12" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes_Chamada%20Internacional_CDTI.2026.pdf</t>
-        </is>
-      </c>
-      <c r="N12" s="2" t="inlineStr">
-        <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_CDTI_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1302,7 +1323,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA CONFAP &amp; WBI - BÉLGICA 2026</t>
+          <t>CHAMADA CONFAP CDTI 2026</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -1312,53 +1333,49 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília), exclusivamente por meio da plataforma https://sistema.confap.org.br.)</t>
+          <t>2026-10-08: Submissão de propostas (Até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Os formulários devem ser preenchidos em língua inglesa.)</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Apoiar projetos conjuntos de Pesquisa e Inovação, promovendo o intercâmbio científico entre grupos de pesquisa do Espírito Santo e da região da Valônia-Bruxelas, na Bélgica, em áreas como inovação em saúde, energia sustentável, gestão ambiental e aeronáutica. Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas.</t>
+          <t>Apoiar projetos colaborativos de pesquisa e inovação tecnológica entre o Brasil e a Espanha, abrangendo qualquer setor de atividade. Destina-se a profissionais vinculados a universidades, centros de pesquisa ou empresas do Espírito Santo que desenvolvam atividades de P,D&amp;I e que apresentem propostas conjuntas com empresas espanholas.</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores brasileiros com doutorado, vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) localizadas no estado do Espírito Santo, residentes no estado, que atuem como pesquisador principal ou coordenador do projeto, e que participem de propostas conjuntas com pesquisadores da Valônia-Bruxelas, Bélgica.</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>R$ 300.000,00</t>
-        </is>
-      </c>
+          <t>Pesquisadores principais ou coordenadores de projetos, brasileiros ou estrangeiros com visto permanente, residentes no Espírito Santo, com vínculo ativo a universidades, centros de pesquisa ou empresas localizadas no estado do Espírito Santo, que realizem atividades de pesquisa, desenvolvimento e inovação tecnológica e que integrem proposta conjunta com empresa espanhola.</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="n"/>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>R$ 150.000,00</t>
+          <t>€ 75.000,00</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
+          <t>internacional.confap@gmail.com, brasil@cdti.es, carlos.quintana@cdti.es, global4@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília), exclusivamente por meio da plataforma https://sistema.confap.org.br.)</t>
+          <t>2026-10-08: Submissão de propostas (Até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Os formulários devem ser preenchidos em língua inglesa.)</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas. O prazo de vigência máximo para cada projeto é de 24 meses. O apoio financeiro da Fapes destina-se exclusivamente a despesas de mobilidade, excluindo bolsas. Cada proponente pode submeter apenas uma proposta; em caso de múltiplas submissões, apenas a última será considerada. As propostas devem ser submetidas utilizando o modelo do Anexo I (Application Form Template) em ambas as plataformas (CONFAP).</t>
+          <t>A FAPES apoiará um único projeto. Os projetos terão duração de 12 a 36 meses. O apoio financeiro da FAPES destina-se a despesas de capital e custeio, excluindo bolsas, conforme Resolução nº 309/2022. Cada proponente pode submeter apenas uma proposta. A submissão à FAPES (via SigFapes) para contratação ocorrerá somente após a aprovação da proposta pelo CDTI. Os projetos devem ter um orçamento total mínimo de € 250.000,00, e o apoio da FAPES deve corresponder a no mínimo 30% da contrapartida do valor total da proposta.</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20WBI%20-2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes_Chamada%20Internacional_CDTI.2026.pdf</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WBI_-_BÉLGICA_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_CDTI_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1370,7 +1387,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA ERC-CONFAP 2026</t>
+          <t>CHAMADA CONFAP &amp; WBI - BÉLGICA 2026</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1378,52 +1395,55 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr"/>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília), exclusivamente por meio da plataforma https://sistema.confap.org.br.)</t>
+        </is>
+      </c>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Apoiar a mobilidade de pesquisadores do estado do Espírito Santo para integrar equipes de pesquisa na Europa, em projetos financiados pelo Conselho Europeu de Pesquisa (ERC). O objetivo é possibilitar colaborações de pesquisa, promover oportunidades em equipes internacionais de excelência e fortalecer a internacionalização da ciência, tecnologia e inovação desenvolvida no Espírito Santo.</t>
+          <t>Apoiar projetos conjuntos de Pesquisa e Inovação, promovendo o intercâmbio científico entre grupos de pesquisa do Espírito Santo e da região da Valônia-Bruxelas, na Bélgica, em áreas como inovação em saúde, energia sustentável, gestão ambiental e aeronáutica. Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas.</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores ativos do Brasil, com título de doutor, que implementam atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros. Para FAPES, o proponente deve ser pesquisador principal ou coordenador do projeto, vinculado a IES/P no Espírito Santo, residente no estado, brasileiro ou estrangeiro com visto permanente, com currículo Lattes atualizado, adimplente com a FAPES e em regularidade perante as normas legais vigentes.</t>
+          <t>Pesquisadores brasileiros com doutorado, vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) localizadas no estado do Espírito Santo, residentes no estado, que atuem como pesquisador principal ou coordenador do projeto, e que participem de propostas conjuntas com pesquisadores da Valônia-Bruxelas, Bélgica.</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>US$ 18.000,00</t>
+          <t>R$ 300.000,00</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>US$ 6.000,00</t>
+          <t>R$ 150.000,00</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com, global@fapes.es.gov.br</t>
+          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>2026-08-10: Submissão de propostas (CONFAP) (Propostas completas, incluindo todos os documentos solicitados no Item 6 do edital geral, devem ser submetidas via portal https://sistema.confap.org.br/.)
-2026-08-10: Submissão de documentação para verificação de elegibilidade (FAPES) (Submeter via SigFapes a documentação exigida conforme Instrução de Serviços nº 082/2025 e Item 4, alínea B do edital específico da FAPES.)</t>
+          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília), exclusivamente por meio da plataforma https://sistema.confap.org.br.)</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>A FAPES apoiará até 3 projetos selecionados. Os recursos podem ser usados como auxílios individuais para estágios ou visitas técnicas de curta duração. O acesso à lista de projetos ERC é liberado após análise de elegibilidade básica pelo CONFAP. Os pesquisadores devem contatar os PIs dos projetos ERC para definir o Plano de Trabalho e condições.</t>
+          <t>Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas. O prazo de vigência máximo para cada projeto é de 24 meses. O apoio financeiro da Fapes destina-se exclusivamente a despesas de mobilidade, excluindo bolsas. Cada proponente pode submeter apenas uma proposta; em caso de múltiplas submissões, apenas a última será considerada. As propostas devem ser submetidas utilizando o modelo do Anexo I (Application Form Template) em ambas as plataformas (CONFAP).</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20WBI%20-2026.pdf</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WBI_-_BÉLGICA_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1435,7 +1455,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA HORIZON EUROPE</t>
+          <t>CHAMADA ERC-CONFAP 2026</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1447,92 +1467,157 @@
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="2" t="inlineStr">
         <is>
+          <t>Apoiar a mobilidade de pesquisadores do estado do Espírito Santo para integrar equipes de pesquisa na Europa, em projetos financiados pelo Conselho Europeu de Pesquisa (ERC). O objetivo é possibilitar colaborações de pesquisa, promover oportunidades em equipes internacionais de excelência e fortalecer a internacionalização da ciência, tecnologia e inovação desenvolvida no Espírito Santo.</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores ativos do Brasil, com título de doutor, que implementam atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros. Para FAPES, o proponente deve ser pesquisador principal ou coordenador do projeto, vinculado a IES/P no Espírito Santo, residente no estado, brasileiro ou estrangeiro com visto permanente, com currículo Lattes atualizado, adimplente com a FAPES e em regularidade perante as normas legais vigentes.</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>US$ 18.000,00</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>US$ 6.000,00</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>internacional.confap@gmail.com, global@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-10: Submissão de propostas (CONFAP) (Propostas completas, incluindo todos os documentos solicitados no Item 6 do edital geral, devem ser submetidas via portal https://sistema.confap.org.br/.)
+2026-08-10: Submissão de documentação para verificação de elegibilidade (FAPES) (Submeter via SigFapes a documentação exigida conforme Instrução de Serviços nº 082/2025 e Item 4, alínea B do edital específico da FAPES.)</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>A FAPES apoiará até 3 projetos selecionados. Os recursos podem ser usados como auxílios individuais para estágios ou visitas técnicas de curta duração. O acesso à lista de projetos ERC é liberado após análise de elegibilidade básica pelo CONFAP. Os pesquisadores devem contatar os PIs dos projetos ERC para definir o Plano de Trabalho e condições.</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
+        </is>
+      </c>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Chamadas Internacionais</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>CHAMADA HORIZON EUROPE</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr"/>
+      <c r="E16" s="2" t="inlineStr"/>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
           <t>Este edital da FAPES visa apoiar a participação de pesquisadores do estado do Espírito Santo, na condição de co-PI (co-Principal Investigator), em projetos de pesquisa e inovação executados por consórcios de parceiros europeus e associados no âmbito do Programa Horizonte Europa. As diretrizes orientam exclusivamente a submissão de propostas na categoria “C - Projetos Colaborativos (Pilar II)”, que se refere a projetos de pesquisa e inovação em grande escala para desenvolver soluções para desafios globais.</t>
         </is>
       </c>
-      <c r="G15" s="2" t="inlineStr">
+      <c r="G16" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores proponentes do estado do Espírito Santo, na condição de co-PI, vinculados a instituições de pesquisa ou acadêmicas, para participação em consórcios de projetos colaborativos da categoria 'C - Projetos Colaborativos (Pilar II)' do Horizonte Europa.</t>
         </is>
       </c>
-      <c r="H15" s="2" t="n"/>
-      <c r="I15" s="2" t="inlineStr">
+      <c r="H16" s="2" t="n"/>
+      <c r="I16" s="2" t="inlineStr">
         <is>
           <t>€ 25.000,00 por ano de projeto</t>
         </is>
       </c>
-      <c r="J15" s="2" t="inlineStr">
+      <c r="J16" s="2" t="inlineStr">
         <is>
           <t>parcerias@fapes.es.gov.br, internacional.confap@confap.org.br</t>
         </is>
       </c>
-      <c r="K15" s="2" t="inlineStr">
+      <c r="K16" s="2" t="inlineStr">
         <is>
           <t>?: Consulta de Elegibilidade à FAPES (Pesquisadores devem consultar a FAPES sobre sua elegibilidade antes de iniciar a preparação da proposta, enviando informações como CV em inglês, nome e instituição do coordenador da proposta do Horizonte Europa, título da proposta, orçamento estimado, duração do projeto e descrição resumida.)
 ?: Submissão da Proposta à FAPES (A FAPES receberá propostas associadas às chamadas do Horizonte Europa a qualquer momento. A proposta deve incluir cópia da proposta em inglês submetida ao Horizonte Europa, seguir diretrizes da FAPES e indicar detalhes da proposta vinculada.)
 ?: Assinatura do Termo de Outorga FAPES (Disponível somente após a submissão do Acordo de Subvenção com o qual a UE concede o apoio financeiro ao consórcio. O cofinanciamento por parte da Fapes somente poderá ser contratado até o término da vigência do Arranjo Administrativo Horizonte Europa 2021–2027.)</t>
         </is>
       </c>
-      <c r="L15" s="2" t="inlineStr">
+      <c r="L16" s="2" t="inlineStr">
         <is>
           <t>Os parceiros do Brasil não podem ser coordenadores das propostas submetidas ao Horizonte Europa, pois não são automaticamente elegíveis para receber financiamento da UE. Portanto, eles não podem ser responsáveis pela gestão administrativa e financeira geral do projeto; eles só podem participar como parceiros (ou co-PIs). A referência da chamada é o título (Programa/Tópico) e o número da chamada. Os recursos financeiros aplicados pela Fapes para financiamento de projetos no contexto do Horizonte Europa serão oriundos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo - Funcitec, fonte 0159, recursos vinculados ao Tesouro do Estado. Outros recursos financeiros, decorrentes de parcerias futuras ou de disponibilidade da Fapes e/ou do Funcitec, poderão ser aplicados na suplementação de propostas aprovadas no âmbito do Horizonte Europa 2021-2027. O número máximo de propostas a serem apoiadas no âmbito destas Diretrizes é de até 2 (DOIS) projetos por ano do Horizonte Europa 2021-2027. Os recursos financeiros aprovados pela Fundação poderão abranger despesas com passagens e diárias, observando suas respectivas regulamentações disponíveis na Resolução CCAF nº 309/2022.</t>
         </is>
       </c>
-      <c r="M15" s="2" t="inlineStr">
+      <c r="M16" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20Horizon%20Europe%202021-2027-1.pdf</t>
         </is>
       </c>
-      <c r="N15" s="2" t="inlineStr">
+      <c r="N16" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_HORIZON_EUROPE.pdf</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
         <is>
           <t>Chamadas Internacionais</t>
         </is>
       </c>
-      <c r="B16" s="2" t="inlineStr">
+      <c r="B17" s="2" t="inlineStr">
         <is>
           <t>CHAMADA DA PARCERIA DE MATÉRIAS-PRIMAS PARA A TRANSIÇÃO VERDE E DIGITAL (RAMP)</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr">
+      <c r="C17" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
+      <c r="D17" s="2" t="inlineStr">
         <is>
           <t>2026-09-22: Prazo final para submissão de pré-propostas (Até as 15:00 CEST)</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr"/>
-      <c r="F16" s="2" t="inlineStr">
+      <c r="E17" s="2" t="inlineStr"/>
+      <c r="F17" s="2" t="inlineStr">
         <is>
           <t>Este edital visa financiar projetos transnacionais de pesquisa e inovação em matérias-primas para a transição verde e digital. Os projetos devem focar em melhorar o acesso a matérias-primas, promover práticas de economia circular, alcançar a sustentabilidade e minimizar custos sociais e ambientais, agregando valor e contribuindo para o desenvolvimento industrial.</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr">
+      <c r="G17" s="2" t="inlineStr">
         <is>
           <t>Organizações de ensino superior e centros de pesquisa públicos. Os consórcios devem ser compostos por, no mínimo, três parceiros de três países diferentes (sendo pelo menos dois da UE ou países associados).</t>
         </is>
       </c>
-      <c r="H16" s="2" t="n"/>
-      <c r="I16" s="2" t="inlineStr">
+      <c r="H17" s="2" t="n"/>
+      <c r="I17" s="2" t="inlineStr">
         <is>
           <t>EUR 100.000,00</t>
         </is>
       </c>
-      <c r="J16" s="2" t="inlineStr">
+      <c r="J17" s="2" t="inlineStr">
         <is>
           <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K16" s="2" t="inlineStr">
+      <c r="K17" s="2" t="inlineStr">
         <is>
           <t>2026-09-22: Prazo final para submissão de pré-propostas (Até as 15:00 CEST)
 2026-09-22: Submissão de propostas nacionais FAPES (Etapa 1) (Recomendado verificar requisitos da FAPES para submissão na plataforma nacional, prazo idêntico ao da submissão da pré-proposta internacional.)
@@ -1546,17 +1631,17 @@
 2027-06-01 a 2027-09-30: Negociações de contrato nacional/regional / Início dos projetos (esperado)</t>
         </is>
       </c>
-      <c r="L16" s="2" t="inlineStr">
+      <c r="L17" s="2" t="inlineStr">
         <is>
           <t>O edital é um Joint Transnational Call (JTC) 2026 da Parceria Europeia em Matérias-Primas para a Transição Verde e Digital (RAMP). A FAPES (Fundação de Amparo à Pesquisa e Inovação do Espírito Santo) participa sob o guarda-chuva do CONFAP. Cada parceiro de projeto é financiado diretamente por sua respectiva agência nacional/regional. A Comissão Europeia cofinancia os JTCs da RAMP, com o cofinanciamento sendo redistribuído pelas agências financiadoras aos seus beneficiários. A duração máxima dos projetos é de 36 meses. Propostas devem se enquadrar em um dos seis tópicos temáticos e adotar princípios de 'Safe and Sustainable by Design'. Conforme a tabela de elegibilidade de parceiros do CONFAP, empresas (SMEs e grandes) e entidades sem fins lucrativos (ONGs, associações, sociedades, fundações) não são elegíveis para financiamento pela FAPES.</t>
         </is>
       </c>
-      <c r="M16" s="2" t="inlineStr">
+      <c r="M17" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20-%20Chamada%20RAMP%202026.pdf</t>
         </is>
       </c>
-      <c r="N16" s="2" t="inlineStr">
+      <c r="N17" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_DA_PARCERIA_DE_MATÉRIAS-PRIMAS_PARA_A_TRANSIÇÃO_VERDE_E_DIGITAL_(RAMP).pdf</t>
         </is>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-09-20 11:25
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,17 +29,12 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFEB9C"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -54,15 +49,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -606,7 +598,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19: Prazo para impugnação do edital (Até 5 dias úteis anteriores ao término da submissão das propostas.)</t>
+          <t>2026-09-24: Submissão das propostas (Até as 17h59)</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr"/>
@@ -738,9 +730,9 @@
           <t>EDITAL FAPES Nº 21/2026 - REDES DE PESQUISA, DESENVOLVIMENTO E INOVAÇÃO EM SETORES ESTRATÉGICOS</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>Atualizado - e-mail enviado em 19/09/2026</t>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -748,13 +740,7 @@
           <t>2026-08-07 a 2026-09-21: Envio da proposta e documentos (até as 17h59, via SigFapes)</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>Objetivo: "O edital Redes de Pesquisa, Desenvolvimento e Inovação (PD&amp;I) em Setores Estratégicos da Fapes tem como finalidade apoiar financeiramente a criação e o fortalecimento de redes que promovam ações coletivas de PD&amp;I. O objetivo geral é selecionar projetos para criar e fortalecer redes estruturantes de PD&amp;I em setores estratégicos e de interesse do Espírito Santo, consolidando grupos de referência em áreas do conhecimento." → "Apoiar financeiramente a criação e o fortalecimento de redes de Pesquisa, Desenvolvimento e Inovação (PD&amp;I) em Setores Estratégicos, visando a consolidação de grupos de referência e a geração de conhecimentos e soluções para aplicação em políticas públicas do Espírito Santo."
-Público-alvo: "Pesquisadores doutores vinculados a Instituições de Ensino Superior e/ou de Pesquisa (IES/P) públicas ou privadas, sediadas no Estado do Espírito Santo, que atuem como coordenadores de propostas." → "Pesquisadores doutores vinculados a Instituições de Ensino Superior e/ou de Pesquisa (IES/P) públicas ou privadas, sediadas no Estado do Espírito Santo, com vínculo estatutário ou celetista por tempo indeterminado, que residam no Espírito Santo ou em município limítrofe. As propostas devem ser articuladas com outras instituições científicas e tecnológicas e com a participação de órgão ou instituição que atue na gestão de políticas públicas do Estado."
-Submissão (removida): Submissão de propostas — 2026-08-07 a 2026-09-14</t>
-        </is>
-      </c>
+      <c r="E5" s="2" t="inlineStr"/>
       <c r="F5" s="2" t="inlineStr">
         <is>
           <t>Apoiar financeiramente a criação e o fortalecimento de redes de Pesquisa, Desenvolvimento e Inovação (PD&amp;I) em Setores Estratégicos, visando a consolidação de grupos de referência e a geração de conhecimentos e soluções para aplicação em políticas públicas do Espírito Santo.</t>

</xml_diff>